<commit_message>
Fix RSI sheet visual grouping — style group headers, prefix sub-headers with leg type
</commit_message>
<xml_diff>
--- a/public/AMSC_Combine_Data_Template.xlsx
+++ b/public/AMSC_Combine_Data_Template.xlsx
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="23">
+  <fonts count="25">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -176,8 +176,20 @@
       <color rgb="FF000000"/>
       <sz val="11"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="9"/>
+    </font>
   </fonts>
-  <fills count="11">
+  <fills count="15">
     <fill>
       <patternFill/>
     </fill>
@@ -229,8 +241,28 @@
         <fgColor rgb="FFf0f0f0"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00820B0B"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C41E3A"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF820B0B"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC41E3A"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="16">
+  <borders count="29">
     <border>
       <left/>
       <right/>
@@ -411,11 +443,105 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
+    <border>
+      <left style="medium"/>
+      <right/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <right style="medium"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <right/>
+      <top/>
+      <bottom style="thin"/>
+    </border>
+    <border>
+      <left style="medium"/>
+      <right/>
+      <top/>
+      <bottom style="thin"/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <right style="medium"/>
+      <top/>
+      <bottom style="thin"/>
+    </border>
+    <border>
+      <left style="medium"/>
+      <right style="thin">
+        <color rgb="FFcccccc"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFcccccc"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFcccccc"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFcccccc"/>
+      </left>
+      <right style="medium"/>
+      <top style="thin">
+        <color rgb="FFcccccc"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFcccccc"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="medium"/>
+      <right style="medium"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin"/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium"/>
+      <top style="thin"/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2"/>
   </cellStyleXfs>
-  <cellXfs count="62">
+  <cellXfs count="80">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
@@ -587,6 +713,52 @@
     </xf>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="11" borderId="16" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="11" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="11" borderId="16" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="23" fillId="11" borderId="18" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="24" fillId="12" borderId="19" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="12" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="12" borderId="21" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="22" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="23" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="22" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="23" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="13" borderId="16" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="13" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="16" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="13" borderId="18" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="24" fillId="14" borderId="16" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="14" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="14" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1403,6 +1575,14 @@
       <c r="R1" s="53" t="n"/>
       <c r="S1" s="53" t="n"/>
       <c r="T1" s="53" t="n"/>
+      <c r="U1" s="53" t="n"/>
+      <c r="V1" s="53" t="n"/>
+      <c r="W1" s="53" t="n"/>
+      <c r="X1" s="53" t="n"/>
+      <c r="Y1" s="53" t="n"/>
+      <c r="Z1" s="53" t="n"/>
+      <c r="AA1" s="53" t="n"/>
+      <c r="AB1" s="53" t="n"/>
       <c r="AC1" s="53" t="n"/>
       <c r="AD1" s="53" t="n"/>
       <c r="AE1" s="53" t="n"/>
@@ -1411,7 +1591,7 @@
       <c r="AH1" s="53" t="n"/>
       <c r="AI1" s="53" t="n"/>
       <c r="AJ1" s="53" t="n"/>
-      <c r="AK1" s="53" t="n"/>
+      <c r="AK1" s="54" t="n"/>
       <c r="AL1" s="53" t="n"/>
       <c r="AM1" s="53" t="n"/>
       <c r="AN1" s="53" t="n"/>
@@ -1446,6 +1626,14 @@
       <c r="R2" s="53" t="n"/>
       <c r="S2" s="53" t="n"/>
       <c r="T2" s="53" t="n"/>
+      <c r="U2" s="53" t="n"/>
+      <c r="V2" s="53" t="n"/>
+      <c r="W2" s="53" t="n"/>
+      <c r="X2" s="53" t="n"/>
+      <c r="Y2" s="53" t="n"/>
+      <c r="Z2" s="53" t="n"/>
+      <c r="AA2" s="53" t="n"/>
+      <c r="AB2" s="53" t="n"/>
       <c r="AC2" s="53" t="n"/>
       <c r="AD2" s="53" t="n"/>
       <c r="AE2" s="53" t="n"/>
@@ -1454,7 +1642,7 @@
       <c r="AH2" s="53" t="n"/>
       <c r="AI2" s="53" t="n"/>
       <c r="AJ2" s="53" t="n"/>
-      <c r="AK2" s="53" t="n"/>
+      <c r="AK2" s="54" t="n"/>
       <c r="AL2" s="53" t="n"/>
       <c r="AM2" s="53" t="n"/>
       <c r="AN2" s="53" t="n"/>
@@ -5355,91 +5543,100 @@
       <c r="M2" s="54" t="n"/>
     </row>
     <row r="3" ht="22" customFormat="1" customHeight="1" s="1">
-      <c r="A3" s="6" t="inlineStr">
+      <c r="A3" s="73" t="inlineStr">
         <is>
           <t>ATHLETE INFO</t>
         </is>
       </c>
-      <c r="B3" s="6" t="inlineStr">
+      <c r="B3" s="74" t="inlineStr">
         <is>
           <t>DOUBLE-LEG</t>
         </is>
       </c>
-      <c r="F3" s="6" t="inlineStr">
+      <c r="C3" s="75" t="n"/>
+      <c r="D3" s="75" t="n"/>
+      <c r="E3" s="76" t="n"/>
+      <c r="F3" s="74" t="inlineStr">
         <is>
           <t>SINGLE-LEG LEFT</t>
         </is>
       </c>
-      <c r="J3" s="6" t="inlineStr">
+      <c r="G3" s="75" t="n"/>
+      <c r="H3" s="75" t="n"/>
+      <c r="I3" s="76" t="n"/>
+      <c r="J3" s="74" t="inlineStr">
         <is>
           <t>SINGLE-LEG RIGHT</t>
         </is>
       </c>
-    </row>
-    <row r="4" ht="36" customFormat="1" customHeight="1" s="1">
-      <c r="A4" s="7" t="inlineStr">
+      <c r="K3" s="75" t="n"/>
+      <c r="L3" s="75" t="n"/>
+      <c r="M3" s="76" t="n"/>
+    </row>
+    <row r="4" ht="30" customFormat="1" customHeight="1" s="1">
+      <c r="A4" s="77" t="inlineStr">
         <is>
           <t>Athlete Name*</t>
         </is>
       </c>
-      <c r="B4" s="7" t="inlineStr">
-        <is>
-          <t>Avg RSI</t>
-        </is>
-      </c>
-      <c r="C4" s="7" t="inlineStr">
-        <is>
-          <t>Avg GCT (s)</t>
-        </is>
-      </c>
-      <c r="D4" s="7" t="inlineStr">
-        <is>
-          <t>Max RSI</t>
-        </is>
-      </c>
-      <c r="E4" s="7" t="inlineStr">
-        <is>
-          <t>Max GCT (s)</t>
-        </is>
-      </c>
-      <c r="F4" s="7" t="inlineStr">
-        <is>
-          <t>Avg RSI</t>
-        </is>
-      </c>
-      <c r="G4" s="7" t="inlineStr">
-        <is>
-          <t>Avg GCT (s)</t>
-        </is>
-      </c>
-      <c r="H4" s="7" t="inlineStr">
-        <is>
-          <t>Max RSI</t>
-        </is>
-      </c>
-      <c r="I4" s="7" t="inlineStr">
-        <is>
-          <t>Max GCT (s)</t>
-        </is>
-      </c>
-      <c r="J4" s="7" t="inlineStr">
-        <is>
-          <t>Avg RSI</t>
-        </is>
-      </c>
-      <c r="K4" s="7" t="inlineStr">
-        <is>
-          <t>Avg GCT (s)</t>
-        </is>
-      </c>
-      <c r="L4" s="7" t="inlineStr">
-        <is>
-          <t>Max RSI</t>
-        </is>
-      </c>
-      <c r="M4" s="7" t="inlineStr">
-        <is>
-          <t>Max GCT (s)</t>
+      <c r="B4" s="78" t="inlineStr">
+        <is>
+          <t>DL — Avg RSI</t>
+        </is>
+      </c>
+      <c r="C4" s="77" t="inlineStr">
+        <is>
+          <t>DL — Avg GCT (s)</t>
+        </is>
+      </c>
+      <c r="D4" s="77" t="inlineStr">
+        <is>
+          <t>DL — Max RSI</t>
+        </is>
+      </c>
+      <c r="E4" s="79" t="inlineStr">
+        <is>
+          <t>DL — Max GCT (s)</t>
+        </is>
+      </c>
+      <c r="F4" s="78" t="inlineStr">
+        <is>
+          <t>SL-L — Avg RSI</t>
+        </is>
+      </c>
+      <c r="G4" s="77" t="inlineStr">
+        <is>
+          <t>SL-L — Avg GCT (s)</t>
+        </is>
+      </c>
+      <c r="H4" s="77" t="inlineStr">
+        <is>
+          <t>SL-L — Max RSI</t>
+        </is>
+      </c>
+      <c r="I4" s="79" t="inlineStr">
+        <is>
+          <t>SL-L — Max GCT (s)</t>
+        </is>
+      </c>
+      <c r="J4" s="78" t="inlineStr">
+        <is>
+          <t>SL-R — Avg RSI</t>
+        </is>
+      </c>
+      <c r="K4" s="77" t="inlineStr">
+        <is>
+          <t>SL-R — Avg GCT (s)</t>
+        </is>
+      </c>
+      <c r="L4" s="77" t="inlineStr">
+        <is>
+          <t>SL-R — Max RSI</t>
+        </is>
+      </c>
+      <c r="M4" s="79" t="inlineStr">
+        <is>
+          <t>SL-R — Max GCT (s)</t>
         </is>
       </c>
     </row>
@@ -5449,14 +5646,14 @@
       <c r="C5" s="8" t="n"/>
       <c r="D5" s="8" t="n"/>
       <c r="E5" s="8" t="n"/>
-      <c r="F5" s="8" t="n"/>
+      <c r="F5" s="69" t="n"/>
       <c r="G5" s="8" t="n"/>
       <c r="H5" s="8" t="n"/>
       <c r="I5" s="8" t="n"/>
-      <c r="J5" s="8" t="n"/>
+      <c r="J5" s="69" t="n"/>
       <c r="K5" s="8" t="n"/>
       <c r="L5" s="8" t="n"/>
-      <c r="M5" s="8" t="n"/>
+      <c r="M5" s="70" t="n"/>
     </row>
     <row r="6" ht="18" customFormat="1" customHeight="1" s="1">
       <c r="A6" s="9" t="n"/>
@@ -5464,14 +5661,14 @@
       <c r="C6" s="9" t="n"/>
       <c r="D6" s="9" t="n"/>
       <c r="E6" s="9" t="n"/>
-      <c r="F6" s="9" t="n"/>
+      <c r="F6" s="71" t="n"/>
       <c r="G6" s="9" t="n"/>
       <c r="H6" s="9" t="n"/>
       <c r="I6" s="9" t="n"/>
-      <c r="J6" s="9" t="n"/>
+      <c r="J6" s="71" t="n"/>
       <c r="K6" s="9" t="n"/>
       <c r="L6" s="9" t="n"/>
-      <c r="M6" s="9" t="n"/>
+      <c r="M6" s="72" t="n"/>
     </row>
     <row r="7" ht="18" customFormat="1" customHeight="1" s="1">
       <c r="A7" s="8" t="n"/>
@@ -5479,14 +5676,14 @@
       <c r="C7" s="8" t="n"/>
       <c r="D7" s="8" t="n"/>
       <c r="E7" s="8" t="n"/>
-      <c r="F7" s="8" t="n"/>
+      <c r="F7" s="69" t="n"/>
       <c r="G7" s="8" t="n"/>
       <c r="H7" s="8" t="n"/>
       <c r="I7" s="8" t="n"/>
-      <c r="J7" s="8" t="n"/>
+      <c r="J7" s="69" t="n"/>
       <c r="K7" s="8" t="n"/>
       <c r="L7" s="8" t="n"/>
-      <c r="M7" s="8" t="n"/>
+      <c r="M7" s="70" t="n"/>
     </row>
     <row r="8" ht="18" customFormat="1" customHeight="1" s="1">
       <c r="A8" s="9" t="n"/>
@@ -5494,14 +5691,14 @@
       <c r="C8" s="9" t="n"/>
       <c r="D8" s="9" t="n"/>
       <c r="E8" s="9" t="n"/>
-      <c r="F8" s="9" t="n"/>
+      <c r="F8" s="71" t="n"/>
       <c r="G8" s="9" t="n"/>
       <c r="H8" s="9" t="n"/>
       <c r="I8" s="9" t="n"/>
-      <c r="J8" s="9" t="n"/>
+      <c r="J8" s="71" t="n"/>
       <c r="K8" s="9" t="n"/>
       <c r="L8" s="9" t="n"/>
-      <c r="M8" s="9" t="n"/>
+      <c r="M8" s="72" t="n"/>
     </row>
     <row r="9" ht="18" customFormat="1" customHeight="1" s="1">
       <c r="A9" s="8" t="n"/>
@@ -5509,14 +5706,14 @@
       <c r="C9" s="8" t="n"/>
       <c r="D9" s="8" t="n"/>
       <c r="E9" s="8" t="n"/>
-      <c r="F9" s="8" t="n"/>
+      <c r="F9" s="69" t="n"/>
       <c r="G9" s="8" t="n"/>
       <c r="H9" s="8" t="n"/>
       <c r="I9" s="8" t="n"/>
-      <c r="J9" s="8" t="n"/>
+      <c r="J9" s="69" t="n"/>
       <c r="K9" s="8" t="n"/>
       <c r="L9" s="8" t="n"/>
-      <c r="M9" s="8" t="n"/>
+      <c r="M9" s="70" t="n"/>
     </row>
     <row r="10" ht="18" customFormat="1" customHeight="1" s="1">
       <c r="A10" s="9" t="n"/>
@@ -5524,14 +5721,14 @@
       <c r="C10" s="9" t="n"/>
       <c r="D10" s="9" t="n"/>
       <c r="E10" s="9" t="n"/>
-      <c r="F10" s="9" t="n"/>
+      <c r="F10" s="71" t="n"/>
       <c r="G10" s="9" t="n"/>
       <c r="H10" s="9" t="n"/>
       <c r="I10" s="9" t="n"/>
-      <c r="J10" s="9" t="n"/>
+      <c r="J10" s="71" t="n"/>
       <c r="K10" s="9" t="n"/>
       <c r="L10" s="9" t="n"/>
-      <c r="M10" s="9" t="n"/>
+      <c r="M10" s="72" t="n"/>
     </row>
     <row r="11" ht="18" customFormat="1" customHeight="1" s="1">
       <c r="A11" s="8" t="n"/>
@@ -5539,14 +5736,14 @@
       <c r="C11" s="8" t="n"/>
       <c r="D11" s="8" t="n"/>
       <c r="E11" s="8" t="n"/>
-      <c r="F11" s="8" t="n"/>
+      <c r="F11" s="69" t="n"/>
       <c r="G11" s="8" t="n"/>
       <c r="H11" s="8" t="n"/>
       <c r="I11" s="8" t="n"/>
-      <c r="J11" s="8" t="n"/>
+      <c r="J11" s="69" t="n"/>
       <c r="K11" s="8" t="n"/>
       <c r="L11" s="8" t="n"/>
-      <c r="M11" s="8" t="n"/>
+      <c r="M11" s="70" t="n"/>
     </row>
     <row r="12" ht="18" customFormat="1" customHeight="1" s="1">
       <c r="A12" s="9" t="n"/>
@@ -5554,14 +5751,14 @@
       <c r="C12" s="9" t="n"/>
       <c r="D12" s="9" t="n"/>
       <c r="E12" s="9" t="n"/>
-      <c r="F12" s="9" t="n"/>
+      <c r="F12" s="71" t="n"/>
       <c r="G12" s="9" t="n"/>
       <c r="H12" s="9" t="n"/>
       <c r="I12" s="9" t="n"/>
-      <c r="J12" s="9" t="n"/>
+      <c r="J12" s="71" t="n"/>
       <c r="K12" s="9" t="n"/>
       <c r="L12" s="9" t="n"/>
-      <c r="M12" s="9" t="n"/>
+      <c r="M12" s="72" t="n"/>
     </row>
     <row r="13" ht="18" customFormat="1" customHeight="1" s="1">
       <c r="A13" s="8" t="n"/>
@@ -5569,14 +5766,14 @@
       <c r="C13" s="8" t="n"/>
       <c r="D13" s="8" t="n"/>
       <c r="E13" s="8" t="n"/>
-      <c r="F13" s="8" t="n"/>
+      <c r="F13" s="69" t="n"/>
       <c r="G13" s="8" t="n"/>
       <c r="H13" s="8" t="n"/>
       <c r="I13" s="8" t="n"/>
-      <c r="J13" s="8" t="n"/>
+      <c r="J13" s="69" t="n"/>
       <c r="K13" s="8" t="n"/>
       <c r="L13" s="8" t="n"/>
-      <c r="M13" s="8" t="n"/>
+      <c r="M13" s="70" t="n"/>
     </row>
     <row r="14" ht="18" customFormat="1" customHeight="1" s="1">
       <c r="A14" s="9" t="n"/>
@@ -5584,14 +5781,14 @@
       <c r="C14" s="9" t="n"/>
       <c r="D14" s="9" t="n"/>
       <c r="E14" s="9" t="n"/>
-      <c r="F14" s="9" t="n"/>
+      <c r="F14" s="71" t="n"/>
       <c r="G14" s="9" t="n"/>
       <c r="H14" s="9" t="n"/>
       <c r="I14" s="9" t="n"/>
-      <c r="J14" s="9" t="n"/>
+      <c r="J14" s="71" t="n"/>
       <c r="K14" s="9" t="n"/>
       <c r="L14" s="9" t="n"/>
-      <c r="M14" s="9" t="n"/>
+      <c r="M14" s="72" t="n"/>
     </row>
     <row r="15" ht="18" customFormat="1" customHeight="1" s="1">
       <c r="A15" s="8" t="n"/>
@@ -5599,14 +5796,14 @@
       <c r="C15" s="8" t="n"/>
       <c r="D15" s="8" t="n"/>
       <c r="E15" s="8" t="n"/>
-      <c r="F15" s="8" t="n"/>
+      <c r="F15" s="69" t="n"/>
       <c r="G15" s="8" t="n"/>
       <c r="H15" s="8" t="n"/>
       <c r="I15" s="8" t="n"/>
-      <c r="J15" s="8" t="n"/>
+      <c r="J15" s="69" t="n"/>
       <c r="K15" s="8" t="n"/>
       <c r="L15" s="8" t="n"/>
-      <c r="M15" s="8" t="n"/>
+      <c r="M15" s="70" t="n"/>
     </row>
     <row r="16" ht="18" customFormat="1" customHeight="1" s="1">
       <c r="A16" s="9" t="n"/>
@@ -5614,14 +5811,14 @@
       <c r="C16" s="9" t="n"/>
       <c r="D16" s="9" t="n"/>
       <c r="E16" s="9" t="n"/>
-      <c r="F16" s="9" t="n"/>
+      <c r="F16" s="71" t="n"/>
       <c r="G16" s="9" t="n"/>
       <c r="H16" s="9" t="n"/>
       <c r="I16" s="9" t="n"/>
-      <c r="J16" s="9" t="n"/>
+      <c r="J16" s="71" t="n"/>
       <c r="K16" s="9" t="n"/>
       <c r="L16" s="9" t="n"/>
-      <c r="M16" s="9" t="n"/>
+      <c r="M16" s="72" t="n"/>
     </row>
     <row r="17" ht="18" customFormat="1" customHeight="1" s="1">
       <c r="A17" s="8" t="n"/>
@@ -5629,14 +5826,14 @@
       <c r="C17" s="8" t="n"/>
       <c r="D17" s="8" t="n"/>
       <c r="E17" s="8" t="n"/>
-      <c r="F17" s="8" t="n"/>
+      <c r="F17" s="69" t="n"/>
       <c r="G17" s="8" t="n"/>
       <c r="H17" s="8" t="n"/>
       <c r="I17" s="8" t="n"/>
-      <c r="J17" s="8" t="n"/>
+      <c r="J17" s="69" t="n"/>
       <c r="K17" s="8" t="n"/>
       <c r="L17" s="8" t="n"/>
-      <c r="M17" s="8" t="n"/>
+      <c r="M17" s="70" t="n"/>
     </row>
     <row r="18" ht="18" customFormat="1" customHeight="1" s="1">
       <c r="A18" s="9" t="n"/>
@@ -5644,14 +5841,14 @@
       <c r="C18" s="9" t="n"/>
       <c r="D18" s="9" t="n"/>
       <c r="E18" s="9" t="n"/>
-      <c r="F18" s="9" t="n"/>
+      <c r="F18" s="71" t="n"/>
       <c r="G18" s="9" t="n"/>
       <c r="H18" s="9" t="n"/>
       <c r="I18" s="9" t="n"/>
-      <c r="J18" s="9" t="n"/>
+      <c r="J18" s="71" t="n"/>
       <c r="K18" s="9" t="n"/>
       <c r="L18" s="9" t="n"/>
-      <c r="M18" s="9" t="n"/>
+      <c r="M18" s="72" t="n"/>
     </row>
     <row r="19" ht="18" customFormat="1" customHeight="1" s="1">
       <c r="A19" s="8" t="n"/>
@@ -5659,14 +5856,14 @@
       <c r="C19" s="8" t="n"/>
       <c r="D19" s="8" t="n"/>
       <c r="E19" s="8" t="n"/>
-      <c r="F19" s="8" t="n"/>
+      <c r="F19" s="69" t="n"/>
       <c r="G19" s="8" t="n"/>
       <c r="H19" s="8" t="n"/>
       <c r="I19" s="8" t="n"/>
-      <c r="J19" s="8" t="n"/>
+      <c r="J19" s="69" t="n"/>
       <c r="K19" s="8" t="n"/>
       <c r="L19" s="8" t="n"/>
-      <c r="M19" s="8" t="n"/>
+      <c r="M19" s="70" t="n"/>
     </row>
     <row r="20" ht="18" customFormat="1" customHeight="1" s="1">
       <c r="A20" s="9" t="n"/>
@@ -5674,14 +5871,14 @@
       <c r="C20" s="9" t="n"/>
       <c r="D20" s="9" t="n"/>
       <c r="E20" s="9" t="n"/>
-      <c r="F20" s="9" t="n"/>
+      <c r="F20" s="71" t="n"/>
       <c r="G20" s="9" t="n"/>
       <c r="H20" s="9" t="n"/>
       <c r="I20" s="9" t="n"/>
-      <c r="J20" s="9" t="n"/>
+      <c r="J20" s="71" t="n"/>
       <c r="K20" s="9" t="n"/>
       <c r="L20" s="9" t="n"/>
-      <c r="M20" s="9" t="n"/>
+      <c r="M20" s="72" t="n"/>
     </row>
     <row r="21" ht="18" customFormat="1" customHeight="1" s="1">
       <c r="A21" s="8" t="n"/>
@@ -5689,14 +5886,14 @@
       <c r="C21" s="8" t="n"/>
       <c r="D21" s="8" t="n"/>
       <c r="E21" s="8" t="n"/>
-      <c r="F21" s="8" t="n"/>
+      <c r="F21" s="69" t="n"/>
       <c r="G21" s="8" t="n"/>
       <c r="H21" s="8" t="n"/>
       <c r="I21" s="8" t="n"/>
-      <c r="J21" s="8" t="n"/>
+      <c r="J21" s="69" t="n"/>
       <c r="K21" s="8" t="n"/>
       <c r="L21" s="8" t="n"/>
-      <c r="M21" s="8" t="n"/>
+      <c r="M21" s="70" t="n"/>
     </row>
     <row r="22" ht="18" customFormat="1" customHeight="1" s="1">
       <c r="A22" s="9" t="n"/>
@@ -5704,14 +5901,14 @@
       <c r="C22" s="9" t="n"/>
       <c r="D22" s="9" t="n"/>
       <c r="E22" s="9" t="n"/>
-      <c r="F22" s="9" t="n"/>
+      <c r="F22" s="71" t="n"/>
       <c r="G22" s="9" t="n"/>
       <c r="H22" s="9" t="n"/>
       <c r="I22" s="9" t="n"/>
-      <c r="J22" s="9" t="n"/>
+      <c r="J22" s="71" t="n"/>
       <c r="K22" s="9" t="n"/>
       <c r="L22" s="9" t="n"/>
-      <c r="M22" s="9" t="n"/>
+      <c r="M22" s="72" t="n"/>
     </row>
     <row r="23" ht="18" customFormat="1" customHeight="1" s="1">
       <c r="A23" s="8" t="n"/>
@@ -5719,14 +5916,14 @@
       <c r="C23" s="8" t="n"/>
       <c r="D23" s="8" t="n"/>
       <c r="E23" s="8" t="n"/>
-      <c r="F23" s="8" t="n"/>
+      <c r="F23" s="69" t="n"/>
       <c r="G23" s="8" t="n"/>
       <c r="H23" s="8" t="n"/>
       <c r="I23" s="8" t="n"/>
-      <c r="J23" s="8" t="n"/>
+      <c r="J23" s="69" t="n"/>
       <c r="K23" s="8" t="n"/>
       <c r="L23" s="8" t="n"/>
-      <c r="M23" s="8" t="n"/>
+      <c r="M23" s="70" t="n"/>
     </row>
     <row r="24" ht="18" customFormat="1" customHeight="1" s="1">
       <c r="A24" s="9" t="n"/>
@@ -5734,14 +5931,14 @@
       <c r="C24" s="9" t="n"/>
       <c r="D24" s="9" t="n"/>
       <c r="E24" s="9" t="n"/>
-      <c r="F24" s="9" t="n"/>
+      <c r="F24" s="71" t="n"/>
       <c r="G24" s="9" t="n"/>
       <c r="H24" s="9" t="n"/>
       <c r="I24" s="9" t="n"/>
-      <c r="J24" s="9" t="n"/>
+      <c r="J24" s="71" t="n"/>
       <c r="K24" s="9" t="n"/>
       <c r="L24" s="9" t="n"/>
-      <c r="M24" s="9" t="n"/>
+      <c r="M24" s="72" t="n"/>
     </row>
     <row r="25" ht="18" customFormat="1" customHeight="1" s="1">
       <c r="A25" s="8" t="n"/>
@@ -5749,14 +5946,14 @@
       <c r="C25" s="8" t="n"/>
       <c r="D25" s="8" t="n"/>
       <c r="E25" s="8" t="n"/>
-      <c r="F25" s="8" t="n"/>
+      <c r="F25" s="69" t="n"/>
       <c r="G25" s="8" t="n"/>
       <c r="H25" s="8" t="n"/>
       <c r="I25" s="8" t="n"/>
-      <c r="J25" s="8" t="n"/>
+      <c r="J25" s="69" t="n"/>
       <c r="K25" s="8" t="n"/>
       <c r="L25" s="8" t="n"/>
-      <c r="M25" s="8" t="n"/>
+      <c r="M25" s="70" t="n"/>
     </row>
     <row r="26" ht="18" customFormat="1" customHeight="1" s="1">
       <c r="A26" s="9" t="n"/>
@@ -5764,14 +5961,14 @@
       <c r="C26" s="9" t="n"/>
       <c r="D26" s="9" t="n"/>
       <c r="E26" s="9" t="n"/>
-      <c r="F26" s="9" t="n"/>
+      <c r="F26" s="71" t="n"/>
       <c r="G26" s="9" t="n"/>
       <c r="H26" s="9" t="n"/>
       <c r="I26" s="9" t="n"/>
-      <c r="J26" s="9" t="n"/>
+      <c r="J26" s="71" t="n"/>
       <c r="K26" s="9" t="n"/>
       <c r="L26" s="9" t="n"/>
-      <c r="M26" s="9" t="n"/>
+      <c r="M26" s="72" t="n"/>
     </row>
     <row r="27" ht="18" customFormat="1" customHeight="1" s="1">
       <c r="A27" s="8" t="n"/>
@@ -5779,14 +5976,14 @@
       <c r="C27" s="8" t="n"/>
       <c r="D27" s="8" t="n"/>
       <c r="E27" s="8" t="n"/>
-      <c r="F27" s="8" t="n"/>
+      <c r="F27" s="69" t="n"/>
       <c r="G27" s="8" t="n"/>
       <c r="H27" s="8" t="n"/>
       <c r="I27" s="8" t="n"/>
-      <c r="J27" s="8" t="n"/>
+      <c r="J27" s="69" t="n"/>
       <c r="K27" s="8" t="n"/>
       <c r="L27" s="8" t="n"/>
-      <c r="M27" s="8" t="n"/>
+      <c r="M27" s="70" t="n"/>
     </row>
     <row r="28" ht="18" customFormat="1" customHeight="1" s="1">
       <c r="A28" s="9" t="n"/>
@@ -5794,14 +5991,14 @@
       <c r="C28" s="9" t="n"/>
       <c r="D28" s="9" t="n"/>
       <c r="E28" s="9" t="n"/>
-      <c r="F28" s="9" t="n"/>
+      <c r="F28" s="71" t="n"/>
       <c r="G28" s="9" t="n"/>
       <c r="H28" s="9" t="n"/>
       <c r="I28" s="9" t="n"/>
-      <c r="J28" s="9" t="n"/>
+      <c r="J28" s="71" t="n"/>
       <c r="K28" s="9" t="n"/>
       <c r="L28" s="9" t="n"/>
-      <c r="M28" s="9" t="n"/>
+      <c r="M28" s="72" t="n"/>
     </row>
     <row r="29" ht="18" customFormat="1" customHeight="1" s="1">
       <c r="A29" s="8" t="n"/>
@@ -5809,14 +6006,14 @@
       <c r="C29" s="8" t="n"/>
       <c r="D29" s="8" t="n"/>
       <c r="E29" s="8" t="n"/>
-      <c r="F29" s="8" t="n"/>
+      <c r="F29" s="69" t="n"/>
       <c r="G29" s="8" t="n"/>
       <c r="H29" s="8" t="n"/>
       <c r="I29" s="8" t="n"/>
-      <c r="J29" s="8" t="n"/>
+      <c r="J29" s="69" t="n"/>
       <c r="K29" s="8" t="n"/>
       <c r="L29" s="8" t="n"/>
-      <c r="M29" s="8" t="n"/>
+      <c r="M29" s="70" t="n"/>
     </row>
     <row r="30" ht="18" customFormat="1" customHeight="1" s="1">
       <c r="A30" s="9" t="n"/>
@@ -5824,14 +6021,14 @@
       <c r="C30" s="9" t="n"/>
       <c r="D30" s="9" t="n"/>
       <c r="E30" s="9" t="n"/>
-      <c r="F30" s="9" t="n"/>
+      <c r="F30" s="71" t="n"/>
       <c r="G30" s="9" t="n"/>
       <c r="H30" s="9" t="n"/>
       <c r="I30" s="9" t="n"/>
-      <c r="J30" s="9" t="n"/>
+      <c r="J30" s="71" t="n"/>
       <c r="K30" s="9" t="n"/>
       <c r="L30" s="9" t="n"/>
-      <c r="M30" s="9" t="n"/>
+      <c r="M30" s="72" t="n"/>
     </row>
     <row r="31" ht="18" customFormat="1" customHeight="1" s="1">
       <c r="A31" s="8" t="n"/>
@@ -5839,14 +6036,14 @@
       <c r="C31" s="8" t="n"/>
       <c r="D31" s="8" t="n"/>
       <c r="E31" s="8" t="n"/>
-      <c r="F31" s="8" t="n"/>
+      <c r="F31" s="69" t="n"/>
       <c r="G31" s="8" t="n"/>
       <c r="H31" s="8" t="n"/>
       <c r="I31" s="8" t="n"/>
-      <c r="J31" s="8" t="n"/>
+      <c r="J31" s="69" t="n"/>
       <c r="K31" s="8" t="n"/>
       <c r="L31" s="8" t="n"/>
-      <c r="M31" s="8" t="n"/>
+      <c r="M31" s="70" t="n"/>
     </row>
     <row r="32" ht="18" customFormat="1" customHeight="1" s="1">
       <c r="A32" s="9" t="n"/>
@@ -5854,14 +6051,14 @@
       <c r="C32" s="9" t="n"/>
       <c r="D32" s="9" t="n"/>
       <c r="E32" s="9" t="n"/>
-      <c r="F32" s="9" t="n"/>
+      <c r="F32" s="71" t="n"/>
       <c r="G32" s="9" t="n"/>
       <c r="H32" s="9" t="n"/>
       <c r="I32" s="9" t="n"/>
-      <c r="J32" s="9" t="n"/>
+      <c r="J32" s="71" t="n"/>
       <c r="K32" s="9" t="n"/>
       <c r="L32" s="9" t="n"/>
-      <c r="M32" s="9" t="n"/>
+      <c r="M32" s="72" t="n"/>
     </row>
     <row r="33" ht="18" customFormat="1" customHeight="1" s="1">
       <c r="A33" s="8" t="n"/>
@@ -5869,14 +6066,14 @@
       <c r="C33" s="8" t="n"/>
       <c r="D33" s="8" t="n"/>
       <c r="E33" s="8" t="n"/>
-      <c r="F33" s="8" t="n"/>
+      <c r="F33" s="69" t="n"/>
       <c r="G33" s="8" t="n"/>
       <c r="H33" s="8" t="n"/>
       <c r="I33" s="8" t="n"/>
-      <c r="J33" s="8" t="n"/>
+      <c r="J33" s="69" t="n"/>
       <c r="K33" s="8" t="n"/>
       <c r="L33" s="8" t="n"/>
-      <c r="M33" s="8" t="n"/>
+      <c r="M33" s="70" t="n"/>
     </row>
     <row r="34" ht="18" customFormat="1" customHeight="1" s="1">
       <c r="A34" s="9" t="n"/>
@@ -5884,14 +6081,14 @@
       <c r="C34" s="9" t="n"/>
       <c r="D34" s="9" t="n"/>
       <c r="E34" s="9" t="n"/>
-      <c r="F34" s="9" t="n"/>
+      <c r="F34" s="71" t="n"/>
       <c r="G34" s="9" t="n"/>
       <c r="H34" s="9" t="n"/>
       <c r="I34" s="9" t="n"/>
-      <c r="J34" s="9" t="n"/>
+      <c r="J34" s="71" t="n"/>
       <c r="K34" s="9" t="n"/>
       <c r="L34" s="9" t="n"/>
-      <c r="M34" s="9" t="n"/>
+      <c r="M34" s="72" t="n"/>
     </row>
     <row r="35" ht="18" customFormat="1" customHeight="1" s="1">
       <c r="A35" s="10" t="inlineStr">

</xml_diff>

<commit_message>
Add drop jump RSI (40/50/60cm) — template columns N-V, transformer, engine classification and optimal height detection
</commit_message>
<xml_diff>
--- a/public/AMSC_Combine_Data_Template.xlsx
+++ b/public/AMSC_Combine_Data_Template.xlsx
@@ -189,7 +189,7 @@
       <sz val="9"/>
     </font>
   </fonts>
-  <fills count="15">
+  <fills count="16">
     <fill>
       <patternFill/>
     </fill>
@@ -261,8 +261,13 @@
         <fgColor rgb="FFC41E3A"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF1A2A4A"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="29">
+  <borders count="32">
     <border>
       <left/>
       <right/>
@@ -537,11 +542,29 @@
       <bottom style="thin"/>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium"/>
+      <right/>
+      <top/>
+      <bottom/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <right/>
+      <top/>
+      <bottom/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <right style="medium"/>
+      <top/>
+      <bottom/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2"/>
   </cellStyleXfs>
-  <cellXfs count="80">
+  <cellXfs count="92">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
@@ -760,6 +783,32 @@
     <xf numFmtId="0" fontId="24" fillId="14" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="23" fillId="13" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="27" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="28" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="23" fillId="15" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="15" borderId="16" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="15" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="15" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="15" borderId="16" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="15" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="29" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="30" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="31" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -5486,7 +5535,7 @@
     <outlinePr summaryBelow="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M35"/>
+  <dimension ref="A1:V35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22.005" bestFit="1" customWidth="1" style="16" min="1" max="1"/>
@@ -5502,6 +5551,15 @@
     <col width="13.005" bestFit="1" customWidth="1" style="38" min="11" max="11"/>
     <col width="13.005" bestFit="1" customWidth="1" style="38" min="12" max="12"/>
     <col width="13.005" bestFit="1" customWidth="1" style="38" min="13" max="13"/>
+    <col width="13" customWidth="1" min="14" max="14"/>
+    <col width="13" customWidth="1" min="15" max="15"/>
+    <col width="13" customWidth="1" min="16" max="16"/>
+    <col width="13" customWidth="1" min="17" max="17"/>
+    <col width="13" customWidth="1" min="18" max="18"/>
+    <col width="13" customWidth="1" min="19" max="19"/>
+    <col width="13" customWidth="1" min="20" max="20"/>
+    <col width="13" customWidth="1" min="21" max="21"/>
+    <col width="13" customWidth="1" min="22" max="22"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customFormat="1" customHeight="1" s="1">
@@ -5548,30 +5606,51 @@
           <t>ATHLETE INFO</t>
         </is>
       </c>
-      <c r="B3" s="74" t="inlineStr">
+      <c r="B3" s="80" t="inlineStr">
         <is>
           <t>DOUBLE-LEG</t>
         </is>
       </c>
-      <c r="C3" s="75" t="n"/>
-      <c r="D3" s="75" t="n"/>
-      <c r="E3" s="76" t="n"/>
-      <c r="F3" s="74" t="inlineStr">
+      <c r="C3" s="81" t="n"/>
+      <c r="D3" s="81" t="n"/>
+      <c r="E3" s="82" t="n"/>
+      <c r="F3" s="80" t="inlineStr">
         <is>
           <t>SINGLE-LEG LEFT</t>
         </is>
       </c>
-      <c r="G3" s="75" t="n"/>
-      <c r="H3" s="75" t="n"/>
-      <c r="I3" s="76" t="n"/>
-      <c r="J3" s="74" t="inlineStr">
+      <c r="G3" s="81" t="n"/>
+      <c r="H3" s="81" t="n"/>
+      <c r="I3" s="82" t="n"/>
+      <c r="J3" s="80" t="inlineStr">
         <is>
           <t>SINGLE-LEG RIGHT</t>
         </is>
       </c>
-      <c r="K3" s="75" t="n"/>
-      <c r="L3" s="75" t="n"/>
-      <c r="M3" s="76" t="n"/>
+      <c r="K3" s="81" t="n"/>
+      <c r="L3" s="81" t="n"/>
+      <c r="M3" s="82" t="n"/>
+      <c r="N3" s="83" t="inlineStr">
+        <is>
+          <t>40cm DROP JUMP</t>
+        </is>
+      </c>
+      <c r="O3" s="84" t="n"/>
+      <c r="P3" s="85" t="n"/>
+      <c r="Q3" s="83" t="inlineStr">
+        <is>
+          <t>50cm DROP JUMP</t>
+        </is>
+      </c>
+      <c r="R3" s="84" t="n"/>
+      <c r="S3" s="85" t="n"/>
+      <c r="T3" s="83" t="inlineStr">
+        <is>
+          <t>60cm DROP JUMP</t>
+        </is>
+      </c>
+      <c r="U3" s="84" t="n"/>
+      <c r="V3" s="85" t="n"/>
     </row>
     <row r="4" ht="30" customFormat="1" customHeight="1" s="1">
       <c r="A4" s="77" t="inlineStr">
@@ -5637,6 +5716,51 @@
       <c r="M4" s="79" t="inlineStr">
         <is>
           <t>SL-R — Max GCT (s)</t>
+        </is>
+      </c>
+      <c r="N4" s="86" t="inlineStr">
+        <is>
+          <t>RSI</t>
+        </is>
+      </c>
+      <c r="O4" s="87" t="inlineStr">
+        <is>
+          <t>Jump Ht (cm)</t>
+        </is>
+      </c>
+      <c r="P4" s="88" t="inlineStr">
+        <is>
+          <t>GCT (s)</t>
+        </is>
+      </c>
+      <c r="Q4" s="86" t="inlineStr">
+        <is>
+          <t>RSI</t>
+        </is>
+      </c>
+      <c r="R4" s="87" t="inlineStr">
+        <is>
+          <t>Jump Ht (cm)</t>
+        </is>
+      </c>
+      <c r="S4" s="88" t="inlineStr">
+        <is>
+          <t>GCT (s)</t>
+        </is>
+      </c>
+      <c r="T4" s="86" t="inlineStr">
+        <is>
+          <t>RSI</t>
+        </is>
+      </c>
+      <c r="U4" s="87" t="inlineStr">
+        <is>
+          <t>Jump Ht (cm)</t>
+        </is>
+      </c>
+      <c r="V4" s="88" t="inlineStr">
+        <is>
+          <t>GCT (s)</t>
         </is>
       </c>
     </row>
@@ -5654,6 +5778,15 @@
       <c r="K5" s="8" t="n"/>
       <c r="L5" s="8" t="n"/>
       <c r="M5" s="70" t="n"/>
+      <c r="N5" s="89" t="n"/>
+      <c r="O5" s="90" t="n"/>
+      <c r="P5" s="91" t="n"/>
+      <c r="Q5" s="89" t="n"/>
+      <c r="R5" s="90" t="n"/>
+      <c r="S5" s="91" t="n"/>
+      <c r="T5" s="89" t="n"/>
+      <c r="U5" s="90" t="n"/>
+      <c r="V5" s="91" t="n"/>
     </row>
     <row r="6" ht="18" customFormat="1" customHeight="1" s="1">
       <c r="A6" s="9" t="n"/>
@@ -5669,6 +5802,15 @@
       <c r="K6" s="9" t="n"/>
       <c r="L6" s="9" t="n"/>
       <c r="M6" s="72" t="n"/>
+      <c r="N6" s="89" t="n"/>
+      <c r="O6" s="90" t="n"/>
+      <c r="P6" s="91" t="n"/>
+      <c r="Q6" s="89" t="n"/>
+      <c r="R6" s="90" t="n"/>
+      <c r="S6" s="91" t="n"/>
+      <c r="T6" s="89" t="n"/>
+      <c r="U6" s="90" t="n"/>
+      <c r="V6" s="91" t="n"/>
     </row>
     <row r="7" ht="18" customFormat="1" customHeight="1" s="1">
       <c r="A7" s="8" t="n"/>
@@ -5684,6 +5826,15 @@
       <c r="K7" s="8" t="n"/>
       <c r="L7" s="8" t="n"/>
       <c r="M7" s="70" t="n"/>
+      <c r="N7" s="89" t="n"/>
+      <c r="O7" s="90" t="n"/>
+      <c r="P7" s="91" t="n"/>
+      <c r="Q7" s="89" t="n"/>
+      <c r="R7" s="90" t="n"/>
+      <c r="S7" s="91" t="n"/>
+      <c r="T7" s="89" t="n"/>
+      <c r="U7" s="90" t="n"/>
+      <c r="V7" s="91" t="n"/>
     </row>
     <row r="8" ht="18" customFormat="1" customHeight="1" s="1">
       <c r="A8" s="9" t="n"/>
@@ -5699,6 +5850,15 @@
       <c r="K8" s="9" t="n"/>
       <c r="L8" s="9" t="n"/>
       <c r="M8" s="72" t="n"/>
+      <c r="N8" s="89" t="n"/>
+      <c r="O8" s="90" t="n"/>
+      <c r="P8" s="91" t="n"/>
+      <c r="Q8" s="89" t="n"/>
+      <c r="R8" s="90" t="n"/>
+      <c r="S8" s="91" t="n"/>
+      <c r="T8" s="89" t="n"/>
+      <c r="U8" s="90" t="n"/>
+      <c r="V8" s="91" t="n"/>
     </row>
     <row r="9" ht="18" customFormat="1" customHeight="1" s="1">
       <c r="A9" s="8" t="n"/>
@@ -5714,6 +5874,15 @@
       <c r="K9" s="8" t="n"/>
       <c r="L9" s="8" t="n"/>
       <c r="M9" s="70" t="n"/>
+      <c r="N9" s="89" t="n"/>
+      <c r="O9" s="90" t="n"/>
+      <c r="P9" s="91" t="n"/>
+      <c r="Q9" s="89" t="n"/>
+      <c r="R9" s="90" t="n"/>
+      <c r="S9" s="91" t="n"/>
+      <c r="T9" s="89" t="n"/>
+      <c r="U9" s="90" t="n"/>
+      <c r="V9" s="91" t="n"/>
     </row>
     <row r="10" ht="18" customFormat="1" customHeight="1" s="1">
       <c r="A10" s="9" t="n"/>
@@ -5729,6 +5898,15 @@
       <c r="K10" s="9" t="n"/>
       <c r="L10" s="9" t="n"/>
       <c r="M10" s="72" t="n"/>
+      <c r="N10" s="89" t="n"/>
+      <c r="O10" s="90" t="n"/>
+      <c r="P10" s="91" t="n"/>
+      <c r="Q10" s="89" t="n"/>
+      <c r="R10" s="90" t="n"/>
+      <c r="S10" s="91" t="n"/>
+      <c r="T10" s="89" t="n"/>
+      <c r="U10" s="90" t="n"/>
+      <c r="V10" s="91" t="n"/>
     </row>
     <row r="11" ht="18" customFormat="1" customHeight="1" s="1">
       <c r="A11" s="8" t="n"/>
@@ -5744,6 +5922,15 @@
       <c r="K11" s="8" t="n"/>
       <c r="L11" s="8" t="n"/>
       <c r="M11" s="70" t="n"/>
+      <c r="N11" s="89" t="n"/>
+      <c r="O11" s="90" t="n"/>
+      <c r="P11" s="91" t="n"/>
+      <c r="Q11" s="89" t="n"/>
+      <c r="R11" s="90" t="n"/>
+      <c r="S11" s="91" t="n"/>
+      <c r="T11" s="89" t="n"/>
+      <c r="U11" s="90" t="n"/>
+      <c r="V11" s="91" t="n"/>
     </row>
     <row r="12" ht="18" customFormat="1" customHeight="1" s="1">
       <c r="A12" s="9" t="n"/>
@@ -5759,6 +5946,15 @@
       <c r="K12" s="9" t="n"/>
       <c r="L12" s="9" t="n"/>
       <c r="M12" s="72" t="n"/>
+      <c r="N12" s="89" t="n"/>
+      <c r="O12" s="90" t="n"/>
+      <c r="P12" s="91" t="n"/>
+      <c r="Q12" s="89" t="n"/>
+      <c r="R12" s="90" t="n"/>
+      <c r="S12" s="91" t="n"/>
+      <c r="T12" s="89" t="n"/>
+      <c r="U12" s="90" t="n"/>
+      <c r="V12" s="91" t="n"/>
     </row>
     <row r="13" ht="18" customFormat="1" customHeight="1" s="1">
       <c r="A13" s="8" t="n"/>
@@ -5774,6 +5970,15 @@
       <c r="K13" s="8" t="n"/>
       <c r="L13" s="8" t="n"/>
       <c r="M13" s="70" t="n"/>
+      <c r="N13" s="89" t="n"/>
+      <c r="O13" s="90" t="n"/>
+      <c r="P13" s="91" t="n"/>
+      <c r="Q13" s="89" t="n"/>
+      <c r="R13" s="90" t="n"/>
+      <c r="S13" s="91" t="n"/>
+      <c r="T13" s="89" t="n"/>
+      <c r="U13" s="90" t="n"/>
+      <c r="V13" s="91" t="n"/>
     </row>
     <row r="14" ht="18" customFormat="1" customHeight="1" s="1">
       <c r="A14" s="9" t="n"/>
@@ -5789,6 +5994,15 @@
       <c r="K14" s="9" t="n"/>
       <c r="L14" s="9" t="n"/>
       <c r="M14" s="72" t="n"/>
+      <c r="N14" s="89" t="n"/>
+      <c r="O14" s="90" t="n"/>
+      <c r="P14" s="91" t="n"/>
+      <c r="Q14" s="89" t="n"/>
+      <c r="R14" s="90" t="n"/>
+      <c r="S14" s="91" t="n"/>
+      <c r="T14" s="89" t="n"/>
+      <c r="U14" s="90" t="n"/>
+      <c r="V14" s="91" t="n"/>
     </row>
     <row r="15" ht="18" customFormat="1" customHeight="1" s="1">
       <c r="A15" s="8" t="n"/>
@@ -5804,6 +6018,15 @@
       <c r="K15" s="8" t="n"/>
       <c r="L15" s="8" t="n"/>
       <c r="M15" s="70" t="n"/>
+      <c r="N15" s="89" t="n"/>
+      <c r="O15" s="90" t="n"/>
+      <c r="P15" s="91" t="n"/>
+      <c r="Q15" s="89" t="n"/>
+      <c r="R15" s="90" t="n"/>
+      <c r="S15" s="91" t="n"/>
+      <c r="T15" s="89" t="n"/>
+      <c r="U15" s="90" t="n"/>
+      <c r="V15" s="91" t="n"/>
     </row>
     <row r="16" ht="18" customFormat="1" customHeight="1" s="1">
       <c r="A16" s="9" t="n"/>
@@ -5819,6 +6042,15 @@
       <c r="K16" s="9" t="n"/>
       <c r="L16" s="9" t="n"/>
       <c r="M16" s="72" t="n"/>
+      <c r="N16" s="89" t="n"/>
+      <c r="O16" s="90" t="n"/>
+      <c r="P16" s="91" t="n"/>
+      <c r="Q16" s="89" t="n"/>
+      <c r="R16" s="90" t="n"/>
+      <c r="S16" s="91" t="n"/>
+      <c r="T16" s="89" t="n"/>
+      <c r="U16" s="90" t="n"/>
+      <c r="V16" s="91" t="n"/>
     </row>
     <row r="17" ht="18" customFormat="1" customHeight="1" s="1">
       <c r="A17" s="8" t="n"/>
@@ -5834,6 +6066,15 @@
       <c r="K17" s="8" t="n"/>
       <c r="L17" s="8" t="n"/>
       <c r="M17" s="70" t="n"/>
+      <c r="N17" s="89" t="n"/>
+      <c r="O17" s="90" t="n"/>
+      <c r="P17" s="91" t="n"/>
+      <c r="Q17" s="89" t="n"/>
+      <c r="R17" s="90" t="n"/>
+      <c r="S17" s="91" t="n"/>
+      <c r="T17" s="89" t="n"/>
+      <c r="U17" s="90" t="n"/>
+      <c r="V17" s="91" t="n"/>
     </row>
     <row r="18" ht="18" customFormat="1" customHeight="1" s="1">
       <c r="A18" s="9" t="n"/>
@@ -5849,6 +6090,15 @@
       <c r="K18" s="9" t="n"/>
       <c r="L18" s="9" t="n"/>
       <c r="M18" s="72" t="n"/>
+      <c r="N18" s="89" t="n"/>
+      <c r="O18" s="90" t="n"/>
+      <c r="P18" s="91" t="n"/>
+      <c r="Q18" s="89" t="n"/>
+      <c r="R18" s="90" t="n"/>
+      <c r="S18" s="91" t="n"/>
+      <c r="T18" s="89" t="n"/>
+      <c r="U18" s="90" t="n"/>
+      <c r="V18" s="91" t="n"/>
     </row>
     <row r="19" ht="18" customFormat="1" customHeight="1" s="1">
       <c r="A19" s="8" t="n"/>
@@ -5864,6 +6114,15 @@
       <c r="K19" s="8" t="n"/>
       <c r="L19" s="8" t="n"/>
       <c r="M19" s="70" t="n"/>
+      <c r="N19" s="89" t="n"/>
+      <c r="O19" s="90" t="n"/>
+      <c r="P19" s="91" t="n"/>
+      <c r="Q19" s="89" t="n"/>
+      <c r="R19" s="90" t="n"/>
+      <c r="S19" s="91" t="n"/>
+      <c r="T19" s="89" t="n"/>
+      <c r="U19" s="90" t="n"/>
+      <c r="V19" s="91" t="n"/>
     </row>
     <row r="20" ht="18" customFormat="1" customHeight="1" s="1">
       <c r="A20" s="9" t="n"/>
@@ -5879,6 +6138,15 @@
       <c r="K20" s="9" t="n"/>
       <c r="L20" s="9" t="n"/>
       <c r="M20" s="72" t="n"/>
+      <c r="N20" s="89" t="n"/>
+      <c r="O20" s="90" t="n"/>
+      <c r="P20" s="91" t="n"/>
+      <c r="Q20" s="89" t="n"/>
+      <c r="R20" s="90" t="n"/>
+      <c r="S20" s="91" t="n"/>
+      <c r="T20" s="89" t="n"/>
+      <c r="U20" s="90" t="n"/>
+      <c r="V20" s="91" t="n"/>
     </row>
     <row r="21" ht="18" customFormat="1" customHeight="1" s="1">
       <c r="A21" s="8" t="n"/>
@@ -5894,6 +6162,15 @@
       <c r="K21" s="8" t="n"/>
       <c r="L21" s="8" t="n"/>
       <c r="M21" s="70" t="n"/>
+      <c r="N21" s="89" t="n"/>
+      <c r="O21" s="90" t="n"/>
+      <c r="P21" s="91" t="n"/>
+      <c r="Q21" s="89" t="n"/>
+      <c r="R21" s="90" t="n"/>
+      <c r="S21" s="91" t="n"/>
+      <c r="T21" s="89" t="n"/>
+      <c r="U21" s="90" t="n"/>
+      <c r="V21" s="91" t="n"/>
     </row>
     <row r="22" ht="18" customFormat="1" customHeight="1" s="1">
       <c r="A22" s="9" t="n"/>
@@ -5909,6 +6186,15 @@
       <c r="K22" s="9" t="n"/>
       <c r="L22" s="9" t="n"/>
       <c r="M22" s="72" t="n"/>
+      <c r="N22" s="89" t="n"/>
+      <c r="O22" s="90" t="n"/>
+      <c r="P22" s="91" t="n"/>
+      <c r="Q22" s="89" t="n"/>
+      <c r="R22" s="90" t="n"/>
+      <c r="S22" s="91" t="n"/>
+      <c r="T22" s="89" t="n"/>
+      <c r="U22" s="90" t="n"/>
+      <c r="V22" s="91" t="n"/>
     </row>
     <row r="23" ht="18" customFormat="1" customHeight="1" s="1">
       <c r="A23" s="8" t="n"/>
@@ -5924,6 +6210,15 @@
       <c r="K23" s="8" t="n"/>
       <c r="L23" s="8" t="n"/>
       <c r="M23" s="70" t="n"/>
+      <c r="N23" s="89" t="n"/>
+      <c r="O23" s="90" t="n"/>
+      <c r="P23" s="91" t="n"/>
+      <c r="Q23" s="89" t="n"/>
+      <c r="R23" s="90" t="n"/>
+      <c r="S23" s="91" t="n"/>
+      <c r="T23" s="89" t="n"/>
+      <c r="U23" s="90" t="n"/>
+      <c r="V23" s="91" t="n"/>
     </row>
     <row r="24" ht="18" customFormat="1" customHeight="1" s="1">
       <c r="A24" s="9" t="n"/>
@@ -5939,6 +6234,15 @@
       <c r="K24" s="9" t="n"/>
       <c r="L24" s="9" t="n"/>
       <c r="M24" s="72" t="n"/>
+      <c r="N24" s="89" t="n"/>
+      <c r="O24" s="90" t="n"/>
+      <c r="P24" s="91" t="n"/>
+      <c r="Q24" s="89" t="n"/>
+      <c r="R24" s="90" t="n"/>
+      <c r="S24" s="91" t="n"/>
+      <c r="T24" s="89" t="n"/>
+      <c r="U24" s="90" t="n"/>
+      <c r="V24" s="91" t="n"/>
     </row>
     <row r="25" ht="18" customFormat="1" customHeight="1" s="1">
       <c r="A25" s="8" t="n"/>
@@ -5954,6 +6258,15 @@
       <c r="K25" s="8" t="n"/>
       <c r="L25" s="8" t="n"/>
       <c r="M25" s="70" t="n"/>
+      <c r="N25" s="89" t="n"/>
+      <c r="O25" s="90" t="n"/>
+      <c r="P25" s="91" t="n"/>
+      <c r="Q25" s="89" t="n"/>
+      <c r="R25" s="90" t="n"/>
+      <c r="S25" s="91" t="n"/>
+      <c r="T25" s="89" t="n"/>
+      <c r="U25" s="90" t="n"/>
+      <c r="V25" s="91" t="n"/>
     </row>
     <row r="26" ht="18" customFormat="1" customHeight="1" s="1">
       <c r="A26" s="9" t="n"/>
@@ -5969,6 +6282,15 @@
       <c r="K26" s="9" t="n"/>
       <c r="L26" s="9" t="n"/>
       <c r="M26" s="72" t="n"/>
+      <c r="N26" s="89" t="n"/>
+      <c r="O26" s="90" t="n"/>
+      <c r="P26" s="91" t="n"/>
+      <c r="Q26" s="89" t="n"/>
+      <c r="R26" s="90" t="n"/>
+      <c r="S26" s="91" t="n"/>
+      <c r="T26" s="89" t="n"/>
+      <c r="U26" s="90" t="n"/>
+      <c r="V26" s="91" t="n"/>
     </row>
     <row r="27" ht="18" customFormat="1" customHeight="1" s="1">
       <c r="A27" s="8" t="n"/>
@@ -5984,6 +6306,15 @@
       <c r="K27" s="8" t="n"/>
       <c r="L27" s="8" t="n"/>
       <c r="M27" s="70" t="n"/>
+      <c r="N27" s="89" t="n"/>
+      <c r="O27" s="90" t="n"/>
+      <c r="P27" s="91" t="n"/>
+      <c r="Q27" s="89" t="n"/>
+      <c r="R27" s="90" t="n"/>
+      <c r="S27" s="91" t="n"/>
+      <c r="T27" s="89" t="n"/>
+      <c r="U27" s="90" t="n"/>
+      <c r="V27" s="91" t="n"/>
     </row>
     <row r="28" ht="18" customFormat="1" customHeight="1" s="1">
       <c r="A28" s="9" t="n"/>
@@ -5999,6 +6330,15 @@
       <c r="K28" s="9" t="n"/>
       <c r="L28" s="9" t="n"/>
       <c r="M28" s="72" t="n"/>
+      <c r="N28" s="89" t="n"/>
+      <c r="O28" s="90" t="n"/>
+      <c r="P28" s="91" t="n"/>
+      <c r="Q28" s="89" t="n"/>
+      <c r="R28" s="90" t="n"/>
+      <c r="S28" s="91" t="n"/>
+      <c r="T28" s="89" t="n"/>
+      <c r="U28" s="90" t="n"/>
+      <c r="V28" s="91" t="n"/>
     </row>
     <row r="29" ht="18" customFormat="1" customHeight="1" s="1">
       <c r="A29" s="8" t="n"/>
@@ -6014,6 +6354,15 @@
       <c r="K29" s="8" t="n"/>
       <c r="L29" s="8" t="n"/>
       <c r="M29" s="70" t="n"/>
+      <c r="N29" s="89" t="n"/>
+      <c r="O29" s="90" t="n"/>
+      <c r="P29" s="91" t="n"/>
+      <c r="Q29" s="89" t="n"/>
+      <c r="R29" s="90" t="n"/>
+      <c r="S29" s="91" t="n"/>
+      <c r="T29" s="89" t="n"/>
+      <c r="U29" s="90" t="n"/>
+      <c r="V29" s="91" t="n"/>
     </row>
     <row r="30" ht="18" customFormat="1" customHeight="1" s="1">
       <c r="A30" s="9" t="n"/>
@@ -6029,6 +6378,15 @@
       <c r="K30" s="9" t="n"/>
       <c r="L30" s="9" t="n"/>
       <c r="M30" s="72" t="n"/>
+      <c r="N30" s="89" t="n"/>
+      <c r="O30" s="90" t="n"/>
+      <c r="P30" s="91" t="n"/>
+      <c r="Q30" s="89" t="n"/>
+      <c r="R30" s="90" t="n"/>
+      <c r="S30" s="91" t="n"/>
+      <c r="T30" s="89" t="n"/>
+      <c r="U30" s="90" t="n"/>
+      <c r="V30" s="91" t="n"/>
     </row>
     <row r="31" ht="18" customFormat="1" customHeight="1" s="1">
       <c r="A31" s="8" t="n"/>
@@ -6044,6 +6402,15 @@
       <c r="K31" s="8" t="n"/>
       <c r="L31" s="8" t="n"/>
       <c r="M31" s="70" t="n"/>
+      <c r="N31" s="89" t="n"/>
+      <c r="O31" s="90" t="n"/>
+      <c r="P31" s="91" t="n"/>
+      <c r="Q31" s="89" t="n"/>
+      <c r="R31" s="90" t="n"/>
+      <c r="S31" s="91" t="n"/>
+      <c r="T31" s="89" t="n"/>
+      <c r="U31" s="90" t="n"/>
+      <c r="V31" s="91" t="n"/>
     </row>
     <row r="32" ht="18" customFormat="1" customHeight="1" s="1">
       <c r="A32" s="9" t="n"/>
@@ -6059,6 +6426,15 @@
       <c r="K32" s="9" t="n"/>
       <c r="L32" s="9" t="n"/>
       <c r="M32" s="72" t="n"/>
+      <c r="N32" s="89" t="n"/>
+      <c r="O32" s="90" t="n"/>
+      <c r="P32" s="91" t="n"/>
+      <c r="Q32" s="89" t="n"/>
+      <c r="R32" s="90" t="n"/>
+      <c r="S32" s="91" t="n"/>
+      <c r="T32" s="89" t="n"/>
+      <c r="U32" s="90" t="n"/>
+      <c r="V32" s="91" t="n"/>
     </row>
     <row r="33" ht="18" customFormat="1" customHeight="1" s="1">
       <c r="A33" s="8" t="n"/>
@@ -6074,6 +6450,15 @@
       <c r="K33" s="8" t="n"/>
       <c r="L33" s="8" t="n"/>
       <c r="M33" s="70" t="n"/>
+      <c r="N33" s="89" t="n"/>
+      <c r="O33" s="90" t="n"/>
+      <c r="P33" s="91" t="n"/>
+      <c r="Q33" s="89" t="n"/>
+      <c r="R33" s="90" t="n"/>
+      <c r="S33" s="91" t="n"/>
+      <c r="T33" s="89" t="n"/>
+      <c r="U33" s="90" t="n"/>
+      <c r="V33" s="91" t="n"/>
     </row>
     <row r="34" ht="18" customFormat="1" customHeight="1" s="1">
       <c r="A34" s="9" t="n"/>
@@ -6089,6 +6474,15 @@
       <c r="K34" s="9" t="n"/>
       <c r="L34" s="9" t="n"/>
       <c r="M34" s="72" t="n"/>
+      <c r="N34" s="89" t="n"/>
+      <c r="O34" s="90" t="n"/>
+      <c r="P34" s="91" t="n"/>
+      <c r="Q34" s="89" t="n"/>
+      <c r="R34" s="90" t="n"/>
+      <c r="S34" s="91" t="n"/>
+      <c r="T34" s="89" t="n"/>
+      <c r="U34" s="90" t="n"/>
+      <c r="V34" s="91" t="n"/>
     </row>
     <row r="35" ht="18" customFormat="1" customHeight="1" s="1">
       <c r="A35" s="10" t="inlineStr">
@@ -6110,13 +6504,16 @@
       <c r="M35" s="54" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="6">
+  <mergeCells count="9">
     <mergeCell ref="A1:M1"/>
     <mergeCell ref="F3:I3"/>
     <mergeCell ref="J3:M3"/>
     <mergeCell ref="A35:M35"/>
+    <mergeCell ref="T3:V3"/>
     <mergeCell ref="B3:E3"/>
     <mergeCell ref="A2:M2"/>
+    <mergeCell ref="N3:P3"/>
+    <mergeCell ref="Q3:S3"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
RSI sheet — colour-code SL Left (blue) vs SL Right (green) for clear field differentiation
</commit_message>
<xml_diff>
--- a/public/AMSC_Combine_Data_Template.xlsx
+++ b/public/AMSC_Combine_Data_Template.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="480" yWindow="60" windowWidth="18195" windowHeight="8505" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Instructions" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Sprint Data" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Jump Data" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="RSI Data" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sprint Data" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Jump Data" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RSI Data" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -189,7 +189,7 @@
       <sz val="9"/>
     </font>
   </fonts>
-  <fills count="16">
+  <fills count="21">
     <fill>
       <patternFill/>
     </fill>
@@ -266,8 +266,33 @@
         <fgColor rgb="FF1A2A4A"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF1A3A5C"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF1A4A2A"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF1A0000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF000A18"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF001A04"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="32">
+  <borders count="34">
     <border>
       <left/>
       <right/>
@@ -560,11 +585,33 @@
       <top/>
       <bottom/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin">
+        <color rgb="FFcccccc"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFcccccc"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFcccccc"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin"/>
+      <right style="medium"/>
+      <top style="thin">
+        <color rgb="FFcccccc"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFcccccc"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2"/>
   </cellStyleXfs>
-  <cellXfs count="92">
+  <cellXfs count="117">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
@@ -809,6 +856,73 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="29" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="30" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="31" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="23" fillId="16" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="16" borderId="16" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="16" borderId="18" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="23" fillId="17" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="17" borderId="16" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="17" borderId="18" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="23" fillId="15" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="13" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="13" borderId="16" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="13" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="16" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="16" borderId="16" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="16" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="17" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="17" borderId="16" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="17" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="18" borderId="22" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="18" borderId="32" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="18" borderId="33" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="19" borderId="22" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="19" borderId="32" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="19" borderId="33" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="20" borderId="22" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="20" borderId="32" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="20" borderId="33" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -5606,51 +5720,51 @@
           <t>ATHLETE INFO</t>
         </is>
       </c>
-      <c r="B3" s="80" t="inlineStr">
+      <c r="B3" s="74" t="inlineStr">
         <is>
           <t>DOUBLE-LEG</t>
         </is>
       </c>
-      <c r="C3" s="81" t="n"/>
-      <c r="D3" s="81" t="n"/>
-      <c r="E3" s="82" t="n"/>
-      <c r="F3" s="80" t="inlineStr">
-        <is>
-          <t>SINGLE-LEG LEFT</t>
-        </is>
-      </c>
-      <c r="G3" s="81" t="n"/>
-      <c r="H3" s="81" t="n"/>
-      <c r="I3" s="82" t="n"/>
-      <c r="J3" s="80" t="inlineStr">
-        <is>
-          <t>SINGLE-LEG RIGHT</t>
-        </is>
-      </c>
-      <c r="K3" s="81" t="n"/>
-      <c r="L3" s="81" t="n"/>
-      <c r="M3" s="82" t="n"/>
-      <c r="N3" s="83" t="inlineStr">
+      <c r="C3" s="75" t="n"/>
+      <c r="D3" s="75" t="n"/>
+      <c r="E3" s="76" t="n"/>
+      <c r="F3" s="92" t="inlineStr">
+        <is>
+          <t>SINGLE-LEG — LEFT</t>
+        </is>
+      </c>
+      <c r="G3" s="93" t="n"/>
+      <c r="H3" s="93" t="n"/>
+      <c r="I3" s="94" t="n"/>
+      <c r="J3" s="95" t="inlineStr">
+        <is>
+          <t>SINGLE-LEG — RIGHT</t>
+        </is>
+      </c>
+      <c r="K3" s="96" t="n"/>
+      <c r="L3" s="96" t="n"/>
+      <c r="M3" s="97" t="n"/>
+      <c r="N3" s="98" t="inlineStr">
         <is>
           <t>40cm DROP JUMP</t>
         </is>
       </c>
-      <c r="O3" s="84" t="n"/>
-      <c r="P3" s="85" t="n"/>
-      <c r="Q3" s="83" t="inlineStr">
+      <c r="O3" s="81" t="n"/>
+      <c r="P3" s="82" t="n"/>
+      <c r="Q3" s="98" t="inlineStr">
         <is>
           <t>50cm DROP JUMP</t>
         </is>
       </c>
-      <c r="R3" s="84" t="n"/>
-      <c r="S3" s="85" t="n"/>
-      <c r="T3" s="83" t="inlineStr">
+      <c r="R3" s="81" t="n"/>
+      <c r="S3" s="82" t="n"/>
+      <c r="T3" s="98" t="inlineStr">
         <is>
           <t>60cm DROP JUMP</t>
         </is>
       </c>
-      <c r="U3" s="84" t="n"/>
-      <c r="V3" s="85" t="n"/>
+      <c r="U3" s="81" t="n"/>
+      <c r="V3" s="82" t="n"/>
     </row>
     <row r="4" ht="30" customFormat="1" customHeight="1" s="1">
       <c r="A4" s="77" t="inlineStr">
@@ -5658,64 +5772,64 @@
           <t>Athlete Name*</t>
         </is>
       </c>
-      <c r="B4" s="78" t="inlineStr">
-        <is>
-          <t>DL — Avg RSI</t>
-        </is>
-      </c>
-      <c r="C4" s="77" t="inlineStr">
-        <is>
-          <t>DL — Avg GCT (s)</t>
-        </is>
-      </c>
-      <c r="D4" s="77" t="inlineStr">
-        <is>
-          <t>DL — Max RSI</t>
-        </is>
-      </c>
-      <c r="E4" s="79" t="inlineStr">
-        <is>
-          <t>DL — Max GCT (s)</t>
-        </is>
-      </c>
-      <c r="F4" s="78" t="inlineStr">
-        <is>
-          <t>SL-L — Avg RSI</t>
-        </is>
-      </c>
-      <c r="G4" s="77" t="inlineStr">
-        <is>
-          <t>SL-L — Avg GCT (s)</t>
-        </is>
-      </c>
-      <c r="H4" s="77" t="inlineStr">
-        <is>
-          <t>SL-L — Max RSI</t>
-        </is>
-      </c>
-      <c r="I4" s="79" t="inlineStr">
-        <is>
-          <t>SL-L — Max GCT (s)</t>
-        </is>
-      </c>
-      <c r="J4" s="78" t="inlineStr">
-        <is>
-          <t>SL-R — Avg RSI</t>
-        </is>
-      </c>
-      <c r="K4" s="77" t="inlineStr">
-        <is>
-          <t>SL-R — Avg GCT (s)</t>
-        </is>
-      </c>
-      <c r="L4" s="77" t="inlineStr">
-        <is>
-          <t>SL-R — Max RSI</t>
-        </is>
-      </c>
-      <c r="M4" s="79" t="inlineStr">
-        <is>
-          <t>SL-R — Max GCT (s)</t>
+      <c r="B4" s="99" t="inlineStr">
+        <is>
+          <t>Avg RSI</t>
+        </is>
+      </c>
+      <c r="C4" s="100" t="inlineStr">
+        <is>
+          <t>Avg GCT (s)</t>
+        </is>
+      </c>
+      <c r="D4" s="100" t="inlineStr">
+        <is>
+          <t>Max RSI</t>
+        </is>
+      </c>
+      <c r="E4" s="101" t="inlineStr">
+        <is>
+          <t>Max GCT (s)</t>
+        </is>
+      </c>
+      <c r="F4" s="102" t="inlineStr">
+        <is>
+          <t>Avg RSI</t>
+        </is>
+      </c>
+      <c r="G4" s="103" t="inlineStr">
+        <is>
+          <t>Avg GCT (s)</t>
+        </is>
+      </c>
+      <c r="H4" s="103" t="inlineStr">
+        <is>
+          <t>Max RSI</t>
+        </is>
+      </c>
+      <c r="I4" s="104" t="inlineStr">
+        <is>
+          <t>Max GCT (s)</t>
+        </is>
+      </c>
+      <c r="J4" s="105" t="inlineStr">
+        <is>
+          <t>Avg RSI</t>
+        </is>
+      </c>
+      <c r="K4" s="106" t="inlineStr">
+        <is>
+          <t>Avg GCT (s)</t>
+        </is>
+      </c>
+      <c r="L4" s="106" t="inlineStr">
+        <is>
+          <t>Max RSI</t>
+        </is>
+      </c>
+      <c r="M4" s="107" t="inlineStr">
+        <is>
+          <t>Max GCT (s)</t>
         </is>
       </c>
       <c r="N4" s="86" t="inlineStr">
@@ -5766,18 +5880,18 @@
     </row>
     <row r="5" ht="18" customFormat="1" customHeight="1" s="1">
       <c r="A5" s="8" t="n"/>
-      <c r="B5" s="8" t="n"/>
-      <c r="C5" s="8" t="n"/>
-      <c r="D5" s="8" t="n"/>
-      <c r="E5" s="8" t="n"/>
-      <c r="F5" s="69" t="n"/>
-      <c r="G5" s="8" t="n"/>
-      <c r="H5" s="8" t="n"/>
-      <c r="I5" s="8" t="n"/>
-      <c r="J5" s="69" t="n"/>
-      <c r="K5" s="8" t="n"/>
-      <c r="L5" s="8" t="n"/>
-      <c r="M5" s="70" t="n"/>
+      <c r="B5" s="108" t="n"/>
+      <c r="C5" s="109" t="n"/>
+      <c r="D5" s="109" t="n"/>
+      <c r="E5" s="110" t="n"/>
+      <c r="F5" s="111" t="n"/>
+      <c r="G5" s="112" t="n"/>
+      <c r="H5" s="112" t="n"/>
+      <c r="I5" s="113" t="n"/>
+      <c r="J5" s="114" t="n"/>
+      <c r="K5" s="115" t="n"/>
+      <c r="L5" s="115" t="n"/>
+      <c r="M5" s="116" t="n"/>
       <c r="N5" s="89" t="n"/>
       <c r="O5" s="90" t="n"/>
       <c r="P5" s="91" t="n"/>
@@ -5790,18 +5904,18 @@
     </row>
     <row r="6" ht="18" customFormat="1" customHeight="1" s="1">
       <c r="A6" s="9" t="n"/>
-      <c r="B6" s="9" t="n"/>
-      <c r="C6" s="9" t="n"/>
-      <c r="D6" s="9" t="n"/>
-      <c r="E6" s="9" t="n"/>
-      <c r="F6" s="71" t="n"/>
-      <c r="G6" s="9" t="n"/>
-      <c r="H6" s="9" t="n"/>
-      <c r="I6" s="9" t="n"/>
-      <c r="J6" s="71" t="n"/>
-      <c r="K6" s="9" t="n"/>
-      <c r="L6" s="9" t="n"/>
-      <c r="M6" s="72" t="n"/>
+      <c r="B6" s="108" t="n"/>
+      <c r="C6" s="109" t="n"/>
+      <c r="D6" s="109" t="n"/>
+      <c r="E6" s="110" t="n"/>
+      <c r="F6" s="111" t="n"/>
+      <c r="G6" s="112" t="n"/>
+      <c r="H6" s="112" t="n"/>
+      <c r="I6" s="113" t="n"/>
+      <c r="J6" s="114" t="n"/>
+      <c r="K6" s="115" t="n"/>
+      <c r="L6" s="115" t="n"/>
+      <c r="M6" s="116" t="n"/>
       <c r="N6" s="89" t="n"/>
       <c r="O6" s="90" t="n"/>
       <c r="P6" s="91" t="n"/>
@@ -5814,18 +5928,18 @@
     </row>
     <row r="7" ht="18" customFormat="1" customHeight="1" s="1">
       <c r="A7" s="8" t="n"/>
-      <c r="B7" s="8" t="n"/>
-      <c r="C7" s="8" t="n"/>
-      <c r="D7" s="8" t="n"/>
-      <c r="E7" s="8" t="n"/>
-      <c r="F7" s="69" t="n"/>
-      <c r="G7" s="8" t="n"/>
-      <c r="H7" s="8" t="n"/>
-      <c r="I7" s="8" t="n"/>
-      <c r="J7" s="69" t="n"/>
-      <c r="K7" s="8" t="n"/>
-      <c r="L7" s="8" t="n"/>
-      <c r="M7" s="70" t="n"/>
+      <c r="B7" s="108" t="n"/>
+      <c r="C7" s="109" t="n"/>
+      <c r="D7" s="109" t="n"/>
+      <c r="E7" s="110" t="n"/>
+      <c r="F7" s="111" t="n"/>
+      <c r="G7" s="112" t="n"/>
+      <c r="H7" s="112" t="n"/>
+      <c r="I7" s="113" t="n"/>
+      <c r="J7" s="114" t="n"/>
+      <c r="K7" s="115" t="n"/>
+      <c r="L7" s="115" t="n"/>
+      <c r="M7" s="116" t="n"/>
       <c r="N7" s="89" t="n"/>
       <c r="O7" s="90" t="n"/>
       <c r="P7" s="91" t="n"/>
@@ -5838,18 +5952,18 @@
     </row>
     <row r="8" ht="18" customFormat="1" customHeight="1" s="1">
       <c r="A8" s="9" t="n"/>
-      <c r="B8" s="9" t="n"/>
-      <c r="C8" s="9" t="n"/>
-      <c r="D8" s="9" t="n"/>
-      <c r="E8" s="9" t="n"/>
-      <c r="F8" s="71" t="n"/>
-      <c r="G8" s="9" t="n"/>
-      <c r="H8" s="9" t="n"/>
-      <c r="I8" s="9" t="n"/>
-      <c r="J8" s="71" t="n"/>
-      <c r="K8" s="9" t="n"/>
-      <c r="L8" s="9" t="n"/>
-      <c r="M8" s="72" t="n"/>
+      <c r="B8" s="108" t="n"/>
+      <c r="C8" s="109" t="n"/>
+      <c r="D8" s="109" t="n"/>
+      <c r="E8" s="110" t="n"/>
+      <c r="F8" s="111" t="n"/>
+      <c r="G8" s="112" t="n"/>
+      <c r="H8" s="112" t="n"/>
+      <c r="I8" s="113" t="n"/>
+      <c r="J8" s="114" t="n"/>
+      <c r="K8" s="115" t="n"/>
+      <c r="L8" s="115" t="n"/>
+      <c r="M8" s="116" t="n"/>
       <c r="N8" s="89" t="n"/>
       <c r="O8" s="90" t="n"/>
       <c r="P8" s="91" t="n"/>
@@ -5862,18 +5976,18 @@
     </row>
     <row r="9" ht="18" customFormat="1" customHeight="1" s="1">
       <c r="A9" s="8" t="n"/>
-      <c r="B9" s="8" t="n"/>
-      <c r="C9" s="8" t="n"/>
-      <c r="D9" s="8" t="n"/>
-      <c r="E9" s="8" t="n"/>
-      <c r="F9" s="69" t="n"/>
-      <c r="G9" s="8" t="n"/>
-      <c r="H9" s="8" t="n"/>
-      <c r="I9" s="8" t="n"/>
-      <c r="J9" s="69" t="n"/>
-      <c r="K9" s="8" t="n"/>
-      <c r="L9" s="8" t="n"/>
-      <c r="M9" s="70" t="n"/>
+      <c r="B9" s="108" t="n"/>
+      <c r="C9" s="109" t="n"/>
+      <c r="D9" s="109" t="n"/>
+      <c r="E9" s="110" t="n"/>
+      <c r="F9" s="111" t="n"/>
+      <c r="G9" s="112" t="n"/>
+      <c r="H9" s="112" t="n"/>
+      <c r="I9" s="113" t="n"/>
+      <c r="J9" s="114" t="n"/>
+      <c r="K9" s="115" t="n"/>
+      <c r="L9" s="115" t="n"/>
+      <c r="M9" s="116" t="n"/>
       <c r="N9" s="89" t="n"/>
       <c r="O9" s="90" t="n"/>
       <c r="P9" s="91" t="n"/>
@@ -5886,18 +6000,18 @@
     </row>
     <row r="10" ht="18" customFormat="1" customHeight="1" s="1">
       <c r="A10" s="9" t="n"/>
-      <c r="B10" s="9" t="n"/>
-      <c r="C10" s="9" t="n"/>
-      <c r="D10" s="9" t="n"/>
-      <c r="E10" s="9" t="n"/>
-      <c r="F10" s="71" t="n"/>
-      <c r="G10" s="9" t="n"/>
-      <c r="H10" s="9" t="n"/>
-      <c r="I10" s="9" t="n"/>
-      <c r="J10" s="71" t="n"/>
-      <c r="K10" s="9" t="n"/>
-      <c r="L10" s="9" t="n"/>
-      <c r="M10" s="72" t="n"/>
+      <c r="B10" s="108" t="n"/>
+      <c r="C10" s="109" t="n"/>
+      <c r="D10" s="109" t="n"/>
+      <c r="E10" s="110" t="n"/>
+      <c r="F10" s="111" t="n"/>
+      <c r="G10" s="112" t="n"/>
+      <c r="H10" s="112" t="n"/>
+      <c r="I10" s="113" t="n"/>
+      <c r="J10" s="114" t="n"/>
+      <c r="K10" s="115" t="n"/>
+      <c r="L10" s="115" t="n"/>
+      <c r="M10" s="116" t="n"/>
       <c r="N10" s="89" t="n"/>
       <c r="O10" s="90" t="n"/>
       <c r="P10" s="91" t="n"/>
@@ -5910,18 +6024,18 @@
     </row>
     <row r="11" ht="18" customFormat="1" customHeight="1" s="1">
       <c r="A11" s="8" t="n"/>
-      <c r="B11" s="8" t="n"/>
-      <c r="C11" s="8" t="n"/>
-      <c r="D11" s="8" t="n"/>
-      <c r="E11" s="8" t="n"/>
-      <c r="F11" s="69" t="n"/>
-      <c r="G11" s="8" t="n"/>
-      <c r="H11" s="8" t="n"/>
-      <c r="I11" s="8" t="n"/>
-      <c r="J11" s="69" t="n"/>
-      <c r="K11" s="8" t="n"/>
-      <c r="L11" s="8" t="n"/>
-      <c r="M11" s="70" t="n"/>
+      <c r="B11" s="108" t="n"/>
+      <c r="C11" s="109" t="n"/>
+      <c r="D11" s="109" t="n"/>
+      <c r="E11" s="110" t="n"/>
+      <c r="F11" s="111" t="n"/>
+      <c r="G11" s="112" t="n"/>
+      <c r="H11" s="112" t="n"/>
+      <c r="I11" s="113" t="n"/>
+      <c r="J11" s="114" t="n"/>
+      <c r="K11" s="115" t="n"/>
+      <c r="L11" s="115" t="n"/>
+      <c r="M11" s="116" t="n"/>
       <c r="N11" s="89" t="n"/>
       <c r="O11" s="90" t="n"/>
       <c r="P11" s="91" t="n"/>
@@ -5934,18 +6048,18 @@
     </row>
     <row r="12" ht="18" customFormat="1" customHeight="1" s="1">
       <c r="A12" s="9" t="n"/>
-      <c r="B12" s="9" t="n"/>
-      <c r="C12" s="9" t="n"/>
-      <c r="D12" s="9" t="n"/>
-      <c r="E12" s="9" t="n"/>
-      <c r="F12" s="71" t="n"/>
-      <c r="G12" s="9" t="n"/>
-      <c r="H12" s="9" t="n"/>
-      <c r="I12" s="9" t="n"/>
-      <c r="J12" s="71" t="n"/>
-      <c r="K12" s="9" t="n"/>
-      <c r="L12" s="9" t="n"/>
-      <c r="M12" s="72" t="n"/>
+      <c r="B12" s="108" t="n"/>
+      <c r="C12" s="109" t="n"/>
+      <c r="D12" s="109" t="n"/>
+      <c r="E12" s="110" t="n"/>
+      <c r="F12" s="111" t="n"/>
+      <c r="G12" s="112" t="n"/>
+      <c r="H12" s="112" t="n"/>
+      <c r="I12" s="113" t="n"/>
+      <c r="J12" s="114" t="n"/>
+      <c r="K12" s="115" t="n"/>
+      <c r="L12" s="115" t="n"/>
+      <c r="M12" s="116" t="n"/>
       <c r="N12" s="89" t="n"/>
       <c r="O12" s="90" t="n"/>
       <c r="P12" s="91" t="n"/>
@@ -5958,18 +6072,18 @@
     </row>
     <row r="13" ht="18" customFormat="1" customHeight="1" s="1">
       <c r="A13" s="8" t="n"/>
-      <c r="B13" s="8" t="n"/>
-      <c r="C13" s="8" t="n"/>
-      <c r="D13" s="8" t="n"/>
-      <c r="E13" s="8" t="n"/>
-      <c r="F13" s="69" t="n"/>
-      <c r="G13" s="8" t="n"/>
-      <c r="H13" s="8" t="n"/>
-      <c r="I13" s="8" t="n"/>
-      <c r="J13" s="69" t="n"/>
-      <c r="K13" s="8" t="n"/>
-      <c r="L13" s="8" t="n"/>
-      <c r="M13" s="70" t="n"/>
+      <c r="B13" s="108" t="n"/>
+      <c r="C13" s="109" t="n"/>
+      <c r="D13" s="109" t="n"/>
+      <c r="E13" s="110" t="n"/>
+      <c r="F13" s="111" t="n"/>
+      <c r="G13" s="112" t="n"/>
+      <c r="H13" s="112" t="n"/>
+      <c r="I13" s="113" t="n"/>
+      <c r="J13" s="114" t="n"/>
+      <c r="K13" s="115" t="n"/>
+      <c r="L13" s="115" t="n"/>
+      <c r="M13" s="116" t="n"/>
       <c r="N13" s="89" t="n"/>
       <c r="O13" s="90" t="n"/>
       <c r="P13" s="91" t="n"/>
@@ -5982,18 +6096,18 @@
     </row>
     <row r="14" ht="18" customFormat="1" customHeight="1" s="1">
       <c r="A14" s="9" t="n"/>
-      <c r="B14" s="9" t="n"/>
-      <c r="C14" s="9" t="n"/>
-      <c r="D14" s="9" t="n"/>
-      <c r="E14" s="9" t="n"/>
-      <c r="F14" s="71" t="n"/>
-      <c r="G14" s="9" t="n"/>
-      <c r="H14" s="9" t="n"/>
-      <c r="I14" s="9" t="n"/>
-      <c r="J14" s="71" t="n"/>
-      <c r="K14" s="9" t="n"/>
-      <c r="L14" s="9" t="n"/>
-      <c r="M14" s="72" t="n"/>
+      <c r="B14" s="108" t="n"/>
+      <c r="C14" s="109" t="n"/>
+      <c r="D14" s="109" t="n"/>
+      <c r="E14" s="110" t="n"/>
+      <c r="F14" s="111" t="n"/>
+      <c r="G14" s="112" t="n"/>
+      <c r="H14" s="112" t="n"/>
+      <c r="I14" s="113" t="n"/>
+      <c r="J14" s="114" t="n"/>
+      <c r="K14" s="115" t="n"/>
+      <c r="L14" s="115" t="n"/>
+      <c r="M14" s="116" t="n"/>
       <c r="N14" s="89" t="n"/>
       <c r="O14" s="90" t="n"/>
       <c r="P14" s="91" t="n"/>
@@ -6006,18 +6120,18 @@
     </row>
     <row r="15" ht="18" customFormat="1" customHeight="1" s="1">
       <c r="A15" s="8" t="n"/>
-      <c r="B15" s="8" t="n"/>
-      <c r="C15" s="8" t="n"/>
-      <c r="D15" s="8" t="n"/>
-      <c r="E15" s="8" t="n"/>
-      <c r="F15" s="69" t="n"/>
-      <c r="G15" s="8" t="n"/>
-      <c r="H15" s="8" t="n"/>
-      <c r="I15" s="8" t="n"/>
-      <c r="J15" s="69" t="n"/>
-      <c r="K15" s="8" t="n"/>
-      <c r="L15" s="8" t="n"/>
-      <c r="M15" s="70" t="n"/>
+      <c r="B15" s="108" t="n"/>
+      <c r="C15" s="109" t="n"/>
+      <c r="D15" s="109" t="n"/>
+      <c r="E15" s="110" t="n"/>
+      <c r="F15" s="111" t="n"/>
+      <c r="G15" s="112" t="n"/>
+      <c r="H15" s="112" t="n"/>
+      <c r="I15" s="113" t="n"/>
+      <c r="J15" s="114" t="n"/>
+      <c r="K15" s="115" t="n"/>
+      <c r="L15" s="115" t="n"/>
+      <c r="M15" s="116" t="n"/>
       <c r="N15" s="89" t="n"/>
       <c r="O15" s="90" t="n"/>
       <c r="P15" s="91" t="n"/>
@@ -6030,18 +6144,18 @@
     </row>
     <row r="16" ht="18" customFormat="1" customHeight="1" s="1">
       <c r="A16" s="9" t="n"/>
-      <c r="B16" s="9" t="n"/>
-      <c r="C16" s="9" t="n"/>
-      <c r="D16" s="9" t="n"/>
-      <c r="E16" s="9" t="n"/>
-      <c r="F16" s="71" t="n"/>
-      <c r="G16" s="9" t="n"/>
-      <c r="H16" s="9" t="n"/>
-      <c r="I16" s="9" t="n"/>
-      <c r="J16" s="71" t="n"/>
-      <c r="K16" s="9" t="n"/>
-      <c r="L16" s="9" t="n"/>
-      <c r="M16" s="72" t="n"/>
+      <c r="B16" s="108" t="n"/>
+      <c r="C16" s="109" t="n"/>
+      <c r="D16" s="109" t="n"/>
+      <c r="E16" s="110" t="n"/>
+      <c r="F16" s="111" t="n"/>
+      <c r="G16" s="112" t="n"/>
+      <c r="H16" s="112" t="n"/>
+      <c r="I16" s="113" t="n"/>
+      <c r="J16" s="114" t="n"/>
+      <c r="K16" s="115" t="n"/>
+      <c r="L16" s="115" t="n"/>
+      <c r="M16" s="116" t="n"/>
       <c r="N16" s="89" t="n"/>
       <c r="O16" s="90" t="n"/>
       <c r="P16" s="91" t="n"/>
@@ -6054,18 +6168,18 @@
     </row>
     <row r="17" ht="18" customFormat="1" customHeight="1" s="1">
       <c r="A17" s="8" t="n"/>
-      <c r="B17" s="8" t="n"/>
-      <c r="C17" s="8" t="n"/>
-      <c r="D17" s="8" t="n"/>
-      <c r="E17" s="8" t="n"/>
-      <c r="F17" s="69" t="n"/>
-      <c r="G17" s="8" t="n"/>
-      <c r="H17" s="8" t="n"/>
-      <c r="I17" s="8" t="n"/>
-      <c r="J17" s="69" t="n"/>
-      <c r="K17" s="8" t="n"/>
-      <c r="L17" s="8" t="n"/>
-      <c r="M17" s="70" t="n"/>
+      <c r="B17" s="108" t="n"/>
+      <c r="C17" s="109" t="n"/>
+      <c r="D17" s="109" t="n"/>
+      <c r="E17" s="110" t="n"/>
+      <c r="F17" s="111" t="n"/>
+      <c r="G17" s="112" t="n"/>
+      <c r="H17" s="112" t="n"/>
+      <c r="I17" s="113" t="n"/>
+      <c r="J17" s="114" t="n"/>
+      <c r="K17" s="115" t="n"/>
+      <c r="L17" s="115" t="n"/>
+      <c r="M17" s="116" t="n"/>
       <c r="N17" s="89" t="n"/>
       <c r="O17" s="90" t="n"/>
       <c r="P17" s="91" t="n"/>
@@ -6078,18 +6192,18 @@
     </row>
     <row r="18" ht="18" customFormat="1" customHeight="1" s="1">
       <c r="A18" s="9" t="n"/>
-      <c r="B18" s="9" t="n"/>
-      <c r="C18" s="9" t="n"/>
-      <c r="D18" s="9" t="n"/>
-      <c r="E18" s="9" t="n"/>
-      <c r="F18" s="71" t="n"/>
-      <c r="G18" s="9" t="n"/>
-      <c r="H18" s="9" t="n"/>
-      <c r="I18" s="9" t="n"/>
-      <c r="J18" s="71" t="n"/>
-      <c r="K18" s="9" t="n"/>
-      <c r="L18" s="9" t="n"/>
-      <c r="M18" s="72" t="n"/>
+      <c r="B18" s="108" t="n"/>
+      <c r="C18" s="109" t="n"/>
+      <c r="D18" s="109" t="n"/>
+      <c r="E18" s="110" t="n"/>
+      <c r="F18" s="111" t="n"/>
+      <c r="G18" s="112" t="n"/>
+      <c r="H18" s="112" t="n"/>
+      <c r="I18" s="113" t="n"/>
+      <c r="J18" s="114" t="n"/>
+      <c r="K18" s="115" t="n"/>
+      <c r="L18" s="115" t="n"/>
+      <c r="M18" s="116" t="n"/>
       <c r="N18" s="89" t="n"/>
       <c r="O18" s="90" t="n"/>
       <c r="P18" s="91" t="n"/>
@@ -6102,18 +6216,18 @@
     </row>
     <row r="19" ht="18" customFormat="1" customHeight="1" s="1">
       <c r="A19" s="8" t="n"/>
-      <c r="B19" s="8" t="n"/>
-      <c r="C19" s="8" t="n"/>
-      <c r="D19" s="8" t="n"/>
-      <c r="E19" s="8" t="n"/>
-      <c r="F19" s="69" t="n"/>
-      <c r="G19" s="8" t="n"/>
-      <c r="H19" s="8" t="n"/>
-      <c r="I19" s="8" t="n"/>
-      <c r="J19" s="69" t="n"/>
-      <c r="K19" s="8" t="n"/>
-      <c r="L19" s="8" t="n"/>
-      <c r="M19" s="70" t="n"/>
+      <c r="B19" s="108" t="n"/>
+      <c r="C19" s="109" t="n"/>
+      <c r="D19" s="109" t="n"/>
+      <c r="E19" s="110" t="n"/>
+      <c r="F19" s="111" t="n"/>
+      <c r="G19" s="112" t="n"/>
+      <c r="H19" s="112" t="n"/>
+      <c r="I19" s="113" t="n"/>
+      <c r="J19" s="114" t="n"/>
+      <c r="K19" s="115" t="n"/>
+      <c r="L19" s="115" t="n"/>
+      <c r="M19" s="116" t="n"/>
       <c r="N19" s="89" t="n"/>
       <c r="O19" s="90" t="n"/>
       <c r="P19" s="91" t="n"/>
@@ -6126,18 +6240,18 @@
     </row>
     <row r="20" ht="18" customFormat="1" customHeight="1" s="1">
       <c r="A20" s="9" t="n"/>
-      <c r="B20" s="9" t="n"/>
-      <c r="C20" s="9" t="n"/>
-      <c r="D20" s="9" t="n"/>
-      <c r="E20" s="9" t="n"/>
-      <c r="F20" s="71" t="n"/>
-      <c r="G20" s="9" t="n"/>
-      <c r="H20" s="9" t="n"/>
-      <c r="I20" s="9" t="n"/>
-      <c r="J20" s="71" t="n"/>
-      <c r="K20" s="9" t="n"/>
-      <c r="L20" s="9" t="n"/>
-      <c r="M20" s="72" t="n"/>
+      <c r="B20" s="108" t="n"/>
+      <c r="C20" s="109" t="n"/>
+      <c r="D20" s="109" t="n"/>
+      <c r="E20" s="110" t="n"/>
+      <c r="F20" s="111" t="n"/>
+      <c r="G20" s="112" t="n"/>
+      <c r="H20" s="112" t="n"/>
+      <c r="I20" s="113" t="n"/>
+      <c r="J20" s="114" t="n"/>
+      <c r="K20" s="115" t="n"/>
+      <c r="L20" s="115" t="n"/>
+      <c r="M20" s="116" t="n"/>
       <c r="N20" s="89" t="n"/>
       <c r="O20" s="90" t="n"/>
       <c r="P20" s="91" t="n"/>
@@ -6150,18 +6264,18 @@
     </row>
     <row r="21" ht="18" customFormat="1" customHeight="1" s="1">
       <c r="A21" s="8" t="n"/>
-      <c r="B21" s="8" t="n"/>
-      <c r="C21" s="8" t="n"/>
-      <c r="D21" s="8" t="n"/>
-      <c r="E21" s="8" t="n"/>
-      <c r="F21" s="69" t="n"/>
-      <c r="G21" s="8" t="n"/>
-      <c r="H21" s="8" t="n"/>
-      <c r="I21" s="8" t="n"/>
-      <c r="J21" s="69" t="n"/>
-      <c r="K21" s="8" t="n"/>
-      <c r="L21" s="8" t="n"/>
-      <c r="M21" s="70" t="n"/>
+      <c r="B21" s="108" t="n"/>
+      <c r="C21" s="109" t="n"/>
+      <c r="D21" s="109" t="n"/>
+      <c r="E21" s="110" t="n"/>
+      <c r="F21" s="111" t="n"/>
+      <c r="G21" s="112" t="n"/>
+      <c r="H21" s="112" t="n"/>
+      <c r="I21" s="113" t="n"/>
+      <c r="J21" s="114" t="n"/>
+      <c r="K21" s="115" t="n"/>
+      <c r="L21" s="115" t="n"/>
+      <c r="M21" s="116" t="n"/>
       <c r="N21" s="89" t="n"/>
       <c r="O21" s="90" t="n"/>
       <c r="P21" s="91" t="n"/>
@@ -6174,18 +6288,18 @@
     </row>
     <row r="22" ht="18" customFormat="1" customHeight="1" s="1">
       <c r="A22" s="9" t="n"/>
-      <c r="B22" s="9" t="n"/>
-      <c r="C22" s="9" t="n"/>
-      <c r="D22" s="9" t="n"/>
-      <c r="E22" s="9" t="n"/>
-      <c r="F22" s="71" t="n"/>
-      <c r="G22" s="9" t="n"/>
-      <c r="H22" s="9" t="n"/>
-      <c r="I22" s="9" t="n"/>
-      <c r="J22" s="71" t="n"/>
-      <c r="K22" s="9" t="n"/>
-      <c r="L22" s="9" t="n"/>
-      <c r="M22" s="72" t="n"/>
+      <c r="B22" s="108" t="n"/>
+      <c r="C22" s="109" t="n"/>
+      <c r="D22" s="109" t="n"/>
+      <c r="E22" s="110" t="n"/>
+      <c r="F22" s="111" t="n"/>
+      <c r="G22" s="112" t="n"/>
+      <c r="H22" s="112" t="n"/>
+      <c r="I22" s="113" t="n"/>
+      <c r="J22" s="114" t="n"/>
+      <c r="K22" s="115" t="n"/>
+      <c r="L22" s="115" t="n"/>
+      <c r="M22" s="116" t="n"/>
       <c r="N22" s="89" t="n"/>
       <c r="O22" s="90" t="n"/>
       <c r="P22" s="91" t="n"/>
@@ -6198,18 +6312,18 @@
     </row>
     <row r="23" ht="18" customFormat="1" customHeight="1" s="1">
       <c r="A23" s="8" t="n"/>
-      <c r="B23" s="8" t="n"/>
-      <c r="C23" s="8" t="n"/>
-      <c r="D23" s="8" t="n"/>
-      <c r="E23" s="8" t="n"/>
-      <c r="F23" s="69" t="n"/>
-      <c r="G23" s="8" t="n"/>
-      <c r="H23" s="8" t="n"/>
-      <c r="I23" s="8" t="n"/>
-      <c r="J23" s="69" t="n"/>
-      <c r="K23" s="8" t="n"/>
-      <c r="L23" s="8" t="n"/>
-      <c r="M23" s="70" t="n"/>
+      <c r="B23" s="108" t="n"/>
+      <c r="C23" s="109" t="n"/>
+      <c r="D23" s="109" t="n"/>
+      <c r="E23" s="110" t="n"/>
+      <c r="F23" s="111" t="n"/>
+      <c r="G23" s="112" t="n"/>
+      <c r="H23" s="112" t="n"/>
+      <c r="I23" s="113" t="n"/>
+      <c r="J23" s="114" t="n"/>
+      <c r="K23" s="115" t="n"/>
+      <c r="L23" s="115" t="n"/>
+      <c r="M23" s="116" t="n"/>
       <c r="N23" s="89" t="n"/>
       <c r="O23" s="90" t="n"/>
       <c r="P23" s="91" t="n"/>
@@ -6222,18 +6336,18 @@
     </row>
     <row r="24" ht="18" customFormat="1" customHeight="1" s="1">
       <c r="A24" s="9" t="n"/>
-      <c r="B24" s="9" t="n"/>
-      <c r="C24" s="9" t="n"/>
-      <c r="D24" s="9" t="n"/>
-      <c r="E24" s="9" t="n"/>
-      <c r="F24" s="71" t="n"/>
-      <c r="G24" s="9" t="n"/>
-      <c r="H24" s="9" t="n"/>
-      <c r="I24" s="9" t="n"/>
-      <c r="J24" s="71" t="n"/>
-      <c r="K24" s="9" t="n"/>
-      <c r="L24" s="9" t="n"/>
-      <c r="M24" s="72" t="n"/>
+      <c r="B24" s="108" t="n"/>
+      <c r="C24" s="109" t="n"/>
+      <c r="D24" s="109" t="n"/>
+      <c r="E24" s="110" t="n"/>
+      <c r="F24" s="111" t="n"/>
+      <c r="G24" s="112" t="n"/>
+      <c r="H24" s="112" t="n"/>
+      <c r="I24" s="113" t="n"/>
+      <c r="J24" s="114" t="n"/>
+      <c r="K24" s="115" t="n"/>
+      <c r="L24" s="115" t="n"/>
+      <c r="M24" s="116" t="n"/>
       <c r="N24" s="89" t="n"/>
       <c r="O24" s="90" t="n"/>
       <c r="P24" s="91" t="n"/>
@@ -6246,18 +6360,18 @@
     </row>
     <row r="25" ht="18" customFormat="1" customHeight="1" s="1">
       <c r="A25" s="8" t="n"/>
-      <c r="B25" s="8" t="n"/>
-      <c r="C25" s="8" t="n"/>
-      <c r="D25" s="8" t="n"/>
-      <c r="E25" s="8" t="n"/>
-      <c r="F25" s="69" t="n"/>
-      <c r="G25" s="8" t="n"/>
-      <c r="H25" s="8" t="n"/>
-      <c r="I25" s="8" t="n"/>
-      <c r="J25" s="69" t="n"/>
-      <c r="K25" s="8" t="n"/>
-      <c r="L25" s="8" t="n"/>
-      <c r="M25" s="70" t="n"/>
+      <c r="B25" s="108" t="n"/>
+      <c r="C25" s="109" t="n"/>
+      <c r="D25" s="109" t="n"/>
+      <c r="E25" s="110" t="n"/>
+      <c r="F25" s="111" t="n"/>
+      <c r="G25" s="112" t="n"/>
+      <c r="H25" s="112" t="n"/>
+      <c r="I25" s="113" t="n"/>
+      <c r="J25" s="114" t="n"/>
+      <c r="K25" s="115" t="n"/>
+      <c r="L25" s="115" t="n"/>
+      <c r="M25" s="116" t="n"/>
       <c r="N25" s="89" t="n"/>
       <c r="O25" s="90" t="n"/>
       <c r="P25" s="91" t="n"/>
@@ -6270,18 +6384,18 @@
     </row>
     <row r="26" ht="18" customFormat="1" customHeight="1" s="1">
       <c r="A26" s="9" t="n"/>
-      <c r="B26" s="9" t="n"/>
-      <c r="C26" s="9" t="n"/>
-      <c r="D26" s="9" t="n"/>
-      <c r="E26" s="9" t="n"/>
-      <c r="F26" s="71" t="n"/>
-      <c r="G26" s="9" t="n"/>
-      <c r="H26" s="9" t="n"/>
-      <c r="I26" s="9" t="n"/>
-      <c r="J26" s="71" t="n"/>
-      <c r="K26" s="9" t="n"/>
-      <c r="L26" s="9" t="n"/>
-      <c r="M26" s="72" t="n"/>
+      <c r="B26" s="108" t="n"/>
+      <c r="C26" s="109" t="n"/>
+      <c r="D26" s="109" t="n"/>
+      <c r="E26" s="110" t="n"/>
+      <c r="F26" s="111" t="n"/>
+      <c r="G26" s="112" t="n"/>
+      <c r="H26" s="112" t="n"/>
+      <c r="I26" s="113" t="n"/>
+      <c r="J26" s="114" t="n"/>
+      <c r="K26" s="115" t="n"/>
+      <c r="L26" s="115" t="n"/>
+      <c r="M26" s="116" t="n"/>
       <c r="N26" s="89" t="n"/>
       <c r="O26" s="90" t="n"/>
       <c r="P26" s="91" t="n"/>
@@ -6294,18 +6408,18 @@
     </row>
     <row r="27" ht="18" customFormat="1" customHeight="1" s="1">
       <c r="A27" s="8" t="n"/>
-      <c r="B27" s="8" t="n"/>
-      <c r="C27" s="8" t="n"/>
-      <c r="D27" s="8" t="n"/>
-      <c r="E27" s="8" t="n"/>
-      <c r="F27" s="69" t="n"/>
-      <c r="G27" s="8" t="n"/>
-      <c r="H27" s="8" t="n"/>
-      <c r="I27" s="8" t="n"/>
-      <c r="J27" s="69" t="n"/>
-      <c r="K27" s="8" t="n"/>
-      <c r="L27" s="8" t="n"/>
-      <c r="M27" s="70" t="n"/>
+      <c r="B27" s="108" t="n"/>
+      <c r="C27" s="109" t="n"/>
+      <c r="D27" s="109" t="n"/>
+      <c r="E27" s="110" t="n"/>
+      <c r="F27" s="111" t="n"/>
+      <c r="G27" s="112" t="n"/>
+      <c r="H27" s="112" t="n"/>
+      <c r="I27" s="113" t="n"/>
+      <c r="J27" s="114" t="n"/>
+      <c r="K27" s="115" t="n"/>
+      <c r="L27" s="115" t="n"/>
+      <c r="M27" s="116" t="n"/>
       <c r="N27" s="89" t="n"/>
       <c r="O27" s="90" t="n"/>
       <c r="P27" s="91" t="n"/>
@@ -6318,18 +6432,18 @@
     </row>
     <row r="28" ht="18" customFormat="1" customHeight="1" s="1">
       <c r="A28" s="9" t="n"/>
-      <c r="B28" s="9" t="n"/>
-      <c r="C28" s="9" t="n"/>
-      <c r="D28" s="9" t="n"/>
-      <c r="E28" s="9" t="n"/>
-      <c r="F28" s="71" t="n"/>
-      <c r="G28" s="9" t="n"/>
-      <c r="H28" s="9" t="n"/>
-      <c r="I28" s="9" t="n"/>
-      <c r="J28" s="71" t="n"/>
-      <c r="K28" s="9" t="n"/>
-      <c r="L28" s="9" t="n"/>
-      <c r="M28" s="72" t="n"/>
+      <c r="B28" s="108" t="n"/>
+      <c r="C28" s="109" t="n"/>
+      <c r="D28" s="109" t="n"/>
+      <c r="E28" s="110" t="n"/>
+      <c r="F28" s="111" t="n"/>
+      <c r="G28" s="112" t="n"/>
+      <c r="H28" s="112" t="n"/>
+      <c r="I28" s="113" t="n"/>
+      <c r="J28" s="114" t="n"/>
+      <c r="K28" s="115" t="n"/>
+      <c r="L28" s="115" t="n"/>
+      <c r="M28" s="116" t="n"/>
       <c r="N28" s="89" t="n"/>
       <c r="O28" s="90" t="n"/>
       <c r="P28" s="91" t="n"/>
@@ -6342,18 +6456,18 @@
     </row>
     <row r="29" ht="18" customFormat="1" customHeight="1" s="1">
       <c r="A29" s="8" t="n"/>
-      <c r="B29" s="8" t="n"/>
-      <c r="C29" s="8" t="n"/>
-      <c r="D29" s="8" t="n"/>
-      <c r="E29" s="8" t="n"/>
-      <c r="F29" s="69" t="n"/>
-      <c r="G29" s="8" t="n"/>
-      <c r="H29" s="8" t="n"/>
-      <c r="I29" s="8" t="n"/>
-      <c r="J29" s="69" t="n"/>
-      <c r="K29" s="8" t="n"/>
-      <c r="L29" s="8" t="n"/>
-      <c r="M29" s="70" t="n"/>
+      <c r="B29" s="108" t="n"/>
+      <c r="C29" s="109" t="n"/>
+      <c r="D29" s="109" t="n"/>
+      <c r="E29" s="110" t="n"/>
+      <c r="F29" s="111" t="n"/>
+      <c r="G29" s="112" t="n"/>
+      <c r="H29" s="112" t="n"/>
+      <c r="I29" s="113" t="n"/>
+      <c r="J29" s="114" t="n"/>
+      <c r="K29" s="115" t="n"/>
+      <c r="L29" s="115" t="n"/>
+      <c r="M29" s="116" t="n"/>
       <c r="N29" s="89" t="n"/>
       <c r="O29" s="90" t="n"/>
       <c r="P29" s="91" t="n"/>
@@ -6366,18 +6480,18 @@
     </row>
     <row r="30" ht="18" customFormat="1" customHeight="1" s="1">
       <c r="A30" s="9" t="n"/>
-      <c r="B30" s="9" t="n"/>
-      <c r="C30" s="9" t="n"/>
-      <c r="D30" s="9" t="n"/>
-      <c r="E30" s="9" t="n"/>
-      <c r="F30" s="71" t="n"/>
-      <c r="G30" s="9" t="n"/>
-      <c r="H30" s="9" t="n"/>
-      <c r="I30" s="9" t="n"/>
-      <c r="J30" s="71" t="n"/>
-      <c r="K30" s="9" t="n"/>
-      <c r="L30" s="9" t="n"/>
-      <c r="M30" s="72" t="n"/>
+      <c r="B30" s="108" t="n"/>
+      <c r="C30" s="109" t="n"/>
+      <c r="D30" s="109" t="n"/>
+      <c r="E30" s="110" t="n"/>
+      <c r="F30" s="111" t="n"/>
+      <c r="G30" s="112" t="n"/>
+      <c r="H30" s="112" t="n"/>
+      <c r="I30" s="113" t="n"/>
+      <c r="J30" s="114" t="n"/>
+      <c r="K30" s="115" t="n"/>
+      <c r="L30" s="115" t="n"/>
+      <c r="M30" s="116" t="n"/>
       <c r="N30" s="89" t="n"/>
       <c r="O30" s="90" t="n"/>
       <c r="P30" s="91" t="n"/>
@@ -6390,18 +6504,18 @@
     </row>
     <row r="31" ht="18" customFormat="1" customHeight="1" s="1">
       <c r="A31" s="8" t="n"/>
-      <c r="B31" s="8" t="n"/>
-      <c r="C31" s="8" t="n"/>
-      <c r="D31" s="8" t="n"/>
-      <c r="E31" s="8" t="n"/>
-      <c r="F31" s="69" t="n"/>
-      <c r="G31" s="8" t="n"/>
-      <c r="H31" s="8" t="n"/>
-      <c r="I31" s="8" t="n"/>
-      <c r="J31" s="69" t="n"/>
-      <c r="K31" s="8" t="n"/>
-      <c r="L31" s="8" t="n"/>
-      <c r="M31" s="70" t="n"/>
+      <c r="B31" s="108" t="n"/>
+      <c r="C31" s="109" t="n"/>
+      <c r="D31" s="109" t="n"/>
+      <c r="E31" s="110" t="n"/>
+      <c r="F31" s="111" t="n"/>
+      <c r="G31" s="112" t="n"/>
+      <c r="H31" s="112" t="n"/>
+      <c r="I31" s="113" t="n"/>
+      <c r="J31" s="114" t="n"/>
+      <c r="K31" s="115" t="n"/>
+      <c r="L31" s="115" t="n"/>
+      <c r="M31" s="116" t="n"/>
       <c r="N31" s="89" t="n"/>
       <c r="O31" s="90" t="n"/>
       <c r="P31" s="91" t="n"/>
@@ -6414,18 +6528,18 @@
     </row>
     <row r="32" ht="18" customFormat="1" customHeight="1" s="1">
       <c r="A32" s="9" t="n"/>
-      <c r="B32" s="9" t="n"/>
-      <c r="C32" s="9" t="n"/>
-      <c r="D32" s="9" t="n"/>
-      <c r="E32" s="9" t="n"/>
-      <c r="F32" s="71" t="n"/>
-      <c r="G32" s="9" t="n"/>
-      <c r="H32" s="9" t="n"/>
-      <c r="I32" s="9" t="n"/>
-      <c r="J32" s="71" t="n"/>
-      <c r="K32" s="9" t="n"/>
-      <c r="L32" s="9" t="n"/>
-      <c r="M32" s="72" t="n"/>
+      <c r="B32" s="108" t="n"/>
+      <c r="C32" s="109" t="n"/>
+      <c r="D32" s="109" t="n"/>
+      <c r="E32" s="110" t="n"/>
+      <c r="F32" s="111" t="n"/>
+      <c r="G32" s="112" t="n"/>
+      <c r="H32" s="112" t="n"/>
+      <c r="I32" s="113" t="n"/>
+      <c r="J32" s="114" t="n"/>
+      <c r="K32" s="115" t="n"/>
+      <c r="L32" s="115" t="n"/>
+      <c r="M32" s="116" t="n"/>
       <c r="N32" s="89" t="n"/>
       <c r="O32" s="90" t="n"/>
       <c r="P32" s="91" t="n"/>
@@ -6438,18 +6552,18 @@
     </row>
     <row r="33" ht="18" customFormat="1" customHeight="1" s="1">
       <c r="A33" s="8" t="n"/>
-      <c r="B33" s="8" t="n"/>
-      <c r="C33" s="8" t="n"/>
-      <c r="D33" s="8" t="n"/>
-      <c r="E33" s="8" t="n"/>
-      <c r="F33" s="69" t="n"/>
-      <c r="G33" s="8" t="n"/>
-      <c r="H33" s="8" t="n"/>
-      <c r="I33" s="8" t="n"/>
-      <c r="J33" s="69" t="n"/>
-      <c r="K33" s="8" t="n"/>
-      <c r="L33" s="8" t="n"/>
-      <c r="M33" s="70" t="n"/>
+      <c r="B33" s="108" t="n"/>
+      <c r="C33" s="109" t="n"/>
+      <c r="D33" s="109" t="n"/>
+      <c r="E33" s="110" t="n"/>
+      <c r="F33" s="111" t="n"/>
+      <c r="G33" s="112" t="n"/>
+      <c r="H33" s="112" t="n"/>
+      <c r="I33" s="113" t="n"/>
+      <c r="J33" s="114" t="n"/>
+      <c r="K33" s="115" t="n"/>
+      <c r="L33" s="115" t="n"/>
+      <c r="M33" s="116" t="n"/>
       <c r="N33" s="89" t="n"/>
       <c r="O33" s="90" t="n"/>
       <c r="P33" s="91" t="n"/>
@@ -6462,18 +6576,18 @@
     </row>
     <row r="34" ht="18" customFormat="1" customHeight="1" s="1">
       <c r="A34" s="9" t="n"/>
-      <c r="B34" s="9" t="n"/>
-      <c r="C34" s="9" t="n"/>
-      <c r="D34" s="9" t="n"/>
-      <c r="E34" s="9" t="n"/>
-      <c r="F34" s="71" t="n"/>
-      <c r="G34" s="9" t="n"/>
-      <c r="H34" s="9" t="n"/>
-      <c r="I34" s="9" t="n"/>
-      <c r="J34" s="71" t="n"/>
-      <c r="K34" s="9" t="n"/>
-      <c r="L34" s="9" t="n"/>
-      <c r="M34" s="72" t="n"/>
+      <c r="B34" s="108" t="n"/>
+      <c r="C34" s="109" t="n"/>
+      <c r="D34" s="109" t="n"/>
+      <c r="E34" s="110" t="n"/>
+      <c r="F34" s="111" t="n"/>
+      <c r="G34" s="112" t="n"/>
+      <c r="H34" s="112" t="n"/>
+      <c r="I34" s="113" t="n"/>
+      <c r="J34" s="114" t="n"/>
+      <c r="K34" s="115" t="n"/>
+      <c r="L34" s="115" t="n"/>
+      <c r="M34" s="116" t="n"/>
       <c r="N34" s="89" t="n"/>
       <c r="O34" s="90" t="n"/>
       <c r="P34" s="91" t="n"/>

</xml_diff>

<commit_message>
Redesign RSI Data sheet to A1/A2/A3 attempt columns
Replaces the 4-column summary-value layout (Avg RSI, Avg GCT, Max RSI,
Max GCT per leg) with 6 attempt columns per leg (RSI A1/A2/A3 + GCT
A1/A2/A3), matching the sprint sheet pattern. Engine now auto-computes
avg RSI, best RSI, and avg GCT from whatever attempts are filled —
works with 1, 2, or 3 entries. Fixes the root cause of all RSI data
showing as missing (users were entering slash-separated values like
"1.3/1.3/2.2" in single cells which _safe_float() couldn't parse).

- engine/transform_raw_data.py: add _avg_of(), update RSI_COLS (28 cols,
  was 22), rewrite _transform_rsi_row to compute from attempts
- public/AMSC_Combine_Data_Template.xlsx: rebuild RSI Data sheet header
  with new attempt columns; drop jump section unchanged

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/AMSC_Combine_Data_Template.xlsx
+++ b/public/AMSC_Combine_Data_Template.xlsx
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="25">
+  <fonts count="30">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -188,8 +188,36 @@
       <color rgb="00FFFFFF"/>
       <sz val="9"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="00D3D3D3"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="00F5F5F8"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <i val="1"/>
+      <color rgb="00D3D3D3"/>
+      <sz val="8"/>
+    </font>
   </fonts>
-  <fills count="21">
+  <fills count="26">
     <fill>
       <patternFill/>
     </fill>
@@ -289,6 +317,31 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF001A04"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001A1A1A"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001A3A5C"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001A4A2A"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001A2A4A"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001A0000"/>
       </patternFill>
     </fill>
   </fills>
@@ -611,7 +664,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2"/>
   </cellStyleXfs>
-  <cellXfs count="117">
+  <cellXfs count="146">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
@@ -922,6 +975,93 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="20" borderId="33" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="21" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="12" borderId="16" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="11" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="22" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="23" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="24" borderId="24" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="24" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="11" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="11" borderId="16" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="11" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="22" borderId="16" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="22" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="22" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="23" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="23" borderId="16" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="23" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="24" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="24" borderId="16" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="24" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="25" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="25" borderId="22" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="25" borderId="32" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="25" borderId="33" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="25" borderId="29" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="25" borderId="30" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="25" borderId="31" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="25" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="21" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -5649,35 +5789,41 @@
     <outlinePr summaryBelow="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V35"/>
+  <dimension ref="A1:AB35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="22.005" bestFit="1" customWidth="1" style="16" min="1" max="1"/>
-    <col width="13.005" bestFit="1" customWidth="1" style="38" min="2" max="2"/>
-    <col width="13.005" bestFit="1" customWidth="1" style="38" min="3" max="3"/>
-    <col width="13.005" bestFit="1" customWidth="1" style="38" min="4" max="4"/>
-    <col width="13.005" bestFit="1" customWidth="1" style="38" min="5" max="5"/>
-    <col width="13.005" bestFit="1" customWidth="1" style="38" min="6" max="6"/>
-    <col width="13.005" bestFit="1" customWidth="1" style="38" min="7" max="7"/>
-    <col width="13.005" bestFit="1" customWidth="1" style="38" min="8" max="8"/>
-    <col width="13.005" bestFit="1" customWidth="1" style="38" min="9" max="9"/>
-    <col width="13.005" bestFit="1" customWidth="1" style="38" min="10" max="10"/>
-    <col width="13.005" bestFit="1" customWidth="1" style="38" min="11" max="11"/>
-    <col width="13.005" bestFit="1" customWidth="1" style="38" min="12" max="12"/>
-    <col width="13.005" bestFit="1" customWidth="1" style="38" min="13" max="13"/>
-    <col width="13" customWidth="1" min="14" max="14"/>
-    <col width="13" customWidth="1" min="15" max="15"/>
-    <col width="13" customWidth="1" min="16" max="16"/>
-    <col width="13" customWidth="1" min="17" max="17"/>
-    <col width="13" customWidth="1" min="18" max="18"/>
-    <col width="13" customWidth="1" min="19" max="19"/>
-    <col width="13" customWidth="1" min="20" max="20"/>
-    <col width="13" customWidth="1" min="21" max="21"/>
-    <col width="13" customWidth="1" min="22" max="22"/>
+    <col width="22" bestFit="1" customWidth="1" style="16" min="1" max="1"/>
+    <col width="11" bestFit="1" customWidth="1" style="38" min="2" max="2"/>
+    <col width="11" bestFit="1" customWidth="1" style="38" min="3" max="3"/>
+    <col width="11" bestFit="1" customWidth="1" style="38" min="4" max="4"/>
+    <col width="11" bestFit="1" customWidth="1" style="38" min="5" max="5"/>
+    <col width="11" bestFit="1" customWidth="1" style="38" min="6" max="6"/>
+    <col width="11" bestFit="1" customWidth="1" style="38" min="7" max="7"/>
+    <col width="11" bestFit="1" customWidth="1" style="38" min="8" max="8"/>
+    <col width="11" bestFit="1" customWidth="1" style="38" min="9" max="9"/>
+    <col width="11" bestFit="1" customWidth="1" style="38" min="10" max="10"/>
+    <col width="11" bestFit="1" customWidth="1" style="38" min="11" max="11"/>
+    <col width="11" bestFit="1" customWidth="1" style="38" min="12" max="12"/>
+    <col width="11" bestFit="1" customWidth="1" style="38" min="13" max="13"/>
+    <col width="11" customWidth="1" min="14" max="14"/>
+    <col width="11" customWidth="1" min="15" max="15"/>
+    <col width="11" customWidth="1" min="16" max="16"/>
+    <col width="11" customWidth="1" min="17" max="17"/>
+    <col width="11" customWidth="1" min="18" max="18"/>
+    <col width="11" customWidth="1" min="19" max="19"/>
+    <col width="11" customWidth="1" min="20" max="20"/>
+    <col width="11" customWidth="1" min="21" max="21"/>
+    <col width="11" customWidth="1" min="22" max="22"/>
+    <col width="11" customWidth="1" min="23" max="23"/>
+    <col width="11" customWidth="1" min="24" max="24"/>
+    <col width="11" customWidth="1" min="25" max="25"/>
+    <col width="11" customWidth="1" min="26" max="26"/>
+    <col width="11" customWidth="1" min="27" max="27"/>
+    <col width="11" customWidth="1" min="28" max="28"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customFormat="1" customHeight="1" s="1">
-      <c r="A1" s="2" t="inlineStr">
+      <c r="A1" s="117" t="inlineStr">
         <is>
           <t>AMSC COMBINE — RSI DATA</t>
         </is>
@@ -5693,12 +5839,27 @@
       <c r="J1" s="53" t="n"/>
       <c r="K1" s="53" t="n"/>
       <c r="L1" s="53" t="n"/>
-      <c r="M1" s="54" t="n"/>
-    </row>
-    <row r="2" ht="36" customHeight="1">
-      <c r="A2" s="4" t="inlineStr">
-        <is>
-          <t>Enter the four summary values per leg. Avg RSI = mean RSI across all hops.  Avg GCT = mean ground contact time (s).  Max RSI = best single hop RSI.  Max GCT = GCT recorded at the max RSI hop.  All RSI fields are optional — athletes without RSI data still receive full reports.</t>
+      <c r="M1" s="53" t="n"/>
+      <c r="N1" s="53" t="n"/>
+      <c r="O1" s="53" t="n"/>
+      <c r="P1" s="53" t="n"/>
+      <c r="Q1" s="53" t="n"/>
+      <c r="R1" s="53" t="n"/>
+      <c r="S1" s="53" t="n"/>
+      <c r="T1" s="53" t="n"/>
+      <c r="U1" s="53" t="n"/>
+      <c r="V1" s="53" t="n"/>
+      <c r="W1" s="53" t="n"/>
+      <c r="X1" s="53" t="n"/>
+      <c r="Y1" s="53" t="n"/>
+      <c r="Z1" s="53" t="n"/>
+      <c r="AA1" s="53" t="n"/>
+      <c r="AB1" s="54" t="n"/>
+    </row>
+    <row r="2" ht="42" customHeight="1">
+      <c r="A2" s="118" t="inlineStr">
+        <is>
+          <t>Enter up to 3 hop attempts per leg. The engine automatically computes Avg RSI, Best RSI, and Avg GCT from whichever attempts are filled — 1, 2, or 3.  RSI = Jump Height (m) ÷ GCT (s).  GCT = ground contact time in seconds.  All RSI fields are optional — athletes without RSI data still receive full reports.</t>
         </is>
       </c>
       <c r="B2" s="53" t="n"/>
@@ -5712,896 +5873,1118 @@
       <c r="J2" s="53" t="n"/>
       <c r="K2" s="53" t="n"/>
       <c r="L2" s="53" t="n"/>
-      <c r="M2" s="54" t="n"/>
+      <c r="M2" s="53" t="n"/>
+      <c r="N2" s="53" t="n"/>
+      <c r="O2" s="53" t="n"/>
+      <c r="P2" s="53" t="n"/>
+      <c r="Q2" s="53" t="n"/>
+      <c r="R2" s="53" t="n"/>
+      <c r="S2" s="53" t="n"/>
+      <c r="T2" s="53" t="n"/>
+      <c r="U2" s="53" t="n"/>
+      <c r="V2" s="53" t="n"/>
+      <c r="W2" s="53" t="n"/>
+      <c r="X2" s="53" t="n"/>
+      <c r="Y2" s="53" t="n"/>
+      <c r="Z2" s="53" t="n"/>
+      <c r="AA2" s="53" t="n"/>
+      <c r="AB2" s="54" t="n"/>
     </row>
     <row r="3" ht="22" customFormat="1" customHeight="1" s="1">
-      <c r="A3" s="73" t="inlineStr">
+      <c r="A3" s="119" t="inlineStr">
         <is>
           <t>ATHLETE INFO</t>
         </is>
       </c>
-      <c r="B3" s="74" t="inlineStr">
-        <is>
-          <t>DOUBLE-LEG</t>
-        </is>
-      </c>
-      <c r="C3" s="75" t="n"/>
-      <c r="D3" s="75" t="n"/>
-      <c r="E3" s="76" t="n"/>
-      <c r="F3" s="92" t="inlineStr">
+      <c r="B3" s="120" t="inlineStr">
+        <is>
+          <t>DOUBLE-LEG HOP</t>
+        </is>
+      </c>
+      <c r="C3" s="81" t="n"/>
+      <c r="D3" s="81" t="n"/>
+      <c r="E3" s="81" t="n"/>
+      <c r="F3" s="81" t="n"/>
+      <c r="G3" s="82" t="n"/>
+      <c r="H3" s="121" t="inlineStr">
         <is>
           <t>SINGLE-LEG — LEFT</t>
         </is>
       </c>
-      <c r="G3" s="93" t="n"/>
-      <c r="H3" s="93" t="n"/>
-      <c r="I3" s="94" t="n"/>
-      <c r="J3" s="95" t="inlineStr">
+      <c r="N3" s="122" t="inlineStr">
         <is>
           <t>SINGLE-LEG — RIGHT</t>
         </is>
       </c>
-      <c r="K3" s="96" t="n"/>
-      <c r="L3" s="96" t="n"/>
-      <c r="M3" s="97" t="n"/>
-      <c r="N3" s="98" t="inlineStr">
-        <is>
-          <t>40cm DROP JUMP</t>
-        </is>
-      </c>
       <c r="O3" s="81" t="n"/>
-      <c r="P3" s="82" t="n"/>
-      <c r="Q3" s="98" t="inlineStr">
-        <is>
-          <t>50cm DROP JUMP</t>
-        </is>
-      </c>
+      <c r="P3" s="81" t="n"/>
+      <c r="Q3" s="81" t="n"/>
       <c r="R3" s="81" t="n"/>
       <c r="S3" s="82" t="n"/>
-      <c r="T3" s="98" t="inlineStr">
-        <is>
-          <t>60cm DROP JUMP</t>
+      <c r="T3" s="123" t="inlineStr">
+        <is>
+          <t>40cm DROP JUMP</t>
         </is>
       </c>
       <c r="U3" s="81" t="n"/>
       <c r="V3" s="82" t="n"/>
+      <c r="W3" s="124" t="inlineStr">
+        <is>
+          <t>50cm DROP JUMP</t>
+        </is>
+      </c>
+      <c r="Z3" s="124" t="inlineStr">
+        <is>
+          <t>60cm DROP JUMP</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="30" customFormat="1" customHeight="1" s="1">
-      <c r="A4" s="77" t="inlineStr">
+      <c r="A4" s="119" t="inlineStr">
         <is>
           <t>Athlete Name*</t>
         </is>
       </c>
-      <c r="B4" s="99" t="inlineStr">
-        <is>
-          <t>Avg RSI</t>
-        </is>
-      </c>
-      <c r="C4" s="100" t="inlineStr">
-        <is>
-          <t>Avg GCT (s)</t>
-        </is>
-      </c>
-      <c r="D4" s="100" t="inlineStr">
-        <is>
-          <t>Max RSI</t>
-        </is>
-      </c>
-      <c r="E4" s="101" t="inlineStr">
-        <is>
-          <t>Max GCT (s)</t>
-        </is>
-      </c>
-      <c r="F4" s="102" t="inlineStr">
-        <is>
-          <t>Avg RSI</t>
-        </is>
-      </c>
-      <c r="G4" s="103" t="inlineStr">
-        <is>
-          <t>Avg GCT (s)</t>
-        </is>
-      </c>
-      <c r="H4" s="103" t="inlineStr">
-        <is>
-          <t>Max RSI</t>
-        </is>
-      </c>
-      <c r="I4" s="104" t="inlineStr">
-        <is>
-          <t>Max GCT (s)</t>
-        </is>
-      </c>
-      <c r="J4" s="105" t="inlineStr">
-        <is>
-          <t>Avg RSI</t>
-        </is>
-      </c>
-      <c r="K4" s="106" t="inlineStr">
-        <is>
-          <t>Avg GCT (s)</t>
-        </is>
-      </c>
-      <c r="L4" s="106" t="inlineStr">
-        <is>
-          <t>Max RSI</t>
-        </is>
-      </c>
-      <c r="M4" s="107" t="inlineStr">
-        <is>
-          <t>Max GCT (s)</t>
-        </is>
-      </c>
-      <c r="N4" s="86" t="inlineStr">
+      <c r="B4" s="125" t="inlineStr">
+        <is>
+          <t>RSI A1</t>
+        </is>
+      </c>
+      <c r="C4" s="126" t="inlineStr">
+        <is>
+          <t>RSI A2</t>
+        </is>
+      </c>
+      <c r="D4" s="126" t="inlineStr">
+        <is>
+          <t>RSI A3</t>
+        </is>
+      </c>
+      <c r="E4" s="127" t="inlineStr">
+        <is>
+          <t>GCT A1 (s)</t>
+        </is>
+      </c>
+      <c r="F4" s="125" t="inlineStr">
+        <is>
+          <t>GCT A2 (s)</t>
+        </is>
+      </c>
+      <c r="G4" s="126" t="inlineStr">
+        <is>
+          <t>GCT A3 (s)</t>
+        </is>
+      </c>
+      <c r="H4" s="128" t="inlineStr">
+        <is>
+          <t>RSI A1</t>
+        </is>
+      </c>
+      <c r="I4" s="129" t="inlineStr">
+        <is>
+          <t>RSI A2</t>
+        </is>
+      </c>
+      <c r="J4" s="130" t="inlineStr">
+        <is>
+          <t>RSI A3</t>
+        </is>
+      </c>
+      <c r="K4" s="128" t="inlineStr">
+        <is>
+          <t>GCT A1 (s)</t>
+        </is>
+      </c>
+      <c r="L4" s="128" t="inlineStr">
+        <is>
+          <t>GCT A2 (s)</t>
+        </is>
+      </c>
+      <c r="M4" s="129" t="inlineStr">
+        <is>
+          <t>GCT A3 (s)</t>
+        </is>
+      </c>
+      <c r="N4" s="131" t="inlineStr">
+        <is>
+          <t>RSI A1</t>
+        </is>
+      </c>
+      <c r="O4" s="132" t="inlineStr">
+        <is>
+          <t>RSI A2</t>
+        </is>
+      </c>
+      <c r="P4" s="133" t="inlineStr">
+        <is>
+          <t>RSI A3</t>
+        </is>
+      </c>
+      <c r="Q4" s="131" t="inlineStr">
+        <is>
+          <t>GCT A1 (s)</t>
+        </is>
+      </c>
+      <c r="R4" s="132" t="inlineStr">
+        <is>
+          <t>GCT A2 (s)</t>
+        </is>
+      </c>
+      <c r="S4" s="133" t="inlineStr">
+        <is>
+          <t>GCT A3 (s)</t>
+        </is>
+      </c>
+      <c r="T4" s="134" t="inlineStr">
         <is>
           <t>RSI</t>
         </is>
       </c>
-      <c r="O4" s="87" t="inlineStr">
+      <c r="U4" s="135" t="inlineStr">
         <is>
           <t>Jump Ht (cm)</t>
         </is>
       </c>
-      <c r="P4" s="88" t="inlineStr">
+      <c r="V4" s="136" t="inlineStr">
         <is>
           <t>GCT (s)</t>
         </is>
       </c>
-      <c r="Q4" s="86" t="inlineStr">
+      <c r="W4" s="124" t="inlineStr">
         <is>
           <t>RSI</t>
         </is>
       </c>
-      <c r="R4" s="87" t="inlineStr">
+      <c r="X4" s="124" t="inlineStr">
         <is>
           <t>Jump Ht (cm)</t>
         </is>
       </c>
-      <c r="S4" s="88" t="inlineStr">
+      <c r="Y4" s="124" t="inlineStr">
         <is>
           <t>GCT (s)</t>
         </is>
       </c>
-      <c r="T4" s="86" t="inlineStr">
+      <c r="Z4" s="124" t="inlineStr">
         <is>
           <t>RSI</t>
         </is>
       </c>
-      <c r="U4" s="87" t="inlineStr">
+      <c r="AA4" s="124" t="inlineStr">
         <is>
           <t>Jump Ht (cm)</t>
         </is>
       </c>
-      <c r="V4" s="88" t="inlineStr">
+      <c r="AB4" s="124" t="inlineStr">
         <is>
           <t>GCT (s)</t>
         </is>
       </c>
     </row>
     <row r="5" ht="18" customFormat="1" customHeight="1" s="1">
-      <c r="A5" s="8" t="n"/>
-      <c r="B5" s="108" t="n"/>
-      <c r="C5" s="109" t="n"/>
-      <c r="D5" s="109" t="n"/>
-      <c r="E5" s="110" t="n"/>
-      <c r="F5" s="111" t="n"/>
-      <c r="G5" s="112" t="n"/>
-      <c r="H5" s="112" t="n"/>
-      <c r="I5" s="113" t="n"/>
-      <c r="J5" s="114" t="n"/>
-      <c r="K5" s="115" t="n"/>
-      <c r="L5" s="115" t="n"/>
-      <c r="M5" s="116" t="n"/>
-      <c r="N5" s="89" t="n"/>
-      <c r="O5" s="90" t="n"/>
-      <c r="P5" s="91" t="n"/>
-      <c r="Q5" s="89" t="n"/>
-      <c r="R5" s="90" t="n"/>
-      <c r="S5" s="91" t="n"/>
-      <c r="T5" s="89" t="n"/>
-      <c r="U5" s="90" t="n"/>
-      <c r="V5" s="91" t="n"/>
+      <c r="A5" s="137" t="n"/>
+      <c r="B5" s="138" t="n"/>
+      <c r="C5" s="139" t="n"/>
+      <c r="D5" s="139" t="n"/>
+      <c r="E5" s="140" t="n"/>
+      <c r="F5" s="138" t="n"/>
+      <c r="G5" s="139" t="n"/>
+      <c r="H5" s="139" t="n"/>
+      <c r="I5" s="140" t="n"/>
+      <c r="J5" s="138" t="n"/>
+      <c r="K5" s="139" t="n"/>
+      <c r="L5" s="139" t="n"/>
+      <c r="M5" s="140" t="n"/>
+      <c r="N5" s="141" t="n"/>
+      <c r="O5" s="142" t="n"/>
+      <c r="P5" s="143" t="n"/>
+      <c r="Q5" s="141" t="n"/>
+      <c r="R5" s="142" t="n"/>
+      <c r="S5" s="143" t="n"/>
+      <c r="T5" s="141" t="n"/>
+      <c r="U5" s="142" t="n"/>
+      <c r="V5" s="143" t="n"/>
+      <c r="W5" s="144" t="n"/>
+      <c r="X5" s="144" t="n"/>
+      <c r="Y5" s="144" t="n"/>
+      <c r="Z5" s="144" t="n"/>
+      <c r="AA5" s="144" t="n"/>
+      <c r="AB5" s="144" t="n"/>
     </row>
     <row r="6" ht="18" customFormat="1" customHeight="1" s="1">
-      <c r="A6" s="9" t="n"/>
-      <c r="B6" s="108" t="n"/>
-      <c r="C6" s="109" t="n"/>
-      <c r="D6" s="109" t="n"/>
-      <c r="E6" s="110" t="n"/>
-      <c r="F6" s="111" t="n"/>
-      <c r="G6" s="112" t="n"/>
-      <c r="H6" s="112" t="n"/>
-      <c r="I6" s="113" t="n"/>
-      <c r="J6" s="114" t="n"/>
-      <c r="K6" s="115" t="n"/>
-      <c r="L6" s="115" t="n"/>
-      <c r="M6" s="116" t="n"/>
-      <c r="N6" s="89" t="n"/>
-      <c r="O6" s="90" t="n"/>
-      <c r="P6" s="91" t="n"/>
-      <c r="Q6" s="89" t="n"/>
-      <c r="R6" s="90" t="n"/>
-      <c r="S6" s="91" t="n"/>
-      <c r="T6" s="89" t="n"/>
-      <c r="U6" s="90" t="n"/>
-      <c r="V6" s="91" t="n"/>
+      <c r="A6" s="137" t="n"/>
+      <c r="B6" s="138" t="n"/>
+      <c r="C6" s="139" t="n"/>
+      <c r="D6" s="139" t="n"/>
+      <c r="E6" s="140" t="n"/>
+      <c r="F6" s="138" t="n"/>
+      <c r="G6" s="139" t="n"/>
+      <c r="H6" s="139" t="n"/>
+      <c r="I6" s="140" t="n"/>
+      <c r="J6" s="138" t="n"/>
+      <c r="K6" s="139" t="n"/>
+      <c r="L6" s="139" t="n"/>
+      <c r="M6" s="140" t="n"/>
+      <c r="N6" s="141" t="n"/>
+      <c r="O6" s="142" t="n"/>
+      <c r="P6" s="143" t="n"/>
+      <c r="Q6" s="141" t="n"/>
+      <c r="R6" s="142" t="n"/>
+      <c r="S6" s="143" t="n"/>
+      <c r="T6" s="141" t="n"/>
+      <c r="U6" s="142" t="n"/>
+      <c r="V6" s="143" t="n"/>
+      <c r="W6" s="144" t="n"/>
+      <c r="X6" s="144" t="n"/>
+      <c r="Y6" s="144" t="n"/>
+      <c r="Z6" s="144" t="n"/>
+      <c r="AA6" s="144" t="n"/>
+      <c r="AB6" s="144" t="n"/>
     </row>
     <row r="7" ht="18" customFormat="1" customHeight="1" s="1">
-      <c r="A7" s="8" t="n"/>
-      <c r="B7" s="108" t="n"/>
-      <c r="C7" s="109" t="n"/>
-      <c r="D7" s="109" t="n"/>
-      <c r="E7" s="110" t="n"/>
-      <c r="F7" s="111" t="n"/>
-      <c r="G7" s="112" t="n"/>
-      <c r="H7" s="112" t="n"/>
-      <c r="I7" s="113" t="n"/>
-      <c r="J7" s="114" t="n"/>
-      <c r="K7" s="115" t="n"/>
-      <c r="L7" s="115" t="n"/>
-      <c r="M7" s="116" t="n"/>
-      <c r="N7" s="89" t="n"/>
-      <c r="O7" s="90" t="n"/>
-      <c r="P7" s="91" t="n"/>
-      <c r="Q7" s="89" t="n"/>
-      <c r="R7" s="90" t="n"/>
-      <c r="S7" s="91" t="n"/>
-      <c r="T7" s="89" t="n"/>
-      <c r="U7" s="90" t="n"/>
-      <c r="V7" s="91" t="n"/>
+      <c r="A7" s="137" t="n"/>
+      <c r="B7" s="138" t="n"/>
+      <c r="C7" s="139" t="n"/>
+      <c r="D7" s="139" t="n"/>
+      <c r="E7" s="140" t="n"/>
+      <c r="F7" s="138" t="n"/>
+      <c r="G7" s="139" t="n"/>
+      <c r="H7" s="139" t="n"/>
+      <c r="I7" s="140" t="n"/>
+      <c r="J7" s="138" t="n"/>
+      <c r="K7" s="139" t="n"/>
+      <c r="L7" s="139" t="n"/>
+      <c r="M7" s="140" t="n"/>
+      <c r="N7" s="141" t="n"/>
+      <c r="O7" s="142" t="n"/>
+      <c r="P7" s="143" t="n"/>
+      <c r="Q7" s="141" t="n"/>
+      <c r="R7" s="142" t="n"/>
+      <c r="S7" s="143" t="n"/>
+      <c r="T7" s="141" t="n"/>
+      <c r="U7" s="142" t="n"/>
+      <c r="V7" s="143" t="n"/>
+      <c r="W7" s="144" t="n"/>
+      <c r="X7" s="144" t="n"/>
+      <c r="Y7" s="144" t="n"/>
+      <c r="Z7" s="144" t="n"/>
+      <c r="AA7" s="144" t="n"/>
+      <c r="AB7" s="144" t="n"/>
     </row>
     <row r="8" ht="18" customFormat="1" customHeight="1" s="1">
-      <c r="A8" s="9" t="n"/>
-      <c r="B8" s="108" t="n"/>
-      <c r="C8" s="109" t="n"/>
-      <c r="D8" s="109" t="n"/>
-      <c r="E8" s="110" t="n"/>
-      <c r="F8" s="111" t="n"/>
-      <c r="G8" s="112" t="n"/>
-      <c r="H8" s="112" t="n"/>
-      <c r="I8" s="113" t="n"/>
-      <c r="J8" s="114" t="n"/>
-      <c r="K8" s="115" t="n"/>
-      <c r="L8" s="115" t="n"/>
-      <c r="M8" s="116" t="n"/>
-      <c r="N8" s="89" t="n"/>
-      <c r="O8" s="90" t="n"/>
-      <c r="P8" s="91" t="n"/>
-      <c r="Q8" s="89" t="n"/>
-      <c r="R8" s="90" t="n"/>
-      <c r="S8" s="91" t="n"/>
-      <c r="T8" s="89" t="n"/>
-      <c r="U8" s="90" t="n"/>
-      <c r="V8" s="91" t="n"/>
+      <c r="A8" s="137" t="n"/>
+      <c r="B8" s="138" t="n"/>
+      <c r="C8" s="139" t="n"/>
+      <c r="D8" s="139" t="n"/>
+      <c r="E8" s="140" t="n"/>
+      <c r="F8" s="138" t="n"/>
+      <c r="G8" s="139" t="n"/>
+      <c r="H8" s="139" t="n"/>
+      <c r="I8" s="140" t="n"/>
+      <c r="J8" s="138" t="n"/>
+      <c r="K8" s="139" t="n"/>
+      <c r="L8" s="139" t="n"/>
+      <c r="M8" s="140" t="n"/>
+      <c r="N8" s="141" t="n"/>
+      <c r="O8" s="142" t="n"/>
+      <c r="P8" s="143" t="n"/>
+      <c r="Q8" s="141" t="n"/>
+      <c r="R8" s="142" t="n"/>
+      <c r="S8" s="143" t="n"/>
+      <c r="T8" s="141" t="n"/>
+      <c r="U8" s="142" t="n"/>
+      <c r="V8" s="143" t="n"/>
+      <c r="W8" s="144" t="n"/>
+      <c r="X8" s="144" t="n"/>
+      <c r="Y8" s="144" t="n"/>
+      <c r="Z8" s="144" t="n"/>
+      <c r="AA8" s="144" t="n"/>
+      <c r="AB8" s="144" t="n"/>
     </row>
     <row r="9" ht="18" customFormat="1" customHeight="1" s="1">
-      <c r="A9" s="8" t="n"/>
-      <c r="B9" s="108" t="n"/>
-      <c r="C9" s="109" t="n"/>
-      <c r="D9" s="109" t="n"/>
-      <c r="E9" s="110" t="n"/>
-      <c r="F9" s="111" t="n"/>
-      <c r="G9" s="112" t="n"/>
-      <c r="H9" s="112" t="n"/>
-      <c r="I9" s="113" t="n"/>
-      <c r="J9" s="114" t="n"/>
-      <c r="K9" s="115" t="n"/>
-      <c r="L9" s="115" t="n"/>
-      <c r="M9" s="116" t="n"/>
-      <c r="N9" s="89" t="n"/>
-      <c r="O9" s="90" t="n"/>
-      <c r="P9" s="91" t="n"/>
-      <c r="Q9" s="89" t="n"/>
-      <c r="R9" s="90" t="n"/>
-      <c r="S9" s="91" t="n"/>
-      <c r="T9" s="89" t="n"/>
-      <c r="U9" s="90" t="n"/>
-      <c r="V9" s="91" t="n"/>
+      <c r="A9" s="137" t="n"/>
+      <c r="B9" s="138" t="n"/>
+      <c r="C9" s="139" t="n"/>
+      <c r="D9" s="139" t="n"/>
+      <c r="E9" s="140" t="n"/>
+      <c r="F9" s="138" t="n"/>
+      <c r="G9" s="139" t="n"/>
+      <c r="H9" s="139" t="n"/>
+      <c r="I9" s="140" t="n"/>
+      <c r="J9" s="138" t="n"/>
+      <c r="K9" s="139" t="n"/>
+      <c r="L9" s="139" t="n"/>
+      <c r="M9" s="140" t="n"/>
+      <c r="N9" s="141" t="n"/>
+      <c r="O9" s="142" t="n"/>
+      <c r="P9" s="143" t="n"/>
+      <c r="Q9" s="141" t="n"/>
+      <c r="R9" s="142" t="n"/>
+      <c r="S9" s="143" t="n"/>
+      <c r="T9" s="141" t="n"/>
+      <c r="U9" s="142" t="n"/>
+      <c r="V9" s="143" t="n"/>
+      <c r="W9" s="144" t="n"/>
+      <c r="X9" s="144" t="n"/>
+      <c r="Y9" s="144" t="n"/>
+      <c r="Z9" s="144" t="n"/>
+      <c r="AA9" s="144" t="n"/>
+      <c r="AB9" s="144" t="n"/>
     </row>
     <row r="10" ht="18" customFormat="1" customHeight="1" s="1">
-      <c r="A10" s="9" t="n"/>
-      <c r="B10" s="108" t="n"/>
-      <c r="C10" s="109" t="n"/>
-      <c r="D10" s="109" t="n"/>
-      <c r="E10" s="110" t="n"/>
-      <c r="F10" s="111" t="n"/>
-      <c r="G10" s="112" t="n"/>
-      <c r="H10" s="112" t="n"/>
-      <c r="I10" s="113" t="n"/>
-      <c r="J10" s="114" t="n"/>
-      <c r="K10" s="115" t="n"/>
-      <c r="L10" s="115" t="n"/>
-      <c r="M10" s="116" t="n"/>
-      <c r="N10" s="89" t="n"/>
-      <c r="O10" s="90" t="n"/>
-      <c r="P10" s="91" t="n"/>
-      <c r="Q10" s="89" t="n"/>
-      <c r="R10" s="90" t="n"/>
-      <c r="S10" s="91" t="n"/>
-      <c r="T10" s="89" t="n"/>
-      <c r="U10" s="90" t="n"/>
-      <c r="V10" s="91" t="n"/>
+      <c r="A10" s="137" t="n"/>
+      <c r="B10" s="138" t="n"/>
+      <c r="C10" s="139" t="n"/>
+      <c r="D10" s="139" t="n"/>
+      <c r="E10" s="140" t="n"/>
+      <c r="F10" s="138" t="n"/>
+      <c r="G10" s="139" t="n"/>
+      <c r="H10" s="139" t="n"/>
+      <c r="I10" s="140" t="n"/>
+      <c r="J10" s="138" t="n"/>
+      <c r="K10" s="139" t="n"/>
+      <c r="L10" s="139" t="n"/>
+      <c r="M10" s="140" t="n"/>
+      <c r="N10" s="141" t="n"/>
+      <c r="O10" s="142" t="n"/>
+      <c r="P10" s="143" t="n"/>
+      <c r="Q10" s="141" t="n"/>
+      <c r="R10" s="142" t="n"/>
+      <c r="S10" s="143" t="n"/>
+      <c r="T10" s="141" t="n"/>
+      <c r="U10" s="142" t="n"/>
+      <c r="V10" s="143" t="n"/>
+      <c r="W10" s="144" t="n"/>
+      <c r="X10" s="144" t="n"/>
+      <c r="Y10" s="144" t="n"/>
+      <c r="Z10" s="144" t="n"/>
+      <c r="AA10" s="144" t="n"/>
+      <c r="AB10" s="144" t="n"/>
     </row>
     <row r="11" ht="18" customFormat="1" customHeight="1" s="1">
-      <c r="A11" s="8" t="n"/>
-      <c r="B11" s="108" t="n"/>
-      <c r="C11" s="109" t="n"/>
-      <c r="D11" s="109" t="n"/>
-      <c r="E11" s="110" t="n"/>
-      <c r="F11" s="111" t="n"/>
-      <c r="G11" s="112" t="n"/>
-      <c r="H11" s="112" t="n"/>
-      <c r="I11" s="113" t="n"/>
-      <c r="J11" s="114" t="n"/>
-      <c r="K11" s="115" t="n"/>
-      <c r="L11" s="115" t="n"/>
-      <c r="M11" s="116" t="n"/>
-      <c r="N11" s="89" t="n"/>
-      <c r="O11" s="90" t="n"/>
-      <c r="P11" s="91" t="n"/>
-      <c r="Q11" s="89" t="n"/>
-      <c r="R11" s="90" t="n"/>
-      <c r="S11" s="91" t="n"/>
-      <c r="T11" s="89" t="n"/>
-      <c r="U11" s="90" t="n"/>
-      <c r="V11" s="91" t="n"/>
+      <c r="A11" s="137" t="n"/>
+      <c r="B11" s="138" t="n"/>
+      <c r="C11" s="139" t="n"/>
+      <c r="D11" s="139" t="n"/>
+      <c r="E11" s="140" t="n"/>
+      <c r="F11" s="138" t="n"/>
+      <c r="G11" s="139" t="n"/>
+      <c r="H11" s="139" t="n"/>
+      <c r="I11" s="140" t="n"/>
+      <c r="J11" s="138" t="n"/>
+      <c r="K11" s="139" t="n"/>
+      <c r="L11" s="139" t="n"/>
+      <c r="M11" s="140" t="n"/>
+      <c r="N11" s="141" t="n"/>
+      <c r="O11" s="142" t="n"/>
+      <c r="P11" s="143" t="n"/>
+      <c r="Q11" s="141" t="n"/>
+      <c r="R11" s="142" t="n"/>
+      <c r="S11" s="143" t="n"/>
+      <c r="T11" s="141" t="n"/>
+      <c r="U11" s="142" t="n"/>
+      <c r="V11" s="143" t="n"/>
+      <c r="W11" s="144" t="n"/>
+      <c r="X11" s="144" t="n"/>
+      <c r="Y11" s="144" t="n"/>
+      <c r="Z11" s="144" t="n"/>
+      <c r="AA11" s="144" t="n"/>
+      <c r="AB11" s="144" t="n"/>
     </row>
     <row r="12" ht="18" customFormat="1" customHeight="1" s="1">
-      <c r="A12" s="9" t="n"/>
-      <c r="B12" s="108" t="n"/>
-      <c r="C12" s="109" t="n"/>
-      <c r="D12" s="109" t="n"/>
-      <c r="E12" s="110" t="n"/>
-      <c r="F12" s="111" t="n"/>
-      <c r="G12" s="112" t="n"/>
-      <c r="H12" s="112" t="n"/>
-      <c r="I12" s="113" t="n"/>
-      <c r="J12" s="114" t="n"/>
-      <c r="K12" s="115" t="n"/>
-      <c r="L12" s="115" t="n"/>
-      <c r="M12" s="116" t="n"/>
-      <c r="N12" s="89" t="n"/>
-      <c r="O12" s="90" t="n"/>
-      <c r="P12" s="91" t="n"/>
-      <c r="Q12" s="89" t="n"/>
-      <c r="R12" s="90" t="n"/>
-      <c r="S12" s="91" t="n"/>
-      <c r="T12" s="89" t="n"/>
-      <c r="U12" s="90" t="n"/>
-      <c r="V12" s="91" t="n"/>
+      <c r="A12" s="137" t="n"/>
+      <c r="B12" s="138" t="n"/>
+      <c r="C12" s="139" t="n"/>
+      <c r="D12" s="139" t="n"/>
+      <c r="E12" s="140" t="n"/>
+      <c r="F12" s="138" t="n"/>
+      <c r="G12" s="139" t="n"/>
+      <c r="H12" s="139" t="n"/>
+      <c r="I12" s="140" t="n"/>
+      <c r="J12" s="138" t="n"/>
+      <c r="K12" s="139" t="n"/>
+      <c r="L12" s="139" t="n"/>
+      <c r="M12" s="140" t="n"/>
+      <c r="N12" s="141" t="n"/>
+      <c r="O12" s="142" t="n"/>
+      <c r="P12" s="143" t="n"/>
+      <c r="Q12" s="141" t="n"/>
+      <c r="R12" s="142" t="n"/>
+      <c r="S12" s="143" t="n"/>
+      <c r="T12" s="141" t="n"/>
+      <c r="U12" s="142" t="n"/>
+      <c r="V12" s="143" t="n"/>
+      <c r="W12" s="144" t="n"/>
+      <c r="X12" s="144" t="n"/>
+      <c r="Y12" s="144" t="n"/>
+      <c r="Z12" s="144" t="n"/>
+      <c r="AA12" s="144" t="n"/>
+      <c r="AB12" s="144" t="n"/>
     </row>
     <row r="13" ht="18" customFormat="1" customHeight="1" s="1">
-      <c r="A13" s="8" t="n"/>
-      <c r="B13" s="108" t="n"/>
-      <c r="C13" s="109" t="n"/>
-      <c r="D13" s="109" t="n"/>
-      <c r="E13" s="110" t="n"/>
-      <c r="F13" s="111" t="n"/>
-      <c r="G13" s="112" t="n"/>
-      <c r="H13" s="112" t="n"/>
-      <c r="I13" s="113" t="n"/>
-      <c r="J13" s="114" t="n"/>
-      <c r="K13" s="115" t="n"/>
-      <c r="L13" s="115" t="n"/>
-      <c r="M13" s="116" t="n"/>
-      <c r="N13" s="89" t="n"/>
-      <c r="O13" s="90" t="n"/>
-      <c r="P13" s="91" t="n"/>
-      <c r="Q13" s="89" t="n"/>
-      <c r="R13" s="90" t="n"/>
-      <c r="S13" s="91" t="n"/>
-      <c r="T13" s="89" t="n"/>
-      <c r="U13" s="90" t="n"/>
-      <c r="V13" s="91" t="n"/>
+      <c r="A13" s="137" t="n"/>
+      <c r="B13" s="138" t="n"/>
+      <c r="C13" s="139" t="n"/>
+      <c r="D13" s="139" t="n"/>
+      <c r="E13" s="140" t="n"/>
+      <c r="F13" s="138" t="n"/>
+      <c r="G13" s="139" t="n"/>
+      <c r="H13" s="139" t="n"/>
+      <c r="I13" s="140" t="n"/>
+      <c r="J13" s="138" t="n"/>
+      <c r="K13" s="139" t="n"/>
+      <c r="L13" s="139" t="n"/>
+      <c r="M13" s="140" t="n"/>
+      <c r="N13" s="141" t="n"/>
+      <c r="O13" s="142" t="n"/>
+      <c r="P13" s="143" t="n"/>
+      <c r="Q13" s="141" t="n"/>
+      <c r="R13" s="142" t="n"/>
+      <c r="S13" s="143" t="n"/>
+      <c r="T13" s="141" t="n"/>
+      <c r="U13" s="142" t="n"/>
+      <c r="V13" s="143" t="n"/>
+      <c r="W13" s="144" t="n"/>
+      <c r="X13" s="144" t="n"/>
+      <c r="Y13" s="144" t="n"/>
+      <c r="Z13" s="144" t="n"/>
+      <c r="AA13" s="144" t="n"/>
+      <c r="AB13" s="144" t="n"/>
     </row>
     <row r="14" ht="18" customFormat="1" customHeight="1" s="1">
-      <c r="A14" s="9" t="n"/>
-      <c r="B14" s="108" t="n"/>
-      <c r="C14" s="109" t="n"/>
-      <c r="D14" s="109" t="n"/>
-      <c r="E14" s="110" t="n"/>
-      <c r="F14" s="111" t="n"/>
-      <c r="G14" s="112" t="n"/>
-      <c r="H14" s="112" t="n"/>
-      <c r="I14" s="113" t="n"/>
-      <c r="J14" s="114" t="n"/>
-      <c r="K14" s="115" t="n"/>
-      <c r="L14" s="115" t="n"/>
-      <c r="M14" s="116" t="n"/>
-      <c r="N14" s="89" t="n"/>
-      <c r="O14" s="90" t="n"/>
-      <c r="P14" s="91" t="n"/>
-      <c r="Q14" s="89" t="n"/>
-      <c r="R14" s="90" t="n"/>
-      <c r="S14" s="91" t="n"/>
-      <c r="T14" s="89" t="n"/>
-      <c r="U14" s="90" t="n"/>
-      <c r="V14" s="91" t="n"/>
+      <c r="A14" s="137" t="n"/>
+      <c r="B14" s="138" t="n"/>
+      <c r="C14" s="139" t="n"/>
+      <c r="D14" s="139" t="n"/>
+      <c r="E14" s="140" t="n"/>
+      <c r="F14" s="138" t="n"/>
+      <c r="G14" s="139" t="n"/>
+      <c r="H14" s="139" t="n"/>
+      <c r="I14" s="140" t="n"/>
+      <c r="J14" s="138" t="n"/>
+      <c r="K14" s="139" t="n"/>
+      <c r="L14" s="139" t="n"/>
+      <c r="M14" s="140" t="n"/>
+      <c r="N14" s="141" t="n"/>
+      <c r="O14" s="142" t="n"/>
+      <c r="P14" s="143" t="n"/>
+      <c r="Q14" s="141" t="n"/>
+      <c r="R14" s="142" t="n"/>
+      <c r="S14" s="143" t="n"/>
+      <c r="T14" s="141" t="n"/>
+      <c r="U14" s="142" t="n"/>
+      <c r="V14" s="143" t="n"/>
+      <c r="W14" s="144" t="n"/>
+      <c r="X14" s="144" t="n"/>
+      <c r="Y14" s="144" t="n"/>
+      <c r="Z14" s="144" t="n"/>
+      <c r="AA14" s="144" t="n"/>
+      <c r="AB14" s="144" t="n"/>
     </row>
     <row r="15" ht="18" customFormat="1" customHeight="1" s="1">
-      <c r="A15" s="8" t="n"/>
-      <c r="B15" s="108" t="n"/>
-      <c r="C15" s="109" t="n"/>
-      <c r="D15" s="109" t="n"/>
-      <c r="E15" s="110" t="n"/>
-      <c r="F15" s="111" t="n"/>
-      <c r="G15" s="112" t="n"/>
-      <c r="H15" s="112" t="n"/>
-      <c r="I15" s="113" t="n"/>
-      <c r="J15" s="114" t="n"/>
-      <c r="K15" s="115" t="n"/>
-      <c r="L15" s="115" t="n"/>
-      <c r="M15" s="116" t="n"/>
-      <c r="N15" s="89" t="n"/>
-      <c r="O15" s="90" t="n"/>
-      <c r="P15" s="91" t="n"/>
-      <c r="Q15" s="89" t="n"/>
-      <c r="R15" s="90" t="n"/>
-      <c r="S15" s="91" t="n"/>
-      <c r="T15" s="89" t="n"/>
-      <c r="U15" s="90" t="n"/>
-      <c r="V15" s="91" t="n"/>
+      <c r="A15" s="137" t="n"/>
+      <c r="B15" s="138" t="n"/>
+      <c r="C15" s="139" t="n"/>
+      <c r="D15" s="139" t="n"/>
+      <c r="E15" s="140" t="n"/>
+      <c r="F15" s="138" t="n"/>
+      <c r="G15" s="139" t="n"/>
+      <c r="H15" s="139" t="n"/>
+      <c r="I15" s="140" t="n"/>
+      <c r="J15" s="138" t="n"/>
+      <c r="K15" s="139" t="n"/>
+      <c r="L15" s="139" t="n"/>
+      <c r="M15" s="140" t="n"/>
+      <c r="N15" s="141" t="n"/>
+      <c r="O15" s="142" t="n"/>
+      <c r="P15" s="143" t="n"/>
+      <c r="Q15" s="141" t="n"/>
+      <c r="R15" s="142" t="n"/>
+      <c r="S15" s="143" t="n"/>
+      <c r="T15" s="141" t="n"/>
+      <c r="U15" s="142" t="n"/>
+      <c r="V15" s="143" t="n"/>
+      <c r="W15" s="144" t="n"/>
+      <c r="X15" s="144" t="n"/>
+      <c r="Y15" s="144" t="n"/>
+      <c r="Z15" s="144" t="n"/>
+      <c r="AA15" s="144" t="n"/>
+      <c r="AB15" s="144" t="n"/>
     </row>
     <row r="16" ht="18" customFormat="1" customHeight="1" s="1">
-      <c r="A16" s="9" t="n"/>
-      <c r="B16" s="108" t="n"/>
-      <c r="C16" s="109" t="n"/>
-      <c r="D16" s="109" t="n"/>
-      <c r="E16" s="110" t="n"/>
-      <c r="F16" s="111" t="n"/>
-      <c r="G16" s="112" t="n"/>
-      <c r="H16" s="112" t="n"/>
-      <c r="I16" s="113" t="n"/>
-      <c r="J16" s="114" t="n"/>
-      <c r="K16" s="115" t="n"/>
-      <c r="L16" s="115" t="n"/>
-      <c r="M16" s="116" t="n"/>
-      <c r="N16" s="89" t="n"/>
-      <c r="O16" s="90" t="n"/>
-      <c r="P16" s="91" t="n"/>
-      <c r="Q16" s="89" t="n"/>
-      <c r="R16" s="90" t="n"/>
-      <c r="S16" s="91" t="n"/>
-      <c r="T16" s="89" t="n"/>
-      <c r="U16" s="90" t="n"/>
-      <c r="V16" s="91" t="n"/>
+      <c r="A16" s="137" t="n"/>
+      <c r="B16" s="138" t="n"/>
+      <c r="C16" s="139" t="n"/>
+      <c r="D16" s="139" t="n"/>
+      <c r="E16" s="140" t="n"/>
+      <c r="F16" s="138" t="n"/>
+      <c r="G16" s="139" t="n"/>
+      <c r="H16" s="139" t="n"/>
+      <c r="I16" s="140" t="n"/>
+      <c r="J16" s="138" t="n"/>
+      <c r="K16" s="139" t="n"/>
+      <c r="L16" s="139" t="n"/>
+      <c r="M16" s="140" t="n"/>
+      <c r="N16" s="141" t="n"/>
+      <c r="O16" s="142" t="n"/>
+      <c r="P16" s="143" t="n"/>
+      <c r="Q16" s="141" t="n"/>
+      <c r="R16" s="142" t="n"/>
+      <c r="S16" s="143" t="n"/>
+      <c r="T16" s="141" t="n"/>
+      <c r="U16" s="142" t="n"/>
+      <c r="V16" s="143" t="n"/>
+      <c r="W16" s="144" t="n"/>
+      <c r="X16" s="144" t="n"/>
+      <c r="Y16" s="144" t="n"/>
+      <c r="Z16" s="144" t="n"/>
+      <c r="AA16" s="144" t="n"/>
+      <c r="AB16" s="144" t="n"/>
     </row>
     <row r="17" ht="18" customFormat="1" customHeight="1" s="1">
-      <c r="A17" s="8" t="n"/>
-      <c r="B17" s="108" t="n"/>
-      <c r="C17" s="109" t="n"/>
-      <c r="D17" s="109" t="n"/>
-      <c r="E17" s="110" t="n"/>
-      <c r="F17" s="111" t="n"/>
-      <c r="G17" s="112" t="n"/>
-      <c r="H17" s="112" t="n"/>
-      <c r="I17" s="113" t="n"/>
-      <c r="J17" s="114" t="n"/>
-      <c r="K17" s="115" t="n"/>
-      <c r="L17" s="115" t="n"/>
-      <c r="M17" s="116" t="n"/>
-      <c r="N17" s="89" t="n"/>
-      <c r="O17" s="90" t="n"/>
-      <c r="P17" s="91" t="n"/>
-      <c r="Q17" s="89" t="n"/>
-      <c r="R17" s="90" t="n"/>
-      <c r="S17" s="91" t="n"/>
-      <c r="T17" s="89" t="n"/>
-      <c r="U17" s="90" t="n"/>
-      <c r="V17" s="91" t="n"/>
+      <c r="A17" s="137" t="n"/>
+      <c r="B17" s="138" t="n"/>
+      <c r="C17" s="139" t="n"/>
+      <c r="D17" s="139" t="n"/>
+      <c r="E17" s="140" t="n"/>
+      <c r="F17" s="138" t="n"/>
+      <c r="G17" s="139" t="n"/>
+      <c r="H17" s="139" t="n"/>
+      <c r="I17" s="140" t="n"/>
+      <c r="J17" s="138" t="n"/>
+      <c r="K17" s="139" t="n"/>
+      <c r="L17" s="139" t="n"/>
+      <c r="M17" s="140" t="n"/>
+      <c r="N17" s="141" t="n"/>
+      <c r="O17" s="142" t="n"/>
+      <c r="P17" s="143" t="n"/>
+      <c r="Q17" s="141" t="n"/>
+      <c r="R17" s="142" t="n"/>
+      <c r="S17" s="143" t="n"/>
+      <c r="T17" s="141" t="n"/>
+      <c r="U17" s="142" t="n"/>
+      <c r="V17" s="143" t="n"/>
+      <c r="W17" s="144" t="n"/>
+      <c r="X17" s="144" t="n"/>
+      <c r="Y17" s="144" t="n"/>
+      <c r="Z17" s="144" t="n"/>
+      <c r="AA17" s="144" t="n"/>
+      <c r="AB17" s="144" t="n"/>
     </row>
     <row r="18" ht="18" customFormat="1" customHeight="1" s="1">
-      <c r="A18" s="9" t="n"/>
-      <c r="B18" s="108" t="n"/>
-      <c r="C18" s="109" t="n"/>
-      <c r="D18" s="109" t="n"/>
-      <c r="E18" s="110" t="n"/>
-      <c r="F18" s="111" t="n"/>
-      <c r="G18" s="112" t="n"/>
-      <c r="H18" s="112" t="n"/>
-      <c r="I18" s="113" t="n"/>
-      <c r="J18" s="114" t="n"/>
-      <c r="K18" s="115" t="n"/>
-      <c r="L18" s="115" t="n"/>
-      <c r="M18" s="116" t="n"/>
-      <c r="N18" s="89" t="n"/>
-      <c r="O18" s="90" t="n"/>
-      <c r="P18" s="91" t="n"/>
-      <c r="Q18" s="89" t="n"/>
-      <c r="R18" s="90" t="n"/>
-      <c r="S18" s="91" t="n"/>
-      <c r="T18" s="89" t="n"/>
-      <c r="U18" s="90" t="n"/>
-      <c r="V18" s="91" t="n"/>
+      <c r="A18" s="137" t="n"/>
+      <c r="B18" s="138" t="n"/>
+      <c r="C18" s="139" t="n"/>
+      <c r="D18" s="139" t="n"/>
+      <c r="E18" s="140" t="n"/>
+      <c r="F18" s="138" t="n"/>
+      <c r="G18" s="139" t="n"/>
+      <c r="H18" s="139" t="n"/>
+      <c r="I18" s="140" t="n"/>
+      <c r="J18" s="138" t="n"/>
+      <c r="K18" s="139" t="n"/>
+      <c r="L18" s="139" t="n"/>
+      <c r="M18" s="140" t="n"/>
+      <c r="N18" s="141" t="n"/>
+      <c r="O18" s="142" t="n"/>
+      <c r="P18" s="143" t="n"/>
+      <c r="Q18" s="141" t="n"/>
+      <c r="R18" s="142" t="n"/>
+      <c r="S18" s="143" t="n"/>
+      <c r="T18" s="141" t="n"/>
+      <c r="U18" s="142" t="n"/>
+      <c r="V18" s="143" t="n"/>
+      <c r="W18" s="144" t="n"/>
+      <c r="X18" s="144" t="n"/>
+      <c r="Y18" s="144" t="n"/>
+      <c r="Z18" s="144" t="n"/>
+      <c r="AA18" s="144" t="n"/>
+      <c r="AB18" s="144" t="n"/>
     </row>
     <row r="19" ht="18" customFormat="1" customHeight="1" s="1">
-      <c r="A19" s="8" t="n"/>
-      <c r="B19" s="108" t="n"/>
-      <c r="C19" s="109" t="n"/>
-      <c r="D19" s="109" t="n"/>
-      <c r="E19" s="110" t="n"/>
-      <c r="F19" s="111" t="n"/>
-      <c r="G19" s="112" t="n"/>
-      <c r="H19" s="112" t="n"/>
-      <c r="I19" s="113" t="n"/>
-      <c r="J19" s="114" t="n"/>
-      <c r="K19" s="115" t="n"/>
-      <c r="L19" s="115" t="n"/>
-      <c r="M19" s="116" t="n"/>
-      <c r="N19" s="89" t="n"/>
-      <c r="O19" s="90" t="n"/>
-      <c r="P19" s="91" t="n"/>
-      <c r="Q19" s="89" t="n"/>
-      <c r="R19" s="90" t="n"/>
-      <c r="S19" s="91" t="n"/>
-      <c r="T19" s="89" t="n"/>
-      <c r="U19" s="90" t="n"/>
-      <c r="V19" s="91" t="n"/>
+      <c r="A19" s="137" t="n"/>
+      <c r="B19" s="138" t="n"/>
+      <c r="C19" s="139" t="n"/>
+      <c r="D19" s="139" t="n"/>
+      <c r="E19" s="140" t="n"/>
+      <c r="F19" s="138" t="n"/>
+      <c r="G19" s="139" t="n"/>
+      <c r="H19" s="139" t="n"/>
+      <c r="I19" s="140" t="n"/>
+      <c r="J19" s="138" t="n"/>
+      <c r="K19" s="139" t="n"/>
+      <c r="L19" s="139" t="n"/>
+      <c r="M19" s="140" t="n"/>
+      <c r="N19" s="141" t="n"/>
+      <c r="O19" s="142" t="n"/>
+      <c r="P19" s="143" t="n"/>
+      <c r="Q19" s="141" t="n"/>
+      <c r="R19" s="142" t="n"/>
+      <c r="S19" s="143" t="n"/>
+      <c r="T19" s="141" t="n"/>
+      <c r="U19" s="142" t="n"/>
+      <c r="V19" s="143" t="n"/>
+      <c r="W19" s="144" t="n"/>
+      <c r="X19" s="144" t="n"/>
+      <c r="Y19" s="144" t="n"/>
+      <c r="Z19" s="144" t="n"/>
+      <c r="AA19" s="144" t="n"/>
+      <c r="AB19" s="144" t="n"/>
     </row>
     <row r="20" ht="18" customFormat="1" customHeight="1" s="1">
-      <c r="A20" s="9" t="n"/>
-      <c r="B20" s="108" t="n"/>
-      <c r="C20" s="109" t="n"/>
-      <c r="D20" s="109" t="n"/>
-      <c r="E20" s="110" t="n"/>
-      <c r="F20" s="111" t="n"/>
-      <c r="G20" s="112" t="n"/>
-      <c r="H20" s="112" t="n"/>
-      <c r="I20" s="113" t="n"/>
-      <c r="J20" s="114" t="n"/>
-      <c r="K20" s="115" t="n"/>
-      <c r="L20" s="115" t="n"/>
-      <c r="M20" s="116" t="n"/>
-      <c r="N20" s="89" t="n"/>
-      <c r="O20" s="90" t="n"/>
-      <c r="P20" s="91" t="n"/>
-      <c r="Q20" s="89" t="n"/>
-      <c r="R20" s="90" t="n"/>
-      <c r="S20" s="91" t="n"/>
-      <c r="T20" s="89" t="n"/>
-      <c r="U20" s="90" t="n"/>
-      <c r="V20" s="91" t="n"/>
+      <c r="A20" s="137" t="n"/>
+      <c r="B20" s="138" t="n"/>
+      <c r="C20" s="139" t="n"/>
+      <c r="D20" s="139" t="n"/>
+      <c r="E20" s="140" t="n"/>
+      <c r="F20" s="138" t="n"/>
+      <c r="G20" s="139" t="n"/>
+      <c r="H20" s="139" t="n"/>
+      <c r="I20" s="140" t="n"/>
+      <c r="J20" s="138" t="n"/>
+      <c r="K20" s="139" t="n"/>
+      <c r="L20" s="139" t="n"/>
+      <c r="M20" s="140" t="n"/>
+      <c r="N20" s="141" t="n"/>
+      <c r="O20" s="142" t="n"/>
+      <c r="P20" s="143" t="n"/>
+      <c r="Q20" s="141" t="n"/>
+      <c r="R20" s="142" t="n"/>
+      <c r="S20" s="143" t="n"/>
+      <c r="T20" s="141" t="n"/>
+      <c r="U20" s="142" t="n"/>
+      <c r="V20" s="143" t="n"/>
+      <c r="W20" s="144" t="n"/>
+      <c r="X20" s="144" t="n"/>
+      <c r="Y20" s="144" t="n"/>
+      <c r="Z20" s="144" t="n"/>
+      <c r="AA20" s="144" t="n"/>
+      <c r="AB20" s="144" t="n"/>
     </row>
     <row r="21" ht="18" customFormat="1" customHeight="1" s="1">
-      <c r="A21" s="8" t="n"/>
-      <c r="B21" s="108" t="n"/>
-      <c r="C21" s="109" t="n"/>
-      <c r="D21" s="109" t="n"/>
-      <c r="E21" s="110" t="n"/>
-      <c r="F21" s="111" t="n"/>
-      <c r="G21" s="112" t="n"/>
-      <c r="H21" s="112" t="n"/>
-      <c r="I21" s="113" t="n"/>
-      <c r="J21" s="114" t="n"/>
-      <c r="K21" s="115" t="n"/>
-      <c r="L21" s="115" t="n"/>
-      <c r="M21" s="116" t="n"/>
-      <c r="N21" s="89" t="n"/>
-      <c r="O21" s="90" t="n"/>
-      <c r="P21" s="91" t="n"/>
-      <c r="Q21" s="89" t="n"/>
-      <c r="R21" s="90" t="n"/>
-      <c r="S21" s="91" t="n"/>
-      <c r="T21" s="89" t="n"/>
-      <c r="U21" s="90" t="n"/>
-      <c r="V21" s="91" t="n"/>
+      <c r="A21" s="137" t="n"/>
+      <c r="B21" s="138" t="n"/>
+      <c r="C21" s="139" t="n"/>
+      <c r="D21" s="139" t="n"/>
+      <c r="E21" s="140" t="n"/>
+      <c r="F21" s="138" t="n"/>
+      <c r="G21" s="139" t="n"/>
+      <c r="H21" s="139" t="n"/>
+      <c r="I21" s="140" t="n"/>
+      <c r="J21" s="138" t="n"/>
+      <c r="K21" s="139" t="n"/>
+      <c r="L21" s="139" t="n"/>
+      <c r="M21" s="140" t="n"/>
+      <c r="N21" s="141" t="n"/>
+      <c r="O21" s="142" t="n"/>
+      <c r="P21" s="143" t="n"/>
+      <c r="Q21" s="141" t="n"/>
+      <c r="R21" s="142" t="n"/>
+      <c r="S21" s="143" t="n"/>
+      <c r="T21" s="141" t="n"/>
+      <c r="U21" s="142" t="n"/>
+      <c r="V21" s="143" t="n"/>
+      <c r="W21" s="144" t="n"/>
+      <c r="X21" s="144" t="n"/>
+      <c r="Y21" s="144" t="n"/>
+      <c r="Z21" s="144" t="n"/>
+      <c r="AA21" s="144" t="n"/>
+      <c r="AB21" s="144" t="n"/>
     </row>
     <row r="22" ht="18" customFormat="1" customHeight="1" s="1">
-      <c r="A22" s="9" t="n"/>
-      <c r="B22" s="108" t="n"/>
-      <c r="C22" s="109" t="n"/>
-      <c r="D22" s="109" t="n"/>
-      <c r="E22" s="110" t="n"/>
-      <c r="F22" s="111" t="n"/>
-      <c r="G22" s="112" t="n"/>
-      <c r="H22" s="112" t="n"/>
-      <c r="I22" s="113" t="n"/>
-      <c r="J22" s="114" t="n"/>
-      <c r="K22" s="115" t="n"/>
-      <c r="L22" s="115" t="n"/>
-      <c r="M22" s="116" t="n"/>
-      <c r="N22" s="89" t="n"/>
-      <c r="O22" s="90" t="n"/>
-      <c r="P22" s="91" t="n"/>
-      <c r="Q22" s="89" t="n"/>
-      <c r="R22" s="90" t="n"/>
-      <c r="S22" s="91" t="n"/>
-      <c r="T22" s="89" t="n"/>
-      <c r="U22" s="90" t="n"/>
-      <c r="V22" s="91" t="n"/>
+      <c r="A22" s="137" t="n"/>
+      <c r="B22" s="138" t="n"/>
+      <c r="C22" s="139" t="n"/>
+      <c r="D22" s="139" t="n"/>
+      <c r="E22" s="140" t="n"/>
+      <c r="F22" s="138" t="n"/>
+      <c r="G22" s="139" t="n"/>
+      <c r="H22" s="139" t="n"/>
+      <c r="I22" s="140" t="n"/>
+      <c r="J22" s="138" t="n"/>
+      <c r="K22" s="139" t="n"/>
+      <c r="L22" s="139" t="n"/>
+      <c r="M22" s="140" t="n"/>
+      <c r="N22" s="141" t="n"/>
+      <c r="O22" s="142" t="n"/>
+      <c r="P22" s="143" t="n"/>
+      <c r="Q22" s="141" t="n"/>
+      <c r="R22" s="142" t="n"/>
+      <c r="S22" s="143" t="n"/>
+      <c r="T22" s="141" t="n"/>
+      <c r="U22" s="142" t="n"/>
+      <c r="V22" s="143" t="n"/>
+      <c r="W22" s="144" t="n"/>
+      <c r="X22" s="144" t="n"/>
+      <c r="Y22" s="144" t="n"/>
+      <c r="Z22" s="144" t="n"/>
+      <c r="AA22" s="144" t="n"/>
+      <c r="AB22" s="144" t="n"/>
     </row>
     <row r="23" ht="18" customFormat="1" customHeight="1" s="1">
-      <c r="A23" s="8" t="n"/>
-      <c r="B23" s="108" t="n"/>
-      <c r="C23" s="109" t="n"/>
-      <c r="D23" s="109" t="n"/>
-      <c r="E23" s="110" t="n"/>
-      <c r="F23" s="111" t="n"/>
-      <c r="G23" s="112" t="n"/>
-      <c r="H23" s="112" t="n"/>
-      <c r="I23" s="113" t="n"/>
-      <c r="J23" s="114" t="n"/>
-      <c r="K23" s="115" t="n"/>
-      <c r="L23" s="115" t="n"/>
-      <c r="M23" s="116" t="n"/>
-      <c r="N23" s="89" t="n"/>
-      <c r="O23" s="90" t="n"/>
-      <c r="P23" s="91" t="n"/>
-      <c r="Q23" s="89" t="n"/>
-      <c r="R23" s="90" t="n"/>
-      <c r="S23" s="91" t="n"/>
-      <c r="T23" s="89" t="n"/>
-      <c r="U23" s="90" t="n"/>
-      <c r="V23" s="91" t="n"/>
+      <c r="A23" s="137" t="n"/>
+      <c r="B23" s="138" t="n"/>
+      <c r="C23" s="139" t="n"/>
+      <c r="D23" s="139" t="n"/>
+      <c r="E23" s="140" t="n"/>
+      <c r="F23" s="138" t="n"/>
+      <c r="G23" s="139" t="n"/>
+      <c r="H23" s="139" t="n"/>
+      <c r="I23" s="140" t="n"/>
+      <c r="J23" s="138" t="n"/>
+      <c r="K23" s="139" t="n"/>
+      <c r="L23" s="139" t="n"/>
+      <c r="M23" s="140" t="n"/>
+      <c r="N23" s="141" t="n"/>
+      <c r="O23" s="142" t="n"/>
+      <c r="P23" s="143" t="n"/>
+      <c r="Q23" s="141" t="n"/>
+      <c r="R23" s="142" t="n"/>
+      <c r="S23" s="143" t="n"/>
+      <c r="T23" s="141" t="n"/>
+      <c r="U23" s="142" t="n"/>
+      <c r="V23" s="143" t="n"/>
+      <c r="W23" s="144" t="n"/>
+      <c r="X23" s="144" t="n"/>
+      <c r="Y23" s="144" t="n"/>
+      <c r="Z23" s="144" t="n"/>
+      <c r="AA23" s="144" t="n"/>
+      <c r="AB23" s="144" t="n"/>
     </row>
     <row r="24" ht="18" customFormat="1" customHeight="1" s="1">
-      <c r="A24" s="9" t="n"/>
-      <c r="B24" s="108" t="n"/>
-      <c r="C24" s="109" t="n"/>
-      <c r="D24" s="109" t="n"/>
-      <c r="E24" s="110" t="n"/>
-      <c r="F24" s="111" t="n"/>
-      <c r="G24" s="112" t="n"/>
-      <c r="H24" s="112" t="n"/>
-      <c r="I24" s="113" t="n"/>
-      <c r="J24" s="114" t="n"/>
-      <c r="K24" s="115" t="n"/>
-      <c r="L24" s="115" t="n"/>
-      <c r="M24" s="116" t="n"/>
-      <c r="N24" s="89" t="n"/>
-      <c r="O24" s="90" t="n"/>
-      <c r="P24" s="91" t="n"/>
-      <c r="Q24" s="89" t="n"/>
-      <c r="R24" s="90" t="n"/>
-      <c r="S24" s="91" t="n"/>
-      <c r="T24" s="89" t="n"/>
-      <c r="U24" s="90" t="n"/>
-      <c r="V24" s="91" t="n"/>
+      <c r="A24" s="137" t="n"/>
+      <c r="B24" s="138" t="n"/>
+      <c r="C24" s="139" t="n"/>
+      <c r="D24" s="139" t="n"/>
+      <c r="E24" s="140" t="n"/>
+      <c r="F24" s="138" t="n"/>
+      <c r="G24" s="139" t="n"/>
+      <c r="H24" s="139" t="n"/>
+      <c r="I24" s="140" t="n"/>
+      <c r="J24" s="138" t="n"/>
+      <c r="K24" s="139" t="n"/>
+      <c r="L24" s="139" t="n"/>
+      <c r="M24" s="140" t="n"/>
+      <c r="N24" s="141" t="n"/>
+      <c r="O24" s="142" t="n"/>
+      <c r="P24" s="143" t="n"/>
+      <c r="Q24" s="141" t="n"/>
+      <c r="R24" s="142" t="n"/>
+      <c r="S24" s="143" t="n"/>
+      <c r="T24" s="141" t="n"/>
+      <c r="U24" s="142" t="n"/>
+      <c r="V24" s="143" t="n"/>
+      <c r="W24" s="144" t="n"/>
+      <c r="X24" s="144" t="n"/>
+      <c r="Y24" s="144" t="n"/>
+      <c r="Z24" s="144" t="n"/>
+      <c r="AA24" s="144" t="n"/>
+      <c r="AB24" s="144" t="n"/>
     </row>
     <row r="25" ht="18" customFormat="1" customHeight="1" s="1">
-      <c r="A25" s="8" t="n"/>
-      <c r="B25" s="108" t="n"/>
-      <c r="C25" s="109" t="n"/>
-      <c r="D25" s="109" t="n"/>
-      <c r="E25" s="110" t="n"/>
-      <c r="F25" s="111" t="n"/>
-      <c r="G25" s="112" t="n"/>
-      <c r="H25" s="112" t="n"/>
-      <c r="I25" s="113" t="n"/>
-      <c r="J25" s="114" t="n"/>
-      <c r="K25" s="115" t="n"/>
-      <c r="L25" s="115" t="n"/>
-      <c r="M25" s="116" t="n"/>
-      <c r="N25" s="89" t="n"/>
-      <c r="O25" s="90" t="n"/>
-      <c r="P25" s="91" t="n"/>
-      <c r="Q25" s="89" t="n"/>
-      <c r="R25" s="90" t="n"/>
-      <c r="S25" s="91" t="n"/>
-      <c r="T25" s="89" t="n"/>
-      <c r="U25" s="90" t="n"/>
-      <c r="V25" s="91" t="n"/>
+      <c r="A25" s="137" t="n"/>
+      <c r="B25" s="138" t="n"/>
+      <c r="C25" s="139" t="n"/>
+      <c r="D25" s="139" t="n"/>
+      <c r="E25" s="140" t="n"/>
+      <c r="F25" s="138" t="n"/>
+      <c r="G25" s="139" t="n"/>
+      <c r="H25" s="139" t="n"/>
+      <c r="I25" s="140" t="n"/>
+      <c r="J25" s="138" t="n"/>
+      <c r="K25" s="139" t="n"/>
+      <c r="L25" s="139" t="n"/>
+      <c r="M25" s="140" t="n"/>
+      <c r="N25" s="141" t="n"/>
+      <c r="O25" s="142" t="n"/>
+      <c r="P25" s="143" t="n"/>
+      <c r="Q25" s="141" t="n"/>
+      <c r="R25" s="142" t="n"/>
+      <c r="S25" s="143" t="n"/>
+      <c r="T25" s="141" t="n"/>
+      <c r="U25" s="142" t="n"/>
+      <c r="V25" s="143" t="n"/>
+      <c r="W25" s="144" t="n"/>
+      <c r="X25" s="144" t="n"/>
+      <c r="Y25" s="144" t="n"/>
+      <c r="Z25" s="144" t="n"/>
+      <c r="AA25" s="144" t="n"/>
+      <c r="AB25" s="144" t="n"/>
     </row>
     <row r="26" ht="18" customFormat="1" customHeight="1" s="1">
-      <c r="A26" s="9" t="n"/>
-      <c r="B26" s="108" t="n"/>
-      <c r="C26" s="109" t="n"/>
-      <c r="D26" s="109" t="n"/>
-      <c r="E26" s="110" t="n"/>
-      <c r="F26" s="111" t="n"/>
-      <c r="G26" s="112" t="n"/>
-      <c r="H26" s="112" t="n"/>
-      <c r="I26" s="113" t="n"/>
-      <c r="J26" s="114" t="n"/>
-      <c r="K26" s="115" t="n"/>
-      <c r="L26" s="115" t="n"/>
-      <c r="M26" s="116" t="n"/>
-      <c r="N26" s="89" t="n"/>
-      <c r="O26" s="90" t="n"/>
-      <c r="P26" s="91" t="n"/>
-      <c r="Q26" s="89" t="n"/>
-      <c r="R26" s="90" t="n"/>
-      <c r="S26" s="91" t="n"/>
-      <c r="T26" s="89" t="n"/>
-      <c r="U26" s="90" t="n"/>
-      <c r="V26" s="91" t="n"/>
+      <c r="A26" s="137" t="n"/>
+      <c r="B26" s="138" t="n"/>
+      <c r="C26" s="139" t="n"/>
+      <c r="D26" s="139" t="n"/>
+      <c r="E26" s="140" t="n"/>
+      <c r="F26" s="138" t="n"/>
+      <c r="G26" s="139" t="n"/>
+      <c r="H26" s="139" t="n"/>
+      <c r="I26" s="140" t="n"/>
+      <c r="J26" s="138" t="n"/>
+      <c r="K26" s="139" t="n"/>
+      <c r="L26" s="139" t="n"/>
+      <c r="M26" s="140" t="n"/>
+      <c r="N26" s="141" t="n"/>
+      <c r="O26" s="142" t="n"/>
+      <c r="P26" s="143" t="n"/>
+      <c r="Q26" s="141" t="n"/>
+      <c r="R26" s="142" t="n"/>
+      <c r="S26" s="143" t="n"/>
+      <c r="T26" s="141" t="n"/>
+      <c r="U26" s="142" t="n"/>
+      <c r="V26" s="143" t="n"/>
+      <c r="W26" s="144" t="n"/>
+      <c r="X26" s="144" t="n"/>
+      <c r="Y26" s="144" t="n"/>
+      <c r="Z26" s="144" t="n"/>
+      <c r="AA26" s="144" t="n"/>
+      <c r="AB26" s="144" t="n"/>
     </row>
     <row r="27" ht="18" customFormat="1" customHeight="1" s="1">
-      <c r="A27" s="8" t="n"/>
-      <c r="B27" s="108" t="n"/>
-      <c r="C27" s="109" t="n"/>
-      <c r="D27" s="109" t="n"/>
-      <c r="E27" s="110" t="n"/>
-      <c r="F27" s="111" t="n"/>
-      <c r="G27" s="112" t="n"/>
-      <c r="H27" s="112" t="n"/>
-      <c r="I27" s="113" t="n"/>
-      <c r="J27" s="114" t="n"/>
-      <c r="K27" s="115" t="n"/>
-      <c r="L27" s="115" t="n"/>
-      <c r="M27" s="116" t="n"/>
-      <c r="N27" s="89" t="n"/>
-      <c r="O27" s="90" t="n"/>
-      <c r="P27" s="91" t="n"/>
-      <c r="Q27" s="89" t="n"/>
-      <c r="R27" s="90" t="n"/>
-      <c r="S27" s="91" t="n"/>
-      <c r="T27" s="89" t="n"/>
-      <c r="U27" s="90" t="n"/>
-      <c r="V27" s="91" t="n"/>
+      <c r="A27" s="137" t="n"/>
+      <c r="B27" s="138" t="n"/>
+      <c r="C27" s="139" t="n"/>
+      <c r="D27" s="139" t="n"/>
+      <c r="E27" s="140" t="n"/>
+      <c r="F27" s="138" t="n"/>
+      <c r="G27" s="139" t="n"/>
+      <c r="H27" s="139" t="n"/>
+      <c r="I27" s="140" t="n"/>
+      <c r="J27" s="138" t="n"/>
+      <c r="K27" s="139" t="n"/>
+      <c r="L27" s="139" t="n"/>
+      <c r="M27" s="140" t="n"/>
+      <c r="N27" s="141" t="n"/>
+      <c r="O27" s="142" t="n"/>
+      <c r="P27" s="143" t="n"/>
+      <c r="Q27" s="141" t="n"/>
+      <c r="R27" s="142" t="n"/>
+      <c r="S27" s="143" t="n"/>
+      <c r="T27" s="141" t="n"/>
+      <c r="U27" s="142" t="n"/>
+      <c r="V27" s="143" t="n"/>
+      <c r="W27" s="144" t="n"/>
+      <c r="X27" s="144" t="n"/>
+      <c r="Y27" s="144" t="n"/>
+      <c r="Z27" s="144" t="n"/>
+      <c r="AA27" s="144" t="n"/>
+      <c r="AB27" s="144" t="n"/>
     </row>
     <row r="28" ht="18" customFormat="1" customHeight="1" s="1">
-      <c r="A28" s="9" t="n"/>
-      <c r="B28" s="108" t="n"/>
-      <c r="C28" s="109" t="n"/>
-      <c r="D28" s="109" t="n"/>
-      <c r="E28" s="110" t="n"/>
-      <c r="F28" s="111" t="n"/>
-      <c r="G28" s="112" t="n"/>
-      <c r="H28" s="112" t="n"/>
-      <c r="I28" s="113" t="n"/>
-      <c r="J28" s="114" t="n"/>
-      <c r="K28" s="115" t="n"/>
-      <c r="L28" s="115" t="n"/>
-      <c r="M28" s="116" t="n"/>
-      <c r="N28" s="89" t="n"/>
-      <c r="O28" s="90" t="n"/>
-      <c r="P28" s="91" t="n"/>
-      <c r="Q28" s="89" t="n"/>
-      <c r="R28" s="90" t="n"/>
-      <c r="S28" s="91" t="n"/>
-      <c r="T28" s="89" t="n"/>
-      <c r="U28" s="90" t="n"/>
-      <c r="V28" s="91" t="n"/>
+      <c r="A28" s="137" t="n"/>
+      <c r="B28" s="138" t="n"/>
+      <c r="C28" s="139" t="n"/>
+      <c r="D28" s="139" t="n"/>
+      <c r="E28" s="140" t="n"/>
+      <c r="F28" s="138" t="n"/>
+      <c r="G28" s="139" t="n"/>
+      <c r="H28" s="139" t="n"/>
+      <c r="I28" s="140" t="n"/>
+      <c r="J28" s="138" t="n"/>
+      <c r="K28" s="139" t="n"/>
+      <c r="L28" s="139" t="n"/>
+      <c r="M28" s="140" t="n"/>
+      <c r="N28" s="141" t="n"/>
+      <c r="O28" s="142" t="n"/>
+      <c r="P28" s="143" t="n"/>
+      <c r="Q28" s="141" t="n"/>
+      <c r="R28" s="142" t="n"/>
+      <c r="S28" s="143" t="n"/>
+      <c r="T28" s="141" t="n"/>
+      <c r="U28" s="142" t="n"/>
+      <c r="V28" s="143" t="n"/>
+      <c r="W28" s="144" t="n"/>
+      <c r="X28" s="144" t="n"/>
+      <c r="Y28" s="144" t="n"/>
+      <c r="Z28" s="144" t="n"/>
+      <c r="AA28" s="144" t="n"/>
+      <c r="AB28" s="144" t="n"/>
     </row>
     <row r="29" ht="18" customFormat="1" customHeight="1" s="1">
-      <c r="A29" s="8" t="n"/>
-      <c r="B29" s="108" t="n"/>
-      <c r="C29" s="109" t="n"/>
-      <c r="D29" s="109" t="n"/>
-      <c r="E29" s="110" t="n"/>
-      <c r="F29" s="111" t="n"/>
-      <c r="G29" s="112" t="n"/>
-      <c r="H29" s="112" t="n"/>
-      <c r="I29" s="113" t="n"/>
-      <c r="J29" s="114" t="n"/>
-      <c r="K29" s="115" t="n"/>
-      <c r="L29" s="115" t="n"/>
-      <c r="M29" s="116" t="n"/>
-      <c r="N29" s="89" t="n"/>
-      <c r="O29" s="90" t="n"/>
-      <c r="P29" s="91" t="n"/>
-      <c r="Q29" s="89" t="n"/>
-      <c r="R29" s="90" t="n"/>
-      <c r="S29" s="91" t="n"/>
-      <c r="T29" s="89" t="n"/>
-      <c r="U29" s="90" t="n"/>
-      <c r="V29" s="91" t="n"/>
+      <c r="A29" s="137" t="n"/>
+      <c r="B29" s="138" t="n"/>
+      <c r="C29" s="139" t="n"/>
+      <c r="D29" s="139" t="n"/>
+      <c r="E29" s="140" t="n"/>
+      <c r="F29" s="138" t="n"/>
+      <c r="G29" s="139" t="n"/>
+      <c r="H29" s="139" t="n"/>
+      <c r="I29" s="140" t="n"/>
+      <c r="J29" s="138" t="n"/>
+      <c r="K29" s="139" t="n"/>
+      <c r="L29" s="139" t="n"/>
+      <c r="M29" s="140" t="n"/>
+      <c r="N29" s="141" t="n"/>
+      <c r="O29" s="142" t="n"/>
+      <c r="P29" s="143" t="n"/>
+      <c r="Q29" s="141" t="n"/>
+      <c r="R29" s="142" t="n"/>
+      <c r="S29" s="143" t="n"/>
+      <c r="T29" s="141" t="n"/>
+      <c r="U29" s="142" t="n"/>
+      <c r="V29" s="143" t="n"/>
+      <c r="W29" s="144" t="n"/>
+      <c r="X29" s="144" t="n"/>
+      <c r="Y29" s="144" t="n"/>
+      <c r="Z29" s="144" t="n"/>
+      <c r="AA29" s="144" t="n"/>
+      <c r="AB29" s="144" t="n"/>
     </row>
     <row r="30" ht="18" customFormat="1" customHeight="1" s="1">
-      <c r="A30" s="9" t="n"/>
-      <c r="B30" s="108" t="n"/>
-      <c r="C30" s="109" t="n"/>
-      <c r="D30" s="109" t="n"/>
-      <c r="E30" s="110" t="n"/>
-      <c r="F30" s="111" t="n"/>
-      <c r="G30" s="112" t="n"/>
-      <c r="H30" s="112" t="n"/>
-      <c r="I30" s="113" t="n"/>
-      <c r="J30" s="114" t="n"/>
-      <c r="K30" s="115" t="n"/>
-      <c r="L30" s="115" t="n"/>
-      <c r="M30" s="116" t="n"/>
-      <c r="N30" s="89" t="n"/>
-      <c r="O30" s="90" t="n"/>
-      <c r="P30" s="91" t="n"/>
-      <c r="Q30" s="89" t="n"/>
-      <c r="R30" s="90" t="n"/>
-      <c r="S30" s="91" t="n"/>
-      <c r="T30" s="89" t="n"/>
-      <c r="U30" s="90" t="n"/>
-      <c r="V30" s="91" t="n"/>
+      <c r="A30" s="137" t="n"/>
+      <c r="B30" s="138" t="n"/>
+      <c r="C30" s="139" t="n"/>
+      <c r="D30" s="139" t="n"/>
+      <c r="E30" s="140" t="n"/>
+      <c r="F30" s="138" t="n"/>
+      <c r="G30" s="139" t="n"/>
+      <c r="H30" s="139" t="n"/>
+      <c r="I30" s="140" t="n"/>
+      <c r="J30" s="138" t="n"/>
+      <c r="K30" s="139" t="n"/>
+      <c r="L30" s="139" t="n"/>
+      <c r="M30" s="140" t="n"/>
+      <c r="N30" s="141" t="n"/>
+      <c r="O30" s="142" t="n"/>
+      <c r="P30" s="143" t="n"/>
+      <c r="Q30" s="141" t="n"/>
+      <c r="R30" s="142" t="n"/>
+      <c r="S30" s="143" t="n"/>
+      <c r="T30" s="141" t="n"/>
+      <c r="U30" s="142" t="n"/>
+      <c r="V30" s="143" t="n"/>
+      <c r="W30" s="144" t="n"/>
+      <c r="X30" s="144" t="n"/>
+      <c r="Y30" s="144" t="n"/>
+      <c r="Z30" s="144" t="n"/>
+      <c r="AA30" s="144" t="n"/>
+      <c r="AB30" s="144" t="n"/>
     </row>
     <row r="31" ht="18" customFormat="1" customHeight="1" s="1">
-      <c r="A31" s="8" t="n"/>
-      <c r="B31" s="108" t="n"/>
-      <c r="C31" s="109" t="n"/>
-      <c r="D31" s="109" t="n"/>
-      <c r="E31" s="110" t="n"/>
-      <c r="F31" s="111" t="n"/>
-      <c r="G31" s="112" t="n"/>
-      <c r="H31" s="112" t="n"/>
-      <c r="I31" s="113" t="n"/>
-      <c r="J31" s="114" t="n"/>
-      <c r="K31" s="115" t="n"/>
-      <c r="L31" s="115" t="n"/>
-      <c r="M31" s="116" t="n"/>
-      <c r="N31" s="89" t="n"/>
-      <c r="O31" s="90" t="n"/>
-      <c r="P31" s="91" t="n"/>
-      <c r="Q31" s="89" t="n"/>
-      <c r="R31" s="90" t="n"/>
-      <c r="S31" s="91" t="n"/>
-      <c r="T31" s="89" t="n"/>
-      <c r="U31" s="90" t="n"/>
-      <c r="V31" s="91" t="n"/>
+      <c r="A31" s="137" t="n"/>
+      <c r="B31" s="138" t="n"/>
+      <c r="C31" s="139" t="n"/>
+      <c r="D31" s="139" t="n"/>
+      <c r="E31" s="140" t="n"/>
+      <c r="F31" s="138" t="n"/>
+      <c r="G31" s="139" t="n"/>
+      <c r="H31" s="139" t="n"/>
+      <c r="I31" s="140" t="n"/>
+      <c r="J31" s="138" t="n"/>
+      <c r="K31" s="139" t="n"/>
+      <c r="L31" s="139" t="n"/>
+      <c r="M31" s="140" t="n"/>
+      <c r="N31" s="141" t="n"/>
+      <c r="O31" s="142" t="n"/>
+      <c r="P31" s="143" t="n"/>
+      <c r="Q31" s="141" t="n"/>
+      <c r="R31" s="142" t="n"/>
+      <c r="S31" s="143" t="n"/>
+      <c r="T31" s="141" t="n"/>
+      <c r="U31" s="142" t="n"/>
+      <c r="V31" s="143" t="n"/>
+      <c r="W31" s="144" t="n"/>
+      <c r="X31" s="144" t="n"/>
+      <c r="Y31" s="144" t="n"/>
+      <c r="Z31" s="144" t="n"/>
+      <c r="AA31" s="144" t="n"/>
+      <c r="AB31" s="144" t="n"/>
     </row>
     <row r="32" ht="18" customFormat="1" customHeight="1" s="1">
-      <c r="A32" s="9" t="n"/>
-      <c r="B32" s="108" t="n"/>
-      <c r="C32" s="109" t="n"/>
-      <c r="D32" s="109" t="n"/>
-      <c r="E32" s="110" t="n"/>
-      <c r="F32" s="111" t="n"/>
-      <c r="G32" s="112" t="n"/>
-      <c r="H32" s="112" t="n"/>
-      <c r="I32" s="113" t="n"/>
-      <c r="J32" s="114" t="n"/>
-      <c r="K32" s="115" t="n"/>
-      <c r="L32" s="115" t="n"/>
-      <c r="M32" s="116" t="n"/>
-      <c r="N32" s="89" t="n"/>
-      <c r="O32" s="90" t="n"/>
-      <c r="P32" s="91" t="n"/>
-      <c r="Q32" s="89" t="n"/>
-      <c r="R32" s="90" t="n"/>
-      <c r="S32" s="91" t="n"/>
-      <c r="T32" s="89" t="n"/>
-      <c r="U32" s="90" t="n"/>
-      <c r="V32" s="91" t="n"/>
+      <c r="A32" s="137" t="n"/>
+      <c r="B32" s="138" t="n"/>
+      <c r="C32" s="139" t="n"/>
+      <c r="D32" s="139" t="n"/>
+      <c r="E32" s="140" t="n"/>
+      <c r="F32" s="138" t="n"/>
+      <c r="G32" s="139" t="n"/>
+      <c r="H32" s="139" t="n"/>
+      <c r="I32" s="140" t="n"/>
+      <c r="J32" s="138" t="n"/>
+      <c r="K32" s="139" t="n"/>
+      <c r="L32" s="139" t="n"/>
+      <c r="M32" s="140" t="n"/>
+      <c r="N32" s="141" t="n"/>
+      <c r="O32" s="142" t="n"/>
+      <c r="P32" s="143" t="n"/>
+      <c r="Q32" s="141" t="n"/>
+      <c r="R32" s="142" t="n"/>
+      <c r="S32" s="143" t="n"/>
+      <c r="T32" s="141" t="n"/>
+      <c r="U32" s="142" t="n"/>
+      <c r="V32" s="143" t="n"/>
+      <c r="W32" s="144" t="n"/>
+      <c r="X32" s="144" t="n"/>
+      <c r="Y32" s="144" t="n"/>
+      <c r="Z32" s="144" t="n"/>
+      <c r="AA32" s="144" t="n"/>
+      <c r="AB32" s="144" t="n"/>
     </row>
     <row r="33" ht="18" customFormat="1" customHeight="1" s="1">
-      <c r="A33" s="8" t="n"/>
-      <c r="B33" s="108" t="n"/>
-      <c r="C33" s="109" t="n"/>
-      <c r="D33" s="109" t="n"/>
-      <c r="E33" s="110" t="n"/>
-      <c r="F33" s="111" t="n"/>
-      <c r="G33" s="112" t="n"/>
-      <c r="H33" s="112" t="n"/>
-      <c r="I33" s="113" t="n"/>
-      <c r="J33" s="114" t="n"/>
-      <c r="K33" s="115" t="n"/>
-      <c r="L33" s="115" t="n"/>
-      <c r="M33" s="116" t="n"/>
-      <c r="N33" s="89" t="n"/>
-      <c r="O33" s="90" t="n"/>
-      <c r="P33" s="91" t="n"/>
-      <c r="Q33" s="89" t="n"/>
-      <c r="R33" s="90" t="n"/>
-      <c r="S33" s="91" t="n"/>
-      <c r="T33" s="89" t="n"/>
-      <c r="U33" s="90" t="n"/>
-      <c r="V33" s="91" t="n"/>
+      <c r="A33" s="137" t="n"/>
+      <c r="B33" s="138" t="n"/>
+      <c r="C33" s="139" t="n"/>
+      <c r="D33" s="139" t="n"/>
+      <c r="E33" s="140" t="n"/>
+      <c r="F33" s="138" t="n"/>
+      <c r="G33" s="139" t="n"/>
+      <c r="H33" s="139" t="n"/>
+      <c r="I33" s="140" t="n"/>
+      <c r="J33" s="138" t="n"/>
+      <c r="K33" s="139" t="n"/>
+      <c r="L33" s="139" t="n"/>
+      <c r="M33" s="140" t="n"/>
+      <c r="N33" s="141" t="n"/>
+      <c r="O33" s="142" t="n"/>
+      <c r="P33" s="143" t="n"/>
+      <c r="Q33" s="141" t="n"/>
+      <c r="R33" s="142" t="n"/>
+      <c r="S33" s="143" t="n"/>
+      <c r="T33" s="141" t="n"/>
+      <c r="U33" s="142" t="n"/>
+      <c r="V33" s="143" t="n"/>
+      <c r="W33" s="144" t="n"/>
+      <c r="X33" s="144" t="n"/>
+      <c r="Y33" s="144" t="n"/>
+      <c r="Z33" s="144" t="n"/>
+      <c r="AA33" s="144" t="n"/>
+      <c r="AB33" s="144" t="n"/>
     </row>
     <row r="34" ht="18" customFormat="1" customHeight="1" s="1">
-      <c r="A34" s="9" t="n"/>
-      <c r="B34" s="108" t="n"/>
-      <c r="C34" s="109" t="n"/>
-      <c r="D34" s="109" t="n"/>
-      <c r="E34" s="110" t="n"/>
-      <c r="F34" s="111" t="n"/>
-      <c r="G34" s="112" t="n"/>
-      <c r="H34" s="112" t="n"/>
-      <c r="I34" s="113" t="n"/>
-      <c r="J34" s="114" t="n"/>
-      <c r="K34" s="115" t="n"/>
-      <c r="L34" s="115" t="n"/>
-      <c r="M34" s="116" t="n"/>
-      <c r="N34" s="89" t="n"/>
-      <c r="O34" s="90" t="n"/>
-      <c r="P34" s="91" t="n"/>
-      <c r="Q34" s="89" t="n"/>
-      <c r="R34" s="90" t="n"/>
-      <c r="S34" s="91" t="n"/>
-      <c r="T34" s="89" t="n"/>
-      <c r="U34" s="90" t="n"/>
-      <c r="V34" s="91" t="n"/>
+      <c r="A34" s="137" t="n"/>
+      <c r="B34" s="138" t="n"/>
+      <c r="C34" s="139" t="n"/>
+      <c r="D34" s="139" t="n"/>
+      <c r="E34" s="140" t="n"/>
+      <c r="F34" s="138" t="n"/>
+      <c r="G34" s="139" t="n"/>
+      <c r="H34" s="139" t="n"/>
+      <c r="I34" s="140" t="n"/>
+      <c r="J34" s="138" t="n"/>
+      <c r="K34" s="139" t="n"/>
+      <c r="L34" s="139" t="n"/>
+      <c r="M34" s="140" t="n"/>
+      <c r="N34" s="141" t="n"/>
+      <c r="O34" s="142" t="n"/>
+      <c r="P34" s="143" t="n"/>
+      <c r="Q34" s="141" t="n"/>
+      <c r="R34" s="142" t="n"/>
+      <c r="S34" s="143" t="n"/>
+      <c r="T34" s="141" t="n"/>
+      <c r="U34" s="142" t="n"/>
+      <c r="V34" s="143" t="n"/>
+      <c r="W34" s="144" t="n"/>
+      <c r="X34" s="144" t="n"/>
+      <c r="Y34" s="144" t="n"/>
+      <c r="Z34" s="144" t="n"/>
+      <c r="AA34" s="144" t="n"/>
+      <c r="AB34" s="144" t="n"/>
     </row>
     <row r="35" ht="18" customFormat="1" customHeight="1" s="1">
-      <c r="A35" s="10" t="inlineStr">
-        <is>
-          <t>LEGEND  |  RSI = Jump Height (m) ÷ Ground Contact Time (s)  |  GCT = Ground Contact Time in seconds  |  Enter summary values directly — individual hop data not required</t>
+      <c r="A35" s="145" t="inlineStr">
+        <is>
+          <t>LEGEND  |  RSI = Jump Height (m) ÷ Ground Contact Time (s)  |  GCT = Ground Contact Time in seconds  |  Enter raw hop values in A1/A2/A3 cells — the engine computes Avg RSI, Best RSI, and Avg GCT automatically</t>
         </is>
       </c>
       <c r="B35" s="53" t="n"/>
@@ -6615,19 +6998,34 @@
       <c r="J35" s="53" t="n"/>
       <c r="K35" s="53" t="n"/>
       <c r="L35" s="53" t="n"/>
-      <c r="M35" s="54" t="n"/>
+      <c r="M35" s="53" t="n"/>
+      <c r="N35" s="53" t="n"/>
+      <c r="O35" s="53" t="n"/>
+      <c r="P35" s="53" t="n"/>
+      <c r="Q35" s="53" t="n"/>
+      <c r="R35" s="53" t="n"/>
+      <c r="S35" s="53" t="n"/>
+      <c r="T35" s="53" t="n"/>
+      <c r="U35" s="53" t="n"/>
+      <c r="V35" s="53" t="n"/>
+      <c r="W35" s="53" t="n"/>
+      <c r="X35" s="53" t="n"/>
+      <c r="Y35" s="53" t="n"/>
+      <c r="Z35" s="53" t="n"/>
+      <c r="AA35" s="53" t="n"/>
+      <c r="AB35" s="54" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="9">
-    <mergeCell ref="A1:M1"/>
-    <mergeCell ref="F3:I3"/>
-    <mergeCell ref="J3:M3"/>
-    <mergeCell ref="A35:M35"/>
+    <mergeCell ref="B3:G3"/>
+    <mergeCell ref="A2:AB2"/>
+    <mergeCell ref="A35:AB35"/>
+    <mergeCell ref="W3:Y3"/>
+    <mergeCell ref="A1:AB1"/>
     <mergeCell ref="T3:V3"/>
-    <mergeCell ref="B3:E3"/>
-    <mergeCell ref="A2:M2"/>
-    <mergeCell ref="N3:P3"/>
-    <mergeCell ref="Q3:S3"/>
+    <mergeCell ref="Z3:AB3"/>
+    <mergeCell ref="N3:S3"/>
+    <mergeCell ref="H3:M3"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>